<commit_message>
docs: mark #28 done in the Fase 2 Gantt chart
The four #28 rows (database design, modelling and script, login and
user CRUD) move to Francisco, Cumplido, 2026-10-18 to 2026-10-19, with
a note pointing to PR #35. Edited in the sheet XML, so bars, formulas
and conditional formatting stay untouched; the workbook recalculates on
open (summary: 30 done, 1 late). Checked opening it in Excel.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Anexos/Gestion/Carta Gantt Fase 2.xlsx
+++ b/Anexos/Gestion/Carta Gantt Fase 2.xlsx
@@ -19,7 +19,7 @@
     <definedName name="_xlnm.Print_Area" localSheetId="0">'Carta Gantt'!$B$1:$AC$62</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="0">'Carta Gantt'!$8:$9</definedName>
   </definedNames>
-  <calcPr calcId="191029"/>
+  <calcPr calcId="191029" fullCalcOnLoad="1"/>
   <extLst>
     <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
       <xcalcf:calcFeatures>
@@ -40,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="211" uniqueCount="124">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="215" uniqueCount="125">
   <si>
     <t>Carta Gantt · ShelfVision AI</t>
   </si>
@@ -412,6 +412,9 @@
   </si>
   <si>
     <t>Fechas por definir</t>
+  </si>
+  <si>
+    <t>Hecho en el PR #35 (app web Django + SQLite, 2026-10-18 a 2026-10-19).</t>
   </si>
 </sst>
 </file>
@@ -1721,16 +1724,16 @@
         <v>41</v>
       </c>
       <c r="D24" s="19" t="s">
-        <v>23</v>
+        <v>27</v>
       </c>
       <c r="E24" s="20">
-        <v>46315</v>
+        <v>46313</v>
       </c>
       <c r="F24" s="20">
-        <v>46319</v>
+        <v>46314</v>
       </c>
       <c r="G24" s="19" t="s">
-        <v>7</v>
+        <v>4</v>
       </c>
       <c r="H24" s="21" t="s">
         <v>42</v>
@@ -1755,7 +1758,7 @@
       <c r="Z24" s="22"/>
       <c r="AA24" s="22"/>
       <c r="AC24" s="23" t="s">
-        <v>43</v>
+        <v>124</v>
       </c>
     </row>
     <row r="25" spans="2:29" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.2">
@@ -1764,16 +1767,16 @@
         <v>44</v>
       </c>
       <c r="D25" s="19" t="s">
-        <v>23</v>
+        <v>27</v>
       </c>
       <c r="E25" s="20">
-        <v>46315</v>
+        <v>46313</v>
       </c>
       <c r="F25" s="20">
-        <v>46319</v>
+        <v>46314</v>
       </c>
       <c r="G25" s="19" t="s">
-        <v>7</v>
+        <v>4</v>
       </c>
       <c r="H25" s="21" t="s">
         <v>42</v>
@@ -1798,7 +1801,7 @@
       <c r="Z25" s="22"/>
       <c r="AA25" s="22"/>
       <c r="AC25" s="23" t="s">
-        <v>43</v>
+        <v>124</v>
       </c>
     </row>
     <row r="26" spans="2:29" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.2">
@@ -1846,16 +1849,16 @@
         <v>46</v>
       </c>
       <c r="D27" s="19" t="s">
-        <v>23</v>
+        <v>27</v>
       </c>
       <c r="E27" s="20">
-        <v>46315</v>
+        <v>46313</v>
       </c>
       <c r="F27" s="20">
-        <v>46319</v>
+        <v>46314</v>
       </c>
       <c r="G27" s="19" t="s">
-        <v>7</v>
+        <v>4</v>
       </c>
       <c r="H27" s="21" t="s">
         <v>42</v>
@@ -1880,7 +1883,7 @@
       <c r="Z27" s="22"/>
       <c r="AA27" s="22"/>
       <c r="AC27" s="23" t="s">
-        <v>43</v>
+        <v>124</v>
       </c>
     </row>
     <row r="28" spans="2:29" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.2">
@@ -2526,16 +2529,16 @@
         <v>81</v>
       </c>
       <c r="D44" s="19" t="s">
-        <v>23</v>
+        <v>27</v>
       </c>
       <c r="E44" s="20">
-        <v>46315</v>
+        <v>46313</v>
       </c>
       <c r="F44" s="20">
-        <v>46322</v>
+        <v>46314</v>
       </c>
       <c r="G44" s="19" t="s">
-        <v>7</v>
+        <v>4</v>
       </c>
       <c r="H44" s="21" t="s">
         <v>42</v>
@@ -2560,7 +2563,7 @@
       <c r="Z44" s="22"/>
       <c r="AA44" s="22"/>
       <c r="AC44" s="23" t="s">
-        <v>82</v>
+        <v>124</v>
       </c>
     </row>
     <row r="45" spans="2:29" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.2">

</xml_diff>

<commit_message>
docs: interim report draft and results analysis on Kaggle photos (#27, #34)
- #34: run the full pipeline on the 45 Kaggle CC0 photos with their
  annotation; 10 best and 10 worst cases with input/system/expected
  figures, causes and fixes, and a comparison by product type
  (docs/analisis-resultados.md). Detector out of domain: mAP50 0.713,
  recall 0.644; packaged products: alert right in 92% of photos.
- #27: interim report draft in Word (Fase 2/), following the 2.2/2.3
  format, with the #34 results in section 3.
- Backlog: #34 done, #33 step 1 recorded, new #46 (glass-door
  refrigerators), stale dependencies fixed; Gantt updated.
- Test plan: DET-03/DET-04 results, new DET-06, RF01 and run log.
- CLAUDE.md: how to check that the ponytail skill is loaded (drive
  letter case in installed_plugins.json on Windows).

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Anexos/Gestion/Carta Gantt Fase 2.xlsx
+++ b/Anexos/Gestion/Carta Gantt Fase 2.xlsx
@@ -5,10 +5,10 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\panxh\AppData\Local\Temp\claude\d--workspace-capstone\37fde7ac-c8b6-4fc8-b0ff-38b8fae6c95c\scratchpad\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\workspace\capstone\Anexos\Gestion\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A44BAA39-2738-41B0-9A52-E56671370787}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{913D1302-B30E-472F-A254-127B05B1E56E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -19,7 +19,7 @@
     <definedName name="_xlnm.Print_Area" localSheetId="0">'Carta Gantt'!$B$1:$AC$62</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="0">'Carta Gantt'!$8:$9</definedName>
   </definedNames>
-  <calcPr calcId="191029" fullCalcOnLoad="1"/>
+  <calcPr calcId="191029"/>
   <extLst>
     <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
       <xcalcf:calcFeatures>
@@ -40,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="215" uniqueCount="125">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="211" uniqueCount="123">
   <si>
     <t>Carta Gantt · ShelfVision AI</t>
   </si>
@@ -171,9 +171,6 @@
     <t>#28</t>
   </si>
   <si>
-    <t>Sin hacer en la Iteración 1; ahora en #28. Fecha propuesta</t>
-  </si>
-  <si>
     <t>Modelamiento de base de datos</t>
   </si>
   <si>
@@ -286,9 +283,6 @@
   </si>
   <si>
     <t>Login, CRUD de usuarios y roles y base de datos (CU00, CU06)</t>
-  </si>
-  <si>
-    <t>Esperado desde la semana 8. Fecha propuesta</t>
   </si>
   <si>
     <t>Primer demo operativo ante Walmart</t>
@@ -423,7 +417,7 @@
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <numFmts count="2">
     <numFmt numFmtId="164" formatCode="dd"/>
-    <numFmt numFmtId="166" formatCode="dd/mm"/>
+    <numFmt numFmtId="165" formatCode="dd/mm"/>
   </numFmts>
   <fonts count="12" x14ac:knownFonts="1">
     <font>
@@ -676,7 +670,7 @@
     <xf numFmtId="0" fontId="5" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" indent="1"/>
     </xf>
-    <xf numFmtId="166" fontId="2" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="165" fontId="2" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
@@ -1033,7 +1027,7 @@
     <row r="5" spans="2:29" ht="26.1" customHeight="1" x14ac:dyDescent="0.2">
       <c r="D5" s="5">
         <f>COUNTIF($G$10:$G$62,"Cumplido")</f>
-        <v>26</v>
+        <v>31</v>
       </c>
       <c r="E5" s="6">
         <f>COUNTIF($G$10:$G$62,"En curso")</f>
@@ -1041,11 +1035,11 @@
       </c>
       <c r="F5" s="7">
         <f>COUNTIF($G$10:$G$62,"Pendiente")</f>
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="G5" s="8">
         <f>COUNTIF($G$10:$G$62,"Atrasado")</f>
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="H5" s="9">
         <f>COUNTIF($G$10:$G$62,"Bloqueado")</f>
@@ -1758,13 +1752,13 @@
       <c r="Z24" s="22"/>
       <c r="AA24" s="22"/>
       <c r="AC24" s="23" t="s">
-        <v>124</v>
+        <v>122</v>
       </c>
     </row>
     <row r="25" spans="2:29" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B25" s="18"/>
       <c r="C25" s="19" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="D25" s="19" t="s">
         <v>27</v>
@@ -1801,13 +1795,13 @@
       <c r="Z25" s="22"/>
       <c r="AA25" s="22"/>
       <c r="AC25" s="23" t="s">
-        <v>124</v>
+        <v>122</v>
       </c>
     </row>
     <row r="26" spans="2:29" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B26" s="18"/>
       <c r="C26" s="19" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="D26" s="19" t="s">
         <v>31</v>
@@ -1846,7 +1840,7 @@
     <row r="27" spans="2:29" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B27" s="18"/>
       <c r="C27" s="19" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="D27" s="19" t="s">
         <v>27</v>
@@ -1883,13 +1877,13 @@
       <c r="Z27" s="22"/>
       <c r="AA27" s="22"/>
       <c r="AC27" s="23" t="s">
-        <v>124</v>
+        <v>122</v>
       </c>
     </row>
     <row r="28" spans="2:29" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B28" s="16"/>
       <c r="C28" s="17" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="D28" s="16"/>
       <c r="E28" s="16"/>
@@ -1921,7 +1915,7 @@
     <row r="29" spans="2:29" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B29" s="18"/>
       <c r="C29" s="19" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="D29" s="19" t="s">
         <v>27</v>
@@ -1936,7 +1930,7 @@
         <v>4</v>
       </c>
       <c r="H29" s="21" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="I29" s="22"/>
       <c r="J29" s="22"/>
@@ -1962,7 +1956,7 @@
     <row r="30" spans="2:29" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B30" s="18"/>
       <c r="C30" s="19" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="D30" s="19" t="s">
         <v>31</v>
@@ -1977,7 +1971,7 @@
         <v>4</v>
       </c>
       <c r="H30" s="21" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="I30" s="22"/>
       <c r="J30" s="22"/>
@@ -2003,10 +1997,10 @@
     <row r="31" spans="2:29" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B31" s="18"/>
       <c r="C31" s="19" t="s">
+        <v>51</v>
+      </c>
+      <c r="D31" s="19" t="s">
         <v>52</v>
-      </c>
-      <c r="D31" s="19" t="s">
-        <v>53</v>
       </c>
       <c r="E31" s="20">
         <v>46292</v>
@@ -2018,7 +2012,7 @@
         <v>4</v>
       </c>
       <c r="H31" s="21" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="I31" s="22"/>
       <c r="J31" s="22"/>
@@ -2044,7 +2038,7 @@
     <row r="32" spans="2:29" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B32" s="18"/>
       <c r="C32" s="19" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="D32" s="19" t="s">
         <v>27</v>
@@ -2059,7 +2053,7 @@
         <v>4</v>
       </c>
       <c r="H32" s="21" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="I32" s="22"/>
       <c r="J32" s="22"/>
@@ -2085,7 +2079,7 @@
     <row r="33" spans="2:29" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B33" s="16"/>
       <c r="C33" s="17" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="D33" s="16"/>
       <c r="E33" s="16"/>
@@ -2117,7 +2111,7 @@
     <row r="34" spans="2:29" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B34" s="18"/>
       <c r="C34" s="19" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="D34" s="19" t="s">
         <v>27</v>
@@ -2132,7 +2126,7 @@
         <v>4</v>
       </c>
       <c r="H34" s="21" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="I34" s="22"/>
       <c r="J34" s="22"/>
@@ -2158,7 +2152,7 @@
     <row r="35" spans="2:29" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B35" s="18"/>
       <c r="C35" s="19" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="D35" s="19" t="s">
         <v>27</v>
@@ -2173,7 +2167,7 @@
         <v>4</v>
       </c>
       <c r="H35" s="21" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="I35" s="22"/>
       <c r="J35" s="22"/>
@@ -2195,13 +2189,13 @@
       <c r="Z35" s="22"/>
       <c r="AA35" s="22"/>
       <c r="AC35" s="23" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
     </row>
     <row r="36" spans="2:29" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B36" s="18"/>
       <c r="C36" s="19" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="D36" s="19" t="s">
         <v>27</v>
@@ -2216,7 +2210,7 @@
         <v>4</v>
       </c>
       <c r="H36" s="21" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="I36" s="22"/>
       <c r="J36" s="22"/>
@@ -2238,13 +2232,13 @@
       <c r="Z36" s="22"/>
       <c r="AA36" s="22"/>
       <c r="AC36" s="23" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
     </row>
     <row r="37" spans="2:29" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B37" s="18"/>
       <c r="C37" s="19" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="D37" s="19" t="s">
         <v>27</v>
@@ -2259,7 +2253,7 @@
         <v>4</v>
       </c>
       <c r="H37" s="21" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="I37" s="22"/>
       <c r="J37" s="22"/>
@@ -2285,7 +2279,7 @@
     <row r="38" spans="2:29" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B38" s="18"/>
       <c r="C38" s="19" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="D38" s="19" t="s">
         <v>27</v>
@@ -2300,7 +2294,7 @@
         <v>4</v>
       </c>
       <c r="H38" s="21" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="I38" s="22"/>
       <c r="J38" s="22"/>
@@ -2326,7 +2320,7 @@
     <row r="39" spans="2:29" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B39" s="18"/>
       <c r="C39" s="19" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="D39" s="19" t="s">
         <v>27</v>
@@ -2341,7 +2335,7 @@
         <v>4</v>
       </c>
       <c r="H39" s="21" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="I39" s="22"/>
       <c r="J39" s="22"/>
@@ -2367,7 +2361,7 @@
     <row r="40" spans="2:29" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B40" s="18"/>
       <c r="C40" s="19" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="D40" s="19" t="s">
         <v>27</v>
@@ -2382,7 +2376,7 @@
         <v>4</v>
       </c>
       <c r="H40" s="21" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="I40" s="22"/>
       <c r="J40" s="22"/>
@@ -2408,7 +2402,7 @@
     <row r="41" spans="2:29" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B41" s="18"/>
       <c r="C41" s="19" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="D41" s="19" t="s">
         <v>27</v>
@@ -2420,10 +2414,10 @@
         <v>46316</v>
       </c>
       <c r="G41" s="19" t="s">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="H41" s="21" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="I41" s="22"/>
       <c r="J41" s="22"/>
@@ -2445,13 +2439,13 @@
       <c r="Z41" s="22"/>
       <c r="AA41" s="22"/>
       <c r="AC41" s="23" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
     </row>
     <row r="42" spans="2:29" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B42" s="18"/>
       <c r="C42" s="19" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="D42" s="19" t="s">
         <v>31</v>
@@ -2466,7 +2460,7 @@
         <v>6</v>
       </c>
       <c r="H42" s="21" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="I42" s="22"/>
       <c r="J42" s="22"/>
@@ -2488,13 +2482,13 @@
       <c r="Z42" s="22"/>
       <c r="AA42" s="22"/>
       <c r="AC42" s="23" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
     </row>
     <row r="43" spans="2:29" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B43" s="16"/>
       <c r="C43" s="17" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="D43" s="16"/>
       <c r="E43" s="16"/>
@@ -2526,7 +2520,7 @@
     <row r="44" spans="2:29" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B44" s="18"/>
       <c r="C44" s="19" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="D44" s="19" t="s">
         <v>27</v>
@@ -2563,13 +2557,13 @@
       <c r="Z44" s="22"/>
       <c r="AA44" s="22"/>
       <c r="AC44" s="23" t="s">
-        <v>124</v>
+        <v>122</v>
       </c>
     </row>
     <row r="45" spans="2:29" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B45" s="18"/>
       <c r="C45" s="19" t="s">
-        <v>83</v>
+        <v>81</v>
       </c>
       <c r="D45" s="19" t="s">
         <v>23</v>
@@ -2584,7 +2578,7 @@
         <v>6</v>
       </c>
       <c r="H45" s="21" t="s">
-        <v>84</v>
+        <v>82</v>
       </c>
       <c r="I45" s="22"/>
       <c r="J45" s="22"/>
@@ -2606,16 +2600,16 @@
       <c r="Z45" s="22"/>
       <c r="AA45" s="22"/>
       <c r="AC45" s="23" t="s">
-        <v>85</v>
+        <v>83</v>
       </c>
     </row>
     <row r="46" spans="2:29" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B46" s="18"/>
       <c r="C46" s="19" t="s">
-        <v>86</v>
+        <v>84</v>
       </c>
       <c r="D46" s="19" t="s">
-        <v>87</v>
+        <v>85</v>
       </c>
       <c r="E46" s="20"/>
       <c r="F46" s="20"/>
@@ -2623,7 +2617,7 @@
         <v>8</v>
       </c>
       <c r="H46" s="21" t="s">
-        <v>88</v>
+        <v>86</v>
       </c>
       <c r="I46" s="22"/>
       <c r="J46" s="22"/>
@@ -2645,13 +2639,13 @@
       <c r="Z46" s="22"/>
       <c r="AA46" s="22"/>
       <c r="AC46" s="23" t="s">
-        <v>89</v>
+        <v>87</v>
       </c>
     </row>
     <row r="47" spans="2:29" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B47" s="16"/>
       <c r="C47" s="17" t="s">
-        <v>90</v>
+        <v>88</v>
       </c>
       <c r="D47" s="16"/>
       <c r="E47" s="16"/>
@@ -2683,7 +2677,7 @@
     <row r="48" spans="2:29" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B48" s="18"/>
       <c r="C48" s="19" t="s">
-        <v>91</v>
+        <v>89</v>
       </c>
       <c r="D48" s="19" t="s">
         <v>27</v>
@@ -2698,7 +2692,7 @@
         <v>4</v>
       </c>
       <c r="H48" s="21" t="s">
-        <v>92</v>
+        <v>90</v>
       </c>
       <c r="I48" s="22"/>
       <c r="J48" s="22"/>
@@ -2724,7 +2718,7 @@
     <row r="49" spans="2:29" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B49" s="18"/>
       <c r="C49" s="19" t="s">
-        <v>93</v>
+        <v>91</v>
       </c>
       <c r="D49" s="19" t="s">
         <v>27</v>
@@ -2739,7 +2733,7 @@
         <v>4</v>
       </c>
       <c r="H49" s="21" t="s">
-        <v>94</v>
+        <v>92</v>
       </c>
       <c r="I49" s="22"/>
       <c r="J49" s="22"/>
@@ -2765,7 +2759,7 @@
     <row r="50" spans="2:29" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B50" s="18"/>
       <c r="C50" s="19" t="s">
-        <v>95</v>
+        <v>93</v>
       </c>
       <c r="D50" s="19" t="s">
         <v>31</v>
@@ -2780,7 +2774,7 @@
         <v>7</v>
       </c>
       <c r="H50" s="21" t="s">
-        <v>96</v>
+        <v>94</v>
       </c>
       <c r="I50" s="22"/>
       <c r="J50" s="22"/>
@@ -2802,13 +2796,13 @@
       <c r="Z50" s="22"/>
       <c r="AA50" s="22"/>
       <c r="AC50" s="23" t="s">
-        <v>97</v>
+        <v>95</v>
       </c>
     </row>
     <row r="51" spans="2:29" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B51" s="18"/>
       <c r="C51" s="19" t="s">
-        <v>98</v>
+        <v>96</v>
       </c>
       <c r="D51" s="19" t="s">
         <v>27</v>
@@ -2823,7 +2817,7 @@
         <v>5</v>
       </c>
       <c r="H51" s="21" t="s">
-        <v>99</v>
+        <v>97</v>
       </c>
       <c r="I51" s="22"/>
       <c r="J51" s="22"/>
@@ -2845,13 +2839,13 @@
       <c r="Z51" s="22"/>
       <c r="AA51" s="22"/>
       <c r="AC51" s="23" t="s">
-        <v>100</v>
+        <v>98</v>
       </c>
     </row>
     <row r="52" spans="2:29" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B52" s="18"/>
       <c r="C52" s="19" t="s">
-        <v>101</v>
+        <v>99</v>
       </c>
       <c r="D52" s="19" t="s">
         <v>27</v>
@@ -2860,13 +2854,13 @@
         <v>46315</v>
       </c>
       <c r="F52" s="20">
-        <v>46316</v>
+        <v>46315</v>
       </c>
       <c r="G52" s="19" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="H52" s="21" t="s">
-        <v>102</v>
+        <v>100</v>
       </c>
       <c r="I52" s="22"/>
       <c r="J52" s="22"/>
@@ -2892,7 +2886,7 @@
     <row r="53" spans="2:29" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B53" s="18"/>
       <c r="C53" s="19" t="s">
-        <v>103</v>
+        <v>101</v>
       </c>
       <c r="D53" s="19" t="s">
         <v>27</v>
@@ -2907,7 +2901,7 @@
         <v>5</v>
       </c>
       <c r="H53" s="21" t="s">
-        <v>104</v>
+        <v>102</v>
       </c>
       <c r="I53" s="22"/>
       <c r="J53" s="22"/>
@@ -2933,7 +2927,7 @@
     <row r="54" spans="2:29" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B54" s="18"/>
       <c r="C54" s="19" t="s">
-        <v>105</v>
+        <v>103</v>
       </c>
       <c r="D54" s="19" t="s">
         <v>27</v>
@@ -2948,7 +2942,7 @@
         <v>6</v>
       </c>
       <c r="H54" s="21" t="s">
-        <v>106</v>
+        <v>104</v>
       </c>
       <c r="I54" s="22"/>
       <c r="J54" s="22"/>
@@ -2974,7 +2968,7 @@
     <row r="55" spans="2:29" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B55" s="18"/>
       <c r="C55" s="19" t="s">
-        <v>107</v>
+        <v>105</v>
       </c>
       <c r="D55" s="19" t="s">
         <v>31</v>
@@ -2989,7 +2983,7 @@
         <v>6</v>
       </c>
       <c r="H55" s="21" t="s">
-        <v>108</v>
+        <v>106</v>
       </c>
       <c r="I55" s="22"/>
       <c r="J55" s="22"/>
@@ -3011,13 +3005,13 @@
       <c r="Z55" s="22"/>
       <c r="AA55" s="22"/>
       <c r="AC55" s="23" t="s">
-        <v>109</v>
+        <v>107</v>
       </c>
     </row>
     <row r="56" spans="2:29" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B56" s="16"/>
       <c r="C56" s="17" t="s">
-        <v>110</v>
+        <v>108</v>
       </c>
       <c r="D56" s="16"/>
       <c r="E56" s="16"/>
@@ -3049,10 +3043,10 @@
     <row r="57" spans="2:29" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B57" s="18"/>
       <c r="C57" s="19" t="s">
-        <v>111</v>
+        <v>109</v>
       </c>
       <c r="D57" s="19" t="s">
-        <v>112</v>
+        <v>110</v>
       </c>
       <c r="E57" s="20">
         <v>46316</v>
@@ -3084,13 +3078,13 @@
       <c r="Z57" s="22"/>
       <c r="AA57" s="22"/>
       <c r="AC57" s="23" t="s">
-        <v>113</v>
+        <v>111</v>
       </c>
     </row>
     <row r="58" spans="2:29" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B58" s="18"/>
       <c r="C58" s="19" t="s">
-        <v>114</v>
+        <v>112</v>
       </c>
       <c r="D58" s="19" t="s">
         <v>23</v>
@@ -3105,7 +3099,7 @@
         <v>6</v>
       </c>
       <c r="H58" s="21" t="s">
-        <v>115</v>
+        <v>113</v>
       </c>
       <c r="I58" s="22"/>
       <c r="J58" s="22"/>
@@ -3127,16 +3121,16 @@
       <c r="Z58" s="22"/>
       <c r="AA58" s="22"/>
       <c r="AC58" s="23" t="s">
-        <v>116</v>
+        <v>114</v>
       </c>
     </row>
     <row r="59" spans="2:29" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B59" s="18"/>
       <c r="C59" s="19" t="s">
-        <v>117</v>
+        <v>115</v>
       </c>
       <c r="D59" s="19" t="s">
-        <v>112</v>
+        <v>110</v>
       </c>
       <c r="E59" s="20">
         <v>46323</v>
@@ -3168,16 +3162,16 @@
       <c r="Z59" s="22"/>
       <c r="AA59" s="22"/>
       <c r="AC59" s="23" t="s">
-        <v>118</v>
+        <v>116</v>
       </c>
     </row>
     <row r="60" spans="2:29" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B60" s="18"/>
       <c r="C60" s="19" t="s">
-        <v>119</v>
+        <v>117</v>
       </c>
       <c r="D60" s="19" t="s">
-        <v>112</v>
+        <v>110</v>
       </c>
       <c r="E60" s="20">
         <v>46349</v>
@@ -3209,13 +3203,13 @@
       <c r="Z60" s="22"/>
       <c r="AA60" s="22"/>
       <c r="AC60" s="23" t="s">
-        <v>120</v>
+        <v>118</v>
       </c>
     </row>
     <row r="61" spans="2:29" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B61" s="16"/>
       <c r="C61" s="17" t="s">
-        <v>121</v>
+        <v>119</v>
       </c>
       <c r="D61" s="16"/>
       <c r="E61" s="16"/>
@@ -3247,10 +3241,10 @@
     <row r="62" spans="2:29" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B62" s="18"/>
       <c r="C62" s="19" t="s">
-        <v>122</v>
+        <v>120</v>
       </c>
       <c r="D62" s="19" t="s">
-        <v>112</v>
+        <v>110</v>
       </c>
       <c r="E62" s="20">
         <v>46356</v>
@@ -3282,7 +3276,7 @@
       <c r="Z62" s="22"/>
       <c r="AA62" s="22"/>
       <c r="AC62" s="23" t="s">
-        <v>123</v>
+        <v>121</v>
       </c>
     </row>
     <row r="63" spans="2:29" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>

</xml_diff>

<commit_message>
docs: add Fase 1 improvement plan (#26)
Fase 1 was graded 7.0 with no written observations, so the plan compares
what the Fase 1 guide and annexes committed to against the current
project and the Fase 2 progress rubric. It defines ten improvements with
actions, owners, dates, evidence and status, plus measurable specific
objectives and evidence/competency tables for guide 2.4.

The Fase 2 Gantt chart marks the item done on 2026-10-20, late against
the 2026-10-09 deadline.
</commit_message>
<xml_diff>
--- a/Anexos/Gestion/Carta Gantt Fase 2.xlsx
+++ b/Anexos/Gestion/Carta Gantt Fase 2.xlsx
@@ -333,7 +333,7 @@
     <t>#26</t>
   </si>
   <si>
-    <t>Plazo 2026-10-09</t>
+    <t>Hecho el 2026-10-20, con atraso (plazo 2026-10-09). docs/plan-de-mejoras.md</t>
   </si>
   <si>
     <t>Informe intermedio: estado de avance y conclusiones</t>
@@ -2771,13 +2771,13 @@
         <v>31</v>
       </c>
       <c r="E50" s="20">
-        <v>46300</v>
+        <v>46315</v>
       </c>
       <c r="F50" s="20">
-        <v>46304</v>
+        <v>46315</v>
       </c>
       <c r="G50" s="19" t="s">
-        <v>7</v>
+        <v>4</v>
       </c>
       <c r="H50" s="21" t="s">
         <v>96</v>

</xml_diff>

<commit_message>
docs: reassign demo video (#36) to Nicko
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Anexos/Gestion/Carta Gantt Fase 2.xlsx
+++ b/Anexos/Gestion/Carta Gantt Fase 2.xlsx
@@ -655,7 +655,7 @@
     <outlinePr summaryBelow="0" summaryRight="0"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="B1:AC62"/>
+  <dimension ref="A1:AC62"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="12.5703125" defaultRowHeight="15" customHeight="1"/>
   <cols>
     <col width="2" customWidth="1" style="1" min="1" max="1"/>
@@ -2954,7 +2954,7 @@
       </c>
       <c r="D54" s="19" t="inlineStr">
         <is>
-          <t>Francisco</t>
+          <t>Nicko</t>
         </is>
       </c>
       <c r="E54" s="20" t="n">

</xml_diff>

<commit_message>
docs: fill progress guide 2.4 and draft reflection diary 2.1 (#37)
The official 2.4 template (uploaded in PR #42) now holds the progress
summary, adjusted objectives and methodology, evidence and quality
safeguards, the work plan monitoring table built from the Fase 2 Gantt
chart, and the adjustments analysis. The template's floating tables
were made inline so the long plan table flows across pages with its
header repeated.

docs/evidencias-avance.md keeps the same content as Markdown plus the
group answers for diary 2.1, whose template is still missing. Parts
that are the team's opinion are marked for them to complete.

Claims item #37 and marks it in progress in PROGRESS.md and the Gantt.
</commit_message>
<xml_diff>
--- a/Anexos/Gestion/Carta Gantt Fase 2.xlsx
+++ b/Anexos/Gestion/Carta Gantt Fase 2.xlsx
@@ -3006,15 +3006,15 @@
           <t>Mariana</t>
         </is>
       </c>
-      <c r="E55" s="20" t="n">
-        <v>46317</v>
+      <c r="E55" s="20">
+        <v>46315</v>
       </c>
       <c r="F55" s="20" t="n">
         <v>46321</v>
       </c>
       <c r="G55" s="19" t="inlineStr">
         <is>
-          <t>Pendiente</t>
+          <t>En curso</t>
         </is>
       </c>
       <c r="H55" s="21" t="inlineStr">
@@ -3043,7 +3043,7 @@
       <c r="AA55" s="22" t="n"/>
       <c r="AC55" s="23" t="inlineStr">
         <is>
-          <t>Plazo 2026-10-26. Fecha propuesta</t>
+          <t>Plazo 2026-10-26. Guía 2.4 llenada el 2026-10-20 (Fase 2/); falta el diario 2.1 y las partes de opinión del equipo</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
docs: mark use case redesign done (#42)
</commit_message>
<xml_diff>
--- a/Anexos/Gestion/Carta Gantt Fase 2.xlsx
+++ b/Anexos/Gestion/Carta Gantt Fase 2.xlsx
@@ -10,7 +10,7 @@
   </sheets>
   <definedNames>
     <definedName name="_xlnm.Print_Titles" localSheetId="0">'Carta Gantt'!$8:$9</definedName>
-    <definedName name="_xlnm.Print_Area" localSheetId="0">'Carta Gantt'!$B$1:$AC$62</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="0">'Carta Gantt'!$B$1:$AC$63</definedName>
   </definedNames>
   <calcPr calcId="191029" fullCalcOnLoad="1"/>
 </workbook>
@@ -655,7 +655,7 @@
     <outlinePr summaryBelow="0" summaryRight="0"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:AC62"/>
+  <dimension ref="A1:AC63"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="12.5703125" defaultRowHeight="15" customHeight="1"/>
   <cols>
     <col width="2" customWidth="1" style="1" min="1" max="1"/>
@@ -695,23 +695,23 @@
     <row r="4" ht="15.75" customHeight="1" s="1"/>
     <row r="5" ht="26.1" customHeight="1" s="1">
       <c r="D5" s="5">
-        <f>COUNTIF($G$10:$G$62,"Cumplido")</f>
+        <f>COUNTIF($G$10:$G$63,"Cumplido")</f>
         <v/>
       </c>
       <c r="E5" s="6">
-        <f>COUNTIF($G$10:$G$62,"En curso")</f>
+        <f>COUNTIF($G$10:$G$63,"En curso")</f>
         <v/>
       </c>
       <c r="F5" s="7">
-        <f>COUNTIF($G$10:$G$62,"Pendiente")</f>
+        <f>COUNTIF($G$10:$G$63,"Pendiente")</f>
         <v/>
       </c>
       <c r="G5" s="8">
-        <f>COUNTIF($G$10:$G$62,"Atrasado")</f>
+        <f>COUNTIF($G$10:$G$63,"Atrasado")</f>
         <v/>
       </c>
       <c r="H5" s="9">
-        <f>COUNTIF($G$10:$G$62,"Bloqueado")</f>
+        <f>COUNTIF($G$10:$G$63,"Bloqueado")</f>
         <v/>
       </c>
     </row>
@@ -3048,116 +3048,116 @@
       </c>
     </row>
     <row r="56" ht="20.1" customHeight="1" s="1">
-      <c r="B56" s="16" t="n"/>
-      <c r="C56" s="17" t="inlineStr">
+      <c r="B56" s="18" t="n"/>
+      <c r="C56" s="19" t="inlineStr">
+        <is>
+          <t>Rehacer plantillas de C.U y diagramas según la app Django</t>
+        </is>
+      </c>
+      <c r="D56" s="19" t="inlineStr">
+        <is>
+          <t>Mariana</t>
+        </is>
+      </c>
+      <c r="E56" s="20">
+        <v>46316</v>
+      </c>
+      <c r="F56" s="20">
+        <v>46316</v>
+      </c>
+      <c r="G56" s="19" t="inlineStr">
+        <is>
+          <t>Cumplido</t>
+        </is>
+      </c>
+      <c r="H56" s="21" t="inlineStr">
+        <is>
+          <t>#42</t>
+        </is>
+      </c>
+      <c r="I56" s="22" t="n"/>
+      <c r="J56" s="22" t="n"/>
+      <c r="K56" s="22" t="n"/>
+      <c r="L56" s="22" t="n"/>
+      <c r="M56" s="22" t="n"/>
+      <c r="N56" s="22" t="n"/>
+      <c r="O56" s="22" t="n"/>
+      <c r="P56" s="22" t="n"/>
+      <c r="Q56" s="22" t="n"/>
+      <c r="R56" s="22" t="n"/>
+      <c r="S56" s="22" t="n"/>
+      <c r="T56" s="22" t="n"/>
+      <c r="U56" s="22" t="n"/>
+      <c r="V56" s="22" t="n"/>
+      <c r="W56" s="22" t="n"/>
+      <c r="X56" s="22" t="n"/>
+      <c r="Y56" s="22" t="n"/>
+      <c r="Z56" s="22" t="n"/>
+      <c r="AA56" s="22" t="n"/>
+      <c r="AC56" s="23" t="inlineStr">
+        <is>
+          <t>Hecho el 2026-10-21: plantillas, fuentes Mermaid y PNG (CU00-CU06 y arquitectura). docs/cambios-cu.md</t>
+        </is>
+      </c>
+    </row>
+    <row r="57" ht="20.1" customHeight="1" s="1">
+      <c r="B57" s="16" t="n"/>
+      <c r="C57" s="17" t="inlineStr">
         <is>
           <t>HITOS DEL CURSO</t>
         </is>
       </c>
-      <c r="D56" s="16" t="n"/>
-      <c r="E56" s="16" t="n"/>
-      <c r="F56" s="16" t="n"/>
-      <c r="G56" s="16" t="n"/>
-      <c r="H56" s="16" t="n"/>
-      <c r="I56" s="16" t="n"/>
-      <c r="J56" s="16" t="n"/>
-      <c r="K56" s="16" t="n"/>
-      <c r="L56" s="16" t="n"/>
-      <c r="M56" s="16" t="n"/>
-      <c r="N56" s="16" t="n"/>
-      <c r="O56" s="16" t="n"/>
-      <c r="P56" s="16" t="n"/>
-      <c r="Q56" s="16" t="n"/>
-      <c r="R56" s="16" t="n"/>
-      <c r="S56" s="16" t="n"/>
-      <c r="T56" s="16" t="n"/>
-      <c r="U56" s="16" t="n"/>
-      <c r="V56" s="16" t="n"/>
-      <c r="W56" s="16" t="n"/>
-      <c r="X56" s="16" t="n"/>
-      <c r="Y56" s="16" t="n"/>
-      <c r="Z56" s="16" t="n"/>
-      <c r="AA56" s="16" t="n"/>
-      <c r="AB56" s="16" t="n"/>
-      <c r="AC56" s="16" t="n"/>
-    </row>
-    <row r="57" ht="20.1" customHeight="1" s="1">
-      <c r="B57" s="18" t="n"/>
-      <c r="C57" s="19" t="inlineStr">
-        <is>
-          <t>Informe intermedio y video</t>
-        </is>
-      </c>
-      <c r="D57" s="19" t="inlineStr">
-        <is>
-          <t>Equipo</t>
-        </is>
-      </c>
-      <c r="E57" s="20" t="n">
-        <v>46316</v>
-      </c>
-      <c r="F57" s="20" t="n">
-        <v>46316</v>
-      </c>
-      <c r="G57" s="19" t="inlineStr">
-        <is>
-          <t>En curso</t>
-        </is>
-      </c>
-      <c r="H57" s="21" t="n"/>
-      <c r="I57" s="22" t="n"/>
-      <c r="J57" s="22" t="n"/>
-      <c r="K57" s="22" t="n"/>
-      <c r="L57" s="22" t="n"/>
-      <c r="M57" s="22" t="n"/>
-      <c r="N57" s="22" t="n"/>
-      <c r="O57" s="22" t="n"/>
-      <c r="P57" s="22" t="n"/>
-      <c r="Q57" s="22" t="n"/>
-      <c r="R57" s="22" t="n"/>
-      <c r="S57" s="22" t="n"/>
-      <c r="T57" s="22" t="n"/>
-      <c r="U57" s="22" t="n"/>
-      <c r="V57" s="22" t="n"/>
-      <c r="W57" s="22" t="n"/>
-      <c r="X57" s="22" t="n"/>
-      <c r="Y57" s="22" t="n"/>
-      <c r="Z57" s="22" t="n"/>
-      <c r="AA57" s="22" t="n"/>
-      <c r="AC57" s="23" t="inlineStr">
-        <is>
-          <t>Entrega 2026-10-21</t>
-        </is>
-      </c>
+      <c r="D57" s="16" t="n"/>
+      <c r="E57" s="16" t="n"/>
+      <c r="F57" s="16" t="n"/>
+      <c r="G57" s="16" t="n"/>
+      <c r="H57" s="16" t="n"/>
+      <c r="I57" s="16" t="n"/>
+      <c r="J57" s="16" t="n"/>
+      <c r="K57" s="16" t="n"/>
+      <c r="L57" s="16" t="n"/>
+      <c r="M57" s="16" t="n"/>
+      <c r="N57" s="16" t="n"/>
+      <c r="O57" s="16" t="n"/>
+      <c r="P57" s="16" t="n"/>
+      <c r="Q57" s="16" t="n"/>
+      <c r="R57" s="16" t="n"/>
+      <c r="S57" s="16" t="n"/>
+      <c r="T57" s="16" t="n"/>
+      <c r="U57" s="16" t="n"/>
+      <c r="V57" s="16" t="n"/>
+      <c r="W57" s="16" t="n"/>
+      <c r="X57" s="16" t="n"/>
+      <c r="Y57" s="16" t="n"/>
+      <c r="Z57" s="16" t="n"/>
+      <c r="AA57" s="16" t="n"/>
+      <c r="AB57" s="16" t="n"/>
+      <c r="AC57" s="16" t="n"/>
     </row>
     <row r="58" ht="20.1" customHeight="1" s="1">
       <c r="B58" s="18" t="n"/>
       <c r="C58" s="19" t="inlineStr">
         <is>
-          <t>Feria de informática</t>
+          <t>Informe intermedio y video</t>
         </is>
       </c>
       <c r="D58" s="19" t="inlineStr">
         <is>
-          <t>Nicko</t>
+          <t>Equipo</t>
         </is>
       </c>
       <c r="E58" s="20" t="n">
-        <v>46321</v>
+        <v>46316</v>
       </c>
       <c r="F58" s="20" t="n">
-        <v>46325</v>
+        <v>46316</v>
       </c>
       <c r="G58" s="19" t="inlineStr">
         <is>
-          <t>Pendiente</t>
-        </is>
-      </c>
-      <c r="H58" s="21" t="inlineStr">
-        <is>
-          <t>#38</t>
-        </is>
-      </c>
+          <t>En curso</t>
+        </is>
+      </c>
+      <c r="H58" s="21" t="n"/>
       <c r="I58" s="22" t="n"/>
       <c r="J58" s="22" t="n"/>
       <c r="K58" s="22" t="n"/>
@@ -3179,7 +3179,7 @@
       <c r="AA58" s="22" t="n"/>
       <c r="AC58" s="23" t="inlineStr">
         <is>
-          <t>Día y hora por informar</t>
+          <t>Entrega 2026-10-21</t>
         </is>
       </c>
     </row>
@@ -3187,16 +3187,16 @@
       <c r="B59" s="18" t="n"/>
       <c r="C59" s="19" t="inlineStr">
         <is>
-          <t>Evaluación 2 (Avance): 50% de los C.U y demo del Sprint 1</t>
+          <t>Feria de informática</t>
         </is>
       </c>
       <c r="D59" s="19" t="inlineStr">
         <is>
-          <t>Equipo</t>
+          <t>Nicko</t>
         </is>
       </c>
       <c r="E59" s="20" t="n">
-        <v>46323</v>
+        <v>46321</v>
       </c>
       <c r="F59" s="20" t="n">
         <v>46325</v>
@@ -3206,7 +3206,11 @@
           <t>Pendiente</t>
         </is>
       </c>
-      <c r="H59" s="21" t="n"/>
+      <c r="H59" s="21" t="inlineStr">
+        <is>
+          <t>#38</t>
+        </is>
+      </c>
       <c r="I59" s="22" t="n"/>
       <c r="J59" s="22" t="n"/>
       <c r="K59" s="22" t="n"/>
@@ -3228,7 +3232,7 @@
       <c r="AA59" s="22" t="n"/>
       <c r="AC59" s="23" t="inlineStr">
         <is>
-          <t>Día exacto por confirmar</t>
+          <t>Día y hora por informar</t>
         </is>
       </c>
     </row>
@@ -3236,7 +3240,7 @@
       <c r="B60" s="18" t="n"/>
       <c r="C60" s="19" t="inlineStr">
         <is>
-          <t>Entrega final de la Fase 2</t>
+          <t>Evaluación 2 (Avance): 50% de los C.U y demo del Sprint 1</t>
         </is>
       </c>
       <c r="D60" s="19" t="inlineStr">
@@ -3245,10 +3249,10 @@
         </is>
       </c>
       <c r="E60" s="20" t="n">
-        <v>46349</v>
+        <v>46323</v>
       </c>
       <c r="F60" s="20" t="n">
-        <v>46353</v>
+        <v>46325</v>
       </c>
       <c r="G60" s="19" t="inlineStr">
         <is>
@@ -3277,94 +3281,142 @@
       <c r="AA60" s="22" t="n"/>
       <c r="AC60" s="23" t="inlineStr">
         <is>
+          <t>Día exacto por confirmar</t>
+        </is>
+      </c>
+    </row>
+    <row r="61" ht="20.1" customHeight="1" s="1">
+      <c r="B61" s="18" t="n"/>
+      <c r="C61" s="19" t="inlineStr">
+        <is>
+          <t>Entrega final de la Fase 2</t>
+        </is>
+      </c>
+      <c r="D61" s="19" t="inlineStr">
+        <is>
+          <t>Equipo</t>
+        </is>
+      </c>
+      <c r="E61" s="20" t="n">
+        <v>46349</v>
+      </c>
+      <c r="F61" s="20" t="n">
+        <v>46353</v>
+      </c>
+      <c r="G61" s="19" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="H61" s="21" t="n"/>
+      <c r="I61" s="22" t="n"/>
+      <c r="J61" s="22" t="n"/>
+      <c r="K61" s="22" t="n"/>
+      <c r="L61" s="22" t="n"/>
+      <c r="M61" s="22" t="n"/>
+      <c r="N61" s="22" t="n"/>
+      <c r="O61" s="22" t="n"/>
+      <c r="P61" s="22" t="n"/>
+      <c r="Q61" s="22" t="n"/>
+      <c r="R61" s="22" t="n"/>
+      <c r="S61" s="22" t="n"/>
+      <c r="T61" s="22" t="n"/>
+      <c r="U61" s="22" t="n"/>
+      <c r="V61" s="22" t="n"/>
+      <c r="W61" s="22" t="n"/>
+      <c r="X61" s="22" t="n"/>
+      <c r="Y61" s="22" t="n"/>
+      <c r="Z61" s="22" t="n"/>
+      <c r="AA61" s="22" t="n"/>
+      <c r="AC61" s="23" t="inlineStr">
+        <is>
           <t>Semana 15, por confirmar</t>
         </is>
       </c>
     </row>
-    <row r="61" ht="20.1" customHeight="1" s="1">
-      <c r="B61" s="16" t="n"/>
-      <c r="C61" s="17" t="inlineStr">
+    <row r="62" ht="20.1" customHeight="1" s="1">
+      <c r="B62" s="16" t="n"/>
+      <c r="C62" s="17" t="inlineStr">
         <is>
           <t>FASE 3</t>
         </is>
       </c>
-      <c r="D61" s="16" t="n"/>
-      <c r="E61" s="16" t="n"/>
-      <c r="F61" s="16" t="n"/>
-      <c r="G61" s="16" t="n"/>
-      <c r="H61" s="16" t="n"/>
-      <c r="I61" s="16" t="n"/>
-      <c r="J61" s="16" t="n"/>
-      <c r="K61" s="16" t="n"/>
-      <c r="L61" s="16" t="n"/>
-      <c r="M61" s="16" t="n"/>
-      <c r="N61" s="16" t="n"/>
-      <c r="O61" s="16" t="n"/>
-      <c r="P61" s="16" t="n"/>
-      <c r="Q61" s="16" t="n"/>
-      <c r="R61" s="16" t="n"/>
-      <c r="S61" s="16" t="n"/>
-      <c r="T61" s="16" t="n"/>
-      <c r="U61" s="16" t="n"/>
-      <c r="V61" s="16" t="n"/>
-      <c r="W61" s="16" t="n"/>
-      <c r="X61" s="16" t="n"/>
-      <c r="Y61" s="16" t="n"/>
-      <c r="Z61" s="16" t="n"/>
-      <c r="AA61" s="16" t="n"/>
-      <c r="AB61" s="16" t="n"/>
-      <c r="AC61" s="16" t="n"/>
-    </row>
-    <row r="62" ht="20.1" customHeight="1" s="1">
-      <c r="B62" s="18" t="n"/>
-      <c r="C62" s="19" t="inlineStr">
+      <c r="D62" s="16" t="n"/>
+      <c r="E62" s="16" t="n"/>
+      <c r="F62" s="16" t="n"/>
+      <c r="G62" s="16" t="n"/>
+      <c r="H62" s="16" t="n"/>
+      <c r="I62" s="16" t="n"/>
+      <c r="J62" s="16" t="n"/>
+      <c r="K62" s="16" t="n"/>
+      <c r="L62" s="16" t="n"/>
+      <c r="M62" s="16" t="n"/>
+      <c r="N62" s="16" t="n"/>
+      <c r="O62" s="16" t="n"/>
+      <c r="P62" s="16" t="n"/>
+      <c r="Q62" s="16" t="n"/>
+      <c r="R62" s="16" t="n"/>
+      <c r="S62" s="16" t="n"/>
+      <c r="T62" s="16" t="n"/>
+      <c r="U62" s="16" t="n"/>
+      <c r="V62" s="16" t="n"/>
+      <c r="W62" s="16" t="n"/>
+      <c r="X62" s="16" t="n"/>
+      <c r="Y62" s="16" t="n"/>
+      <c r="Z62" s="16" t="n"/>
+      <c r="AA62" s="16" t="n"/>
+      <c r="AB62" s="16" t="n"/>
+      <c r="AC62" s="16" t="n"/>
+    </row>
+    <row r="63" ht="20.1" customHeight="1" s="1">
+      <c r="B63" s="18" t="n"/>
+      <c r="C63" s="19" t="inlineStr">
         <is>
           <t>Ajustes finales, manuales y exposición ante la Comisión</t>
         </is>
       </c>
-      <c r="D62" s="19" t="inlineStr">
+      <c r="D63" s="19" t="inlineStr">
         <is>
           <t>Equipo</t>
         </is>
       </c>
-      <c r="E62" s="20" t="n">
+      <c r="E63" s="20" t="n">
         <v>46356</v>
       </c>
-      <c r="F62" s="20" t="n">
+      <c r="F63" s="20" t="n">
         <v>46374</v>
       </c>
-      <c r="G62" s="19" t="inlineStr">
+      <c r="G63" s="19" t="inlineStr">
         <is>
           <t>Pendiente</t>
         </is>
       </c>
-      <c r="H62" s="21" t="n"/>
-      <c r="I62" s="22" t="n"/>
-      <c r="J62" s="22" t="n"/>
-      <c r="K62" s="22" t="n"/>
-      <c r="L62" s="22" t="n"/>
-      <c r="M62" s="22" t="n"/>
-      <c r="N62" s="22" t="n"/>
-      <c r="O62" s="22" t="n"/>
-      <c r="P62" s="22" t="n"/>
-      <c r="Q62" s="22" t="n"/>
-      <c r="R62" s="22" t="n"/>
-      <c r="S62" s="22" t="n"/>
-      <c r="T62" s="22" t="n"/>
-      <c r="U62" s="22" t="n"/>
-      <c r="V62" s="22" t="n"/>
-      <c r="W62" s="22" t="n"/>
-      <c r="X62" s="22" t="n"/>
-      <c r="Y62" s="22" t="n"/>
-      <c r="Z62" s="22" t="n"/>
-      <c r="AA62" s="22" t="n"/>
-      <c r="AC62" s="23" t="inlineStr">
+      <c r="H63" s="21" t="n"/>
+      <c r="I63" s="22" t="n"/>
+      <c r="J63" s="22" t="n"/>
+      <c r="K63" s="22" t="n"/>
+      <c r="L63" s="22" t="n"/>
+      <c r="M63" s="22" t="n"/>
+      <c r="N63" s="22" t="n"/>
+      <c r="O63" s="22" t="n"/>
+      <c r="P63" s="22" t="n"/>
+      <c r="Q63" s="22" t="n"/>
+      <c r="R63" s="22" t="n"/>
+      <c r="S63" s="22" t="n"/>
+      <c r="T63" s="22" t="n"/>
+      <c r="U63" s="22" t="n"/>
+      <c r="V63" s="22" t="n"/>
+      <c r="W63" s="22" t="n"/>
+      <c r="X63" s="22" t="n"/>
+      <c r="Y63" s="22" t="n"/>
+      <c r="Z63" s="22" t="n"/>
+      <c r="AA63" s="22" t="n"/>
+      <c r="AC63" s="23" t="inlineStr">
         <is>
           <t>Fechas por definir</t>
         </is>
       </c>
     </row>
-    <row r="63" ht="15.75" customHeight="1" s="1"/>
     <row r="64" ht="15.75" customHeight="1" s="1"/>
     <row r="65" ht="15.75" customHeight="1" s="1"/>
     <row r="66" ht="15.75" customHeight="1" s="1"/>
@@ -4302,6 +4354,7 @@
     <row r="998" ht="15.75" customHeight="1" s="1"/>
     <row r="999" ht="15.75" customHeight="1" s="1"/>
     <row r="1000" ht="15.75" customHeight="1" s="1"/>
+    <row r="1001" ht="15.75" customHeight="1" s="1"/>
   </sheetData>
   <mergeCells count="5">
     <mergeCell ref="U8:Y8"/>
@@ -4310,7 +4363,7 @@
     <mergeCell ref="Q8:T8"/>
     <mergeCell ref="I8:L8"/>
   </mergeCells>
-  <conditionalFormatting sqref="B10:B62">
+  <conditionalFormatting sqref="B10:B63">
     <cfRule type="expression" priority="2" dxfId="5" stopIfTrue="1">
       <formula>$G10="Cumplido"</formula>
     </cfRule>
@@ -4327,7 +4380,7 @@
       <formula>$G10="Bloqueado"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="I10:AA62">
+  <conditionalFormatting sqref="I10:AA63">
     <cfRule type="expression" priority="1" dxfId="5" stopIfTrue="1">
       <formula>AND($E10&lt;&gt;"",I$9&lt;=$F10,I$9+6&gt;=$E10,$G10="Cumplido")</formula>
     </cfRule>
@@ -4344,7 +4397,7 @@
       <formula>AND($E10&lt;&gt;"",I$9&lt;=$F10,I$9+6&gt;=$E10,$G10="Bloqueado")</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="S10:S62">
+  <conditionalFormatting sqref="S10:S63">
     <cfRule type="expression" priority="11" dxfId="0">
       <formula>$G10&lt;&gt;""</formula>
     </cfRule>

</xml_diff>

<commit_message>
docs: document report formats and mark #7 done
</commit_message>
<xml_diff>
--- a/Anexos/Gestion/Carta Gantt Fase 2.xlsx
+++ b/Anexos/Gestion/Carta Gantt Fase 2.xlsx
@@ -2379,15 +2379,15 @@
           <t>Mariana</t>
         </is>
       </c>
-      <c r="E42" s="20" t="n">
-        <v>46315</v>
-      </c>
-      <c r="F42" s="20" t="n">
-        <v>46322</v>
+      <c r="E42" s="20">
+        <v>46316</v>
+      </c>
+      <c r="F42" s="20">
+        <v>46316</v>
       </c>
       <c r="G42" s="19" t="inlineStr">
         <is>
-          <t>Pendiente</t>
+          <t>Cumplido</t>
         </is>
       </c>
       <c r="H42" s="21" t="inlineStr">
@@ -2416,7 +2416,7 @@
       <c r="AA42" s="22" t="n"/>
       <c r="AC42" s="23" t="inlineStr">
         <is>
-          <t>Fecha propuesta, a confirmar</t>
+          <t>Hecho el 2026-10-21: src/reporting/export.py y página Reportes de la app web (CU04)</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
docs: close item #33 and add audit findings #49-#54 to the backlog
</commit_message>
<xml_diff>
--- a/Anexos/Gestion/Carta Gantt Fase 2.xlsx
+++ b/Anexos/Gestion/Carta Gantt Fase 2.xlsx
@@ -655,7 +655,7 @@
     <outlinePr summaryBelow="0" summaryRight="0"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:AC62"/>
+  <dimension ref="B1:AC62"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="12.5703125" defaultRowHeight="15" customHeight="1"/>
   <cols>
     <col width="2" customWidth="1" style="1" min="1" max="1"/>
@@ -2334,7 +2334,7 @@
       </c>
       <c r="G41" s="19" t="inlineStr">
         <is>
-          <t>En curso</t>
+          <t>Cumplido</t>
         </is>
       </c>
       <c r="H41" s="21" t="inlineStr">
@@ -2753,10 +2753,10 @@
           <t>Mariana</t>
         </is>
       </c>
-      <c r="E50" s="20">
+      <c r="E50" s="20" t="n">
         <v>46315</v>
       </c>
-      <c r="F50" s="20">
+      <c r="F50" s="20" t="n">
         <v>46315</v>
       </c>
       <c r="G50" s="19" t="inlineStr">
@@ -3006,7 +3006,7 @@
           <t>Mariana</t>
         </is>
       </c>
-      <c r="E55" s="20">
+      <c r="E55" s="20" t="n">
         <v>46315</v>
       </c>
       <c r="F55" s="20" t="n">

</xml_diff>

<commit_message>
docs: deja listo el informe intermedio de avance con los datos al 2026-10-21 (#27)
Actualiza estado por módulo y por C.U (reportes #7, plantillas #42), riesgos y próximos pasos con los hallazgos #49 a #55, el fine-tuning (#33) en métricas y comparativo, el anexo de PR hasta el #57 y los commits por integrante. La Carta Gantt suma 3 filas y el corte pasa al 2026-10-21.
</commit_message>
<xml_diff>
--- a/Anexos/Gestion/Carta Gantt Fase 2.xlsx
+++ b/Anexos/Gestion/Carta Gantt Fase 2.xlsx
@@ -10,7 +10,7 @@
   </sheets>
   <definedNames>
     <definedName name="_xlnm.Print_Titles" localSheetId="0">'Carta Gantt'!$8:$9</definedName>
-    <definedName name="_xlnm.Print_Area" localSheetId="0">'Carta Gantt'!$B$1:$AC$63</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="0">'Carta Gantt'!$B$1:$AC$66</definedName>
   </definedNames>
   <calcPr calcId="191029" fullCalcOnLoad="1"/>
 </workbook>
@@ -655,7 +655,7 @@
     <outlinePr summaryBelow="0" summaryRight="0"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:AC63"/>
+  <dimension ref="A1:AC66"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="12.5703125" defaultRowHeight="15" customHeight="1"/>
   <cols>
     <col width="2" customWidth="1" style="1" min="1" max="1"/>
@@ -688,30 +688,30 @@
     <row r="3" ht="15.75" customHeight="1" s="1">
       <c r="C3" s="4" t="inlineStr">
         <is>
-          <t>Corte: 19-10-2026 (informe intermedio), franja roja en la línea de tiempo. Copia extendida de la Carta Gantt de la Iteración 1.</t>
+          <t>Corte: 21-10-2026 (informe intermedio)</t>
         </is>
       </c>
     </row>
     <row r="4" ht="15.75" customHeight="1" s="1"/>
     <row r="5" ht="26.1" customHeight="1" s="1">
       <c r="D5" s="5">
-        <f>COUNTIF($G$10:$G$63,"Cumplido")</f>
+        <f>COUNTIF($G$10:$G$66,"Cumplido")</f>
         <v/>
       </c>
       <c r="E5" s="6">
-        <f>COUNTIF($G$10:$G$63,"En curso")</f>
+        <f>COUNTIF($G$10:$G$66,"En curso")</f>
         <v/>
       </c>
       <c r="F5" s="7">
-        <f>COUNTIF($G$10:$G$63,"Pendiente")</f>
+        <f>COUNTIF($G$10:$G$66,"Pendiente")</f>
         <v/>
       </c>
       <c r="G5" s="8">
-        <f>COUNTIF($G$10:$G$63,"Atrasado")</f>
+        <f>COUNTIF($G$10:$G$66,"Atrasado")</f>
         <v/>
       </c>
       <c r="H5" s="9">
-        <f>COUNTIF($G$10:$G$63,"Bloqueado")</f>
+        <f>COUNTIF($G$10:$G$66,"Bloqueado")</f>
         <v/>
       </c>
     </row>
@@ -2421,118 +2421,114 @@
       </c>
     </row>
     <row r="43" ht="20.1" customHeight="1" s="1">
-      <c r="B43" s="16" t="n"/>
-      <c r="C43" s="17" t="inlineStr">
+      <c r="B43" s="18" t="n"/>
+      <c r="C43" s="19" t="inlineStr">
+        <is>
+          <t>Detector con ruido de cámara de sala (#55)</t>
+        </is>
+      </c>
+      <c r="D43" s="19" t="inlineStr">
+        <is>
+          <t>Francisco</t>
+        </is>
+      </c>
+      <c r="E43" s="20" t="n">
+        <v>46324</v>
+      </c>
+      <c r="F43" s="20" t="n">
+        <v>46332</v>
+      </c>
+      <c r="G43" s="19" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="H43" s="21" t="inlineStr">
+        <is>
+          <t>#55</t>
+        </is>
+      </c>
+      <c r="I43" s="22" t="n"/>
+      <c r="J43" s="22" t="n"/>
+      <c r="K43" s="22" t="n"/>
+      <c r="L43" s="22" t="n"/>
+      <c r="M43" s="22" t="n"/>
+      <c r="N43" s="22" t="n"/>
+      <c r="O43" s="22" t="n"/>
+      <c r="P43" s="22" t="n"/>
+      <c r="Q43" s="22" t="n"/>
+      <c r="R43" s="22" t="n"/>
+      <c r="S43" s="22" t="n"/>
+      <c r="T43" s="22" t="n"/>
+      <c r="U43" s="22" t="n"/>
+      <c r="V43" s="22" t="n"/>
+      <c r="W43" s="22" t="n"/>
+      <c r="X43" s="22" t="n"/>
+      <c r="Y43" s="22" t="n"/>
+      <c r="Z43" s="22" t="n"/>
+      <c r="AA43" s="22" t="n"/>
+      <c r="AC43" s="23" t="n"/>
+    </row>
+    <row r="44" ht="20.1" customHeight="1" s="1">
+      <c r="B44" s="16" t="n"/>
+      <c r="C44" s="17" t="inlineStr">
         <is>
           <t>FASE 2 · APLICACIÓN WEB</t>
         </is>
       </c>
-      <c r="D43" s="16" t="n"/>
-      <c r="E43" s="16" t="n"/>
-      <c r="F43" s="16" t="n"/>
-      <c r="G43" s="16" t="n"/>
-      <c r="H43" s="16" t="n"/>
-      <c r="I43" s="16" t="n"/>
-      <c r="J43" s="16" t="n"/>
-      <c r="K43" s="16" t="n"/>
-      <c r="L43" s="16" t="n"/>
-      <c r="M43" s="16" t="n"/>
-      <c r="N43" s="16" t="n"/>
-      <c r="O43" s="16" t="n"/>
-      <c r="P43" s="16" t="n"/>
-      <c r="Q43" s="16" t="n"/>
-      <c r="R43" s="16" t="n"/>
-      <c r="S43" s="16" t="n"/>
-      <c r="T43" s="16" t="n"/>
-      <c r="U43" s="16" t="n"/>
-      <c r="V43" s="16" t="n"/>
-      <c r="W43" s="16" t="n"/>
-      <c r="X43" s="16" t="n"/>
-      <c r="Y43" s="16" t="n"/>
-      <c r="Z43" s="16" t="n"/>
-      <c r="AA43" s="16" t="n"/>
-      <c r="AB43" s="16" t="n"/>
-      <c r="AC43" s="16" t="n"/>
-    </row>
-    <row r="44" ht="20.1" customHeight="1" s="1">
-      <c r="B44" s="18" t="n"/>
-      <c r="C44" s="19" t="inlineStr">
-        <is>
-          <t>Login, CRUD de usuarios y roles y base de datos (CU00, CU06)</t>
-        </is>
-      </c>
-      <c r="D44" s="19" t="inlineStr">
-        <is>
-          <t>Francisco</t>
-        </is>
-      </c>
-      <c r="E44" s="20" t="n">
-        <v>46313</v>
-      </c>
-      <c r="F44" s="20" t="n">
-        <v>46314</v>
-      </c>
-      <c r="G44" s="19" t="inlineStr">
-        <is>
-          <t>Cumplido</t>
-        </is>
-      </c>
-      <c r="H44" s="21" t="inlineStr">
-        <is>
-          <t>#28</t>
-        </is>
-      </c>
-      <c r="I44" s="22" t="n"/>
-      <c r="J44" s="22" t="n"/>
-      <c r="K44" s="22" t="n"/>
-      <c r="L44" s="22" t="n"/>
-      <c r="M44" s="22" t="n"/>
-      <c r="N44" s="22" t="n"/>
-      <c r="O44" s="22" t="n"/>
-      <c r="P44" s="22" t="n"/>
-      <c r="Q44" s="22" t="n"/>
-      <c r="R44" s="22" t="n"/>
-      <c r="S44" s="22" t="n"/>
-      <c r="T44" s="22" t="n"/>
-      <c r="U44" s="22" t="n"/>
-      <c r="V44" s="22" t="n"/>
-      <c r="W44" s="22" t="n"/>
-      <c r="X44" s="22" t="n"/>
-      <c r="Y44" s="22" t="n"/>
-      <c r="Z44" s="22" t="n"/>
-      <c r="AA44" s="22" t="n"/>
-      <c r="AC44" s="23" t="inlineStr">
-        <is>
-          <t>Hecho en el PR #35 (app web Django + SQLite, 2026-10-18 a 2026-10-19).</t>
-        </is>
-      </c>
+      <c r="D44" s="16" t="n"/>
+      <c r="E44" s="16" t="n"/>
+      <c r="F44" s="16" t="n"/>
+      <c r="G44" s="16" t="n"/>
+      <c r="H44" s="16" t="n"/>
+      <c r="I44" s="16" t="n"/>
+      <c r="J44" s="16" t="n"/>
+      <c r="K44" s="16" t="n"/>
+      <c r="L44" s="16" t="n"/>
+      <c r="M44" s="16" t="n"/>
+      <c r="N44" s="16" t="n"/>
+      <c r="O44" s="16" t="n"/>
+      <c r="P44" s="16" t="n"/>
+      <c r="Q44" s="16" t="n"/>
+      <c r="R44" s="16" t="n"/>
+      <c r="S44" s="16" t="n"/>
+      <c r="T44" s="16" t="n"/>
+      <c r="U44" s="16" t="n"/>
+      <c r="V44" s="16" t="n"/>
+      <c r="W44" s="16" t="n"/>
+      <c r="X44" s="16" t="n"/>
+      <c r="Y44" s="16" t="n"/>
+      <c r="Z44" s="16" t="n"/>
+      <c r="AA44" s="16" t="n"/>
+      <c r="AB44" s="16" t="n"/>
+      <c r="AC44" s="16" t="n"/>
     </row>
     <row r="45" ht="20.1" customHeight="1" s="1">
       <c r="B45" s="18" t="n"/>
       <c r="C45" s="19" t="inlineStr">
         <is>
-          <t>Primer demo operativo ante Walmart</t>
+          <t>Login, CRUD de usuarios y roles y base de datos (CU00, CU06)</t>
         </is>
       </c>
       <c r="D45" s="19" t="inlineStr">
         <is>
-          <t>Nicko</t>
+          <t>Francisco</t>
         </is>
       </c>
       <c r="E45" s="20" t="n">
-        <v>46322</v>
+        <v>46313</v>
       </c>
       <c r="F45" s="20" t="n">
-        <v>46326</v>
+        <v>46314</v>
       </c>
       <c r="G45" s="19" t="inlineStr">
         <is>
-          <t>Pendiente</t>
+          <t>Cumplido</t>
         </is>
       </c>
       <c r="H45" s="21" t="inlineStr">
         <is>
-          <t>#29</t>
+          <t>#28</t>
         </is>
       </c>
       <c r="I45" s="22" t="n"/>
@@ -2556,7 +2552,7 @@
       <c r="AA45" s="22" t="n"/>
       <c r="AC45" s="23" t="inlineStr">
         <is>
-          <t>Depende de #28</t>
+          <t>Hecho en el PR #35 (app web Django + SQLite, 2026-10-18 a 2026-10-19).</t>
         </is>
       </c>
     </row>
@@ -2564,24 +2560,28 @@
       <c r="B46" s="18" t="n"/>
       <c r="C46" s="19" t="inlineStr">
         <is>
-          <t>Instalación en el servidor del CITT</t>
+          <t>Correcciones de la auditoría de la app web (#49-#53)</t>
         </is>
       </c>
       <c r="D46" s="19" t="inlineStr">
         <is>
-          <t>Por definir</t>
-        </is>
-      </c>
-      <c r="E46" s="20" t="n"/>
-      <c r="F46" s="20" t="n"/>
+          <t>Francisco, Mariana</t>
+        </is>
+      </c>
+      <c r="E46" s="20" t="n">
+        <v>46317</v>
+      </c>
+      <c r="F46" s="20" t="n">
+        <v>46323</v>
+      </c>
       <c r="G46" s="19" t="inlineStr">
         <is>
-          <t>Bloqueado</t>
+          <t>Pendiente</t>
         </is>
       </c>
       <c r="H46" s="21" t="inlineStr">
         <is>
-          <t>#39</t>
+          <t>#49-#53</t>
         </is>
       </c>
       <c r="I46" s="22" t="n"/>
@@ -2603,72 +2603,83 @@
       <c r="Y46" s="22" t="n"/>
       <c r="Z46" s="22" t="n"/>
       <c r="AA46" s="22" t="n"/>
-      <c r="AC46" s="23" t="inlineStr">
-        <is>
-          <t>Faltan las instrucciones del CITT</t>
-        </is>
-      </c>
+      <c r="AC46" s="23" t="n"/>
     </row>
     <row r="47" ht="20.1" customHeight="1" s="1">
-      <c r="B47" s="16" t="n"/>
-      <c r="C47" s="17" t="inlineStr">
-        <is>
-          <t>FASE 2 · DOCUMENTACIÓN</t>
-        </is>
-      </c>
-      <c r="D47" s="16" t="n"/>
-      <c r="E47" s="16" t="n"/>
-      <c r="F47" s="16" t="n"/>
-      <c r="G47" s="16" t="n"/>
-      <c r="H47" s="16" t="n"/>
-      <c r="I47" s="16" t="n"/>
-      <c r="J47" s="16" t="n"/>
-      <c r="K47" s="16" t="n"/>
-      <c r="L47" s="16" t="n"/>
-      <c r="M47" s="16" t="n"/>
-      <c r="N47" s="16" t="n"/>
-      <c r="O47" s="16" t="n"/>
-      <c r="P47" s="16" t="n"/>
-      <c r="Q47" s="16" t="n"/>
-      <c r="R47" s="16" t="n"/>
-      <c r="S47" s="16" t="n"/>
-      <c r="T47" s="16" t="n"/>
-      <c r="U47" s="16" t="n"/>
-      <c r="V47" s="16" t="n"/>
-      <c r="W47" s="16" t="n"/>
-      <c r="X47" s="16" t="n"/>
-      <c r="Y47" s="16" t="n"/>
-      <c r="Z47" s="16" t="n"/>
-      <c r="AA47" s="16" t="n"/>
-      <c r="AB47" s="16" t="n"/>
-      <c r="AC47" s="16" t="n"/>
+      <c r="B47" s="18" t="n"/>
+      <c r="C47" s="19" t="inlineStr">
+        <is>
+          <t>Limpieza de código y CI (#54)</t>
+        </is>
+      </c>
+      <c r="D47" s="19" t="inlineStr">
+        <is>
+          <t>Nicko</t>
+        </is>
+      </c>
+      <c r="E47" s="20" t="n">
+        <v>46323</v>
+      </c>
+      <c r="F47" s="20" t="n">
+        <v>46325</v>
+      </c>
+      <c r="G47" s="19" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="H47" s="21" t="inlineStr">
+        <is>
+          <t>#54</t>
+        </is>
+      </c>
+      <c r="I47" s="22" t="n"/>
+      <c r="J47" s="22" t="n"/>
+      <c r="K47" s="22" t="n"/>
+      <c r="L47" s="22" t="n"/>
+      <c r="M47" s="22" t="n"/>
+      <c r="N47" s="22" t="n"/>
+      <c r="O47" s="22" t="n"/>
+      <c r="P47" s="22" t="n"/>
+      <c r="Q47" s="22" t="n"/>
+      <c r="R47" s="22" t="n"/>
+      <c r="S47" s="22" t="n"/>
+      <c r="T47" s="22" t="n"/>
+      <c r="U47" s="22" t="n"/>
+      <c r="V47" s="22" t="n"/>
+      <c r="W47" s="22" t="n"/>
+      <c r="X47" s="22" t="n"/>
+      <c r="Y47" s="22" t="n"/>
+      <c r="Z47" s="22" t="n"/>
+      <c r="AA47" s="22" t="n"/>
+      <c r="AC47" s="23" t="n"/>
     </row>
     <row r="48" ht="20.1" customHeight="1" s="1">
       <c r="B48" s="18" t="n"/>
       <c r="C48" s="19" t="inlineStr">
         <is>
-          <t>Registro de requisitos y plazos del curso</t>
+          <t>Primer demo operativo ante Walmart</t>
         </is>
       </c>
       <c r="D48" s="19" t="inlineStr">
         <is>
-          <t>Francisco</t>
+          <t>Nicko</t>
         </is>
       </c>
       <c r="E48" s="20" t="n">
-        <v>46304</v>
+        <v>46322</v>
       </c>
       <c r="F48" s="20" t="n">
-        <v>46305</v>
+        <v>46326</v>
       </c>
       <c r="G48" s="19" t="inlineStr">
         <is>
-          <t>Cumplido</t>
+          <t>Pendiente</t>
         </is>
       </c>
       <c r="H48" s="21" t="inlineStr">
         <is>
-          <t>#23, #25</t>
+          <t>#29</t>
         </is>
       </c>
       <c r="I48" s="22" t="n"/>
@@ -2690,34 +2701,34 @@
       <c r="Y48" s="22" t="n"/>
       <c r="Z48" s="22" t="n"/>
       <c r="AA48" s="22" t="n"/>
-      <c r="AC48" s="23" t="n"/>
+      <c r="AC48" s="23" t="inlineStr">
+        <is>
+          <t>Depende de #28</t>
+        </is>
+      </c>
     </row>
     <row r="49" ht="20.1" customHeight="1" s="1">
       <c r="B49" s="18" t="n"/>
       <c r="C49" s="19" t="inlineStr">
         <is>
-          <t>Casos de uso y diagramas alineados con Walmart</t>
+          <t>Instalación en el servidor del CITT</t>
         </is>
       </c>
       <c r="D49" s="19" t="inlineStr">
         <is>
-          <t>Francisco</t>
-        </is>
-      </c>
-      <c r="E49" s="20" t="n">
-        <v>46304</v>
-      </c>
-      <c r="F49" s="20" t="n">
-        <v>46305</v>
-      </c>
+          <t>Por definir</t>
+        </is>
+      </c>
+      <c r="E49" s="20" t="n"/>
+      <c r="F49" s="20" t="n"/>
       <c r="G49" s="19" t="inlineStr">
         <is>
-          <t>Cumplido</t>
+          <t>Bloqueado</t>
         </is>
       </c>
       <c r="H49" s="21" t="inlineStr">
         <is>
-          <t>#30</t>
+          <t>#39</t>
         </is>
       </c>
       <c r="I49" s="22" t="n"/>
@@ -2739,66 +2750,51 @@
       <c r="Y49" s="22" t="n"/>
       <c r="Z49" s="22" t="n"/>
       <c r="AA49" s="22" t="n"/>
-      <c r="AC49" s="23" t="n"/>
+      <c r="AC49" s="23" t="inlineStr">
+        <is>
+          <t>Faltan las instrucciones del CITT</t>
+        </is>
+      </c>
     </row>
     <row r="50" ht="20.1" customHeight="1" s="1">
-      <c r="B50" s="18" t="n"/>
-      <c r="C50" s="19" t="inlineStr">
-        <is>
-          <t>Plan de mejoras de la Fase 1</t>
-        </is>
-      </c>
-      <c r="D50" s="19" t="inlineStr">
-        <is>
-          <t>Mariana</t>
-        </is>
-      </c>
-      <c r="E50" s="20" t="n">
-        <v>46315</v>
-      </c>
-      <c r="F50" s="20" t="n">
-        <v>46315</v>
-      </c>
-      <c r="G50" s="19" t="inlineStr">
-        <is>
-          <t>Cumplido</t>
-        </is>
-      </c>
-      <c r="H50" s="21" t="inlineStr">
-        <is>
-          <t>#26</t>
-        </is>
-      </c>
-      <c r="I50" s="22" t="n"/>
-      <c r="J50" s="22" t="n"/>
-      <c r="K50" s="22" t="n"/>
-      <c r="L50" s="22" t="n"/>
-      <c r="M50" s="22" t="n"/>
-      <c r="N50" s="22" t="n"/>
-      <c r="O50" s="22" t="n"/>
-      <c r="P50" s="22" t="n"/>
-      <c r="Q50" s="22" t="n"/>
-      <c r="R50" s="22" t="n"/>
-      <c r="S50" s="22" t="n"/>
-      <c r="T50" s="22" t="n"/>
-      <c r="U50" s="22" t="n"/>
-      <c r="V50" s="22" t="n"/>
-      <c r="W50" s="22" t="n"/>
-      <c r="X50" s="22" t="n"/>
-      <c r="Y50" s="22" t="n"/>
-      <c r="Z50" s="22" t="n"/>
-      <c r="AA50" s="22" t="n"/>
-      <c r="AC50" s="23" t="inlineStr">
-        <is>
-          <t>Hecho el 2026-10-20, con atraso (plazo 2026-10-09). docs/plan-de-mejoras.md</t>
-        </is>
-      </c>
+      <c r="B50" s="16" t="n"/>
+      <c r="C50" s="17" t="inlineStr">
+        <is>
+          <t>FASE 2 · DOCUMENTACIÓN</t>
+        </is>
+      </c>
+      <c r="D50" s="16" t="n"/>
+      <c r="E50" s="16" t="n"/>
+      <c r="F50" s="16" t="n"/>
+      <c r="G50" s="16" t="n"/>
+      <c r="H50" s="16" t="n"/>
+      <c r="I50" s="16" t="n"/>
+      <c r="J50" s="16" t="n"/>
+      <c r="K50" s="16" t="n"/>
+      <c r="L50" s="16" t="n"/>
+      <c r="M50" s="16" t="n"/>
+      <c r="N50" s="16" t="n"/>
+      <c r="O50" s="16" t="n"/>
+      <c r="P50" s="16" t="n"/>
+      <c r="Q50" s="16" t="n"/>
+      <c r="R50" s="16" t="n"/>
+      <c r="S50" s="16" t="n"/>
+      <c r="T50" s="16" t="n"/>
+      <c r="U50" s="16" t="n"/>
+      <c r="V50" s="16" t="n"/>
+      <c r="W50" s="16" t="n"/>
+      <c r="X50" s="16" t="n"/>
+      <c r="Y50" s="16" t="n"/>
+      <c r="Z50" s="16" t="n"/>
+      <c r="AA50" s="16" t="n"/>
+      <c r="AB50" s="16" t="n"/>
+      <c r="AC50" s="16" t="n"/>
     </row>
     <row r="51" ht="20.1" customHeight="1" s="1">
       <c r="B51" s="18" t="n"/>
       <c r="C51" s="19" t="inlineStr">
         <is>
-          <t>Informe intermedio: estado de avance y conclusiones</t>
+          <t>Registro de requisitos y plazos del curso</t>
         </is>
       </c>
       <c r="D51" s="19" t="inlineStr">
@@ -2807,19 +2803,19 @@
         </is>
       </c>
       <c r="E51" s="20" t="n">
-        <v>46314</v>
+        <v>46304</v>
       </c>
       <c r="F51" s="20" t="n">
-        <v>46316</v>
+        <v>46305</v>
       </c>
       <c r="G51" s="19" t="inlineStr">
         <is>
-          <t>En curso</t>
+          <t>Cumplido</t>
         </is>
       </c>
       <c r="H51" s="21" t="inlineStr">
         <is>
-          <t>#27</t>
+          <t>#23, #25</t>
         </is>
       </c>
       <c r="I51" s="22" t="n"/>
@@ -2841,17 +2837,13 @@
       <c r="Y51" s="22" t="n"/>
       <c r="Z51" s="22" t="n"/>
       <c r="AA51" s="22" t="n"/>
-      <c r="AC51" s="23" t="inlineStr">
-        <is>
-          <t>Antes de Nicko; Francisco lo arma en Word</t>
-        </is>
-      </c>
+      <c r="AC51" s="23" t="n"/>
     </row>
     <row r="52" ht="20.1" customHeight="1" s="1">
       <c r="B52" s="18" t="n"/>
       <c r="C52" s="19" t="inlineStr">
         <is>
-          <t>Análisis de resultados: 10 mejores y 10 peores casos</t>
+          <t>Casos de uso y diagramas alineados con Walmart</t>
         </is>
       </c>
       <c r="D52" s="19" t="inlineStr">
@@ -2860,10 +2852,10 @@
         </is>
       </c>
       <c r="E52" s="20" t="n">
-        <v>46315</v>
+        <v>46304</v>
       </c>
       <c r="F52" s="20" t="n">
-        <v>46315</v>
+        <v>46305</v>
       </c>
       <c r="G52" s="19" t="inlineStr">
         <is>
@@ -2872,7 +2864,7 @@
       </c>
       <c r="H52" s="21" t="inlineStr">
         <is>
-          <t>#34</t>
+          <t>#30</t>
         </is>
       </c>
       <c r="I52" s="22" t="n"/>
@@ -2900,12 +2892,12 @@
       <c r="B53" s="18" t="n"/>
       <c r="C53" s="19" t="inlineStr">
         <is>
-          <t>README completo</t>
+          <t>Plan de mejoras de la Fase 1</t>
         </is>
       </c>
       <c r="D53" s="19" t="inlineStr">
         <is>
-          <t>Francisco</t>
+          <t>Mariana</t>
         </is>
       </c>
       <c r="E53" s="20" t="n">
@@ -2921,7 +2913,7 @@
       </c>
       <c r="H53" s="21" t="inlineStr">
         <is>
-          <t>#35</t>
+          <t>#26</t>
         </is>
       </c>
       <c r="I53" s="22" t="n"/>
@@ -2943,34 +2935,38 @@
       <c r="Y53" s="22" t="n"/>
       <c r="Z53" s="22" t="n"/>
       <c r="AA53" s="22" t="n"/>
-      <c r="AC53" s="23" t="n"/>
+      <c r="AC53" s="23" t="inlineStr">
+        <is>
+          <t>Hecho el 2026-10-20, con atraso (plazo 2026-10-09). docs/plan-de-mejoras.md</t>
+        </is>
+      </c>
     </row>
     <row r="54" ht="20.1" customHeight="1" s="1">
       <c r="B54" s="18" t="n"/>
       <c r="C54" s="19" t="inlineStr">
         <is>
-          <t>Video de demostración (5 a 10 min)</t>
+          <t>Informe intermedio: estado de avance y conclusiones</t>
         </is>
       </c>
       <c r="D54" s="19" t="inlineStr">
         <is>
-          <t>Nicko</t>
+          <t>Francisco</t>
         </is>
       </c>
       <c r="E54" s="20" t="n">
-        <v>46316</v>
+        <v>46314</v>
       </c>
       <c r="F54" s="20" t="n">
         <v>46316</v>
       </c>
       <c r="G54" s="19" t="inlineStr">
         <is>
-          <t>Pendiente</t>
+          <t>En curso</t>
         </is>
       </c>
       <c r="H54" s="21" t="inlineStr">
         <is>
-          <t>#36</t>
+          <t>#27</t>
         </is>
       </c>
       <c r="I54" s="22" t="n"/>
@@ -2992,34 +2988,38 @@
       <c r="Y54" s="22" t="n"/>
       <c r="Z54" s="22" t="n"/>
       <c r="AA54" s="22" t="n"/>
-      <c r="AC54" s="23" t="n"/>
+      <c r="AC54" s="23" t="inlineStr">
+        <is>
+          <t>Antes de Nicko; Francisco lo arma en Word</t>
+        </is>
+      </c>
     </row>
     <row r="55" ht="20.1" customHeight="1" s="1">
       <c r="B55" s="18" t="n"/>
       <c r="C55" s="19" t="inlineStr">
         <is>
-          <t>Evidencias de avance: diario 2.1 y guía 2.4</t>
+          <t>Análisis de resultados: 10 mejores y 10 peores casos</t>
         </is>
       </c>
       <c r="D55" s="19" t="inlineStr">
         <is>
-          <t>Mariana</t>
+          <t>Francisco</t>
         </is>
       </c>
       <c r="E55" s="20" t="n">
         <v>46315</v>
       </c>
       <c r="F55" s="20" t="n">
-        <v>46321</v>
+        <v>46315</v>
       </c>
       <c r="G55" s="19" t="inlineStr">
         <is>
-          <t>En curso</t>
+          <t>Cumplido</t>
         </is>
       </c>
       <c r="H55" s="21" t="inlineStr">
         <is>
-          <t>#37</t>
+          <t>#34</t>
         </is>
       </c>
       <c r="I55" s="22" t="n"/>
@@ -3041,29 +3041,25 @@
       <c r="Y55" s="22" t="n"/>
       <c r="Z55" s="22" t="n"/>
       <c r="AA55" s="22" t="n"/>
-      <c r="AC55" s="23" t="inlineStr">
-        <is>
-          <t>Plazo 2026-10-26. Guía 2.4 llenada el 2026-10-20 (Fase 2/); falta el diario 2.1 y las partes de opinión del equipo</t>
-        </is>
-      </c>
+      <c r="AC55" s="23" t="n"/>
     </row>
     <row r="56" ht="20.1" customHeight="1" s="1">
       <c r="B56" s="18" t="n"/>
       <c r="C56" s="19" t="inlineStr">
         <is>
-          <t>Rehacer plantillas de C.U y diagramas según la app Django</t>
+          <t>README completo</t>
         </is>
       </c>
       <c r="D56" s="19" t="inlineStr">
         <is>
-          <t>Mariana</t>
+          <t>Francisco</t>
         </is>
       </c>
       <c r="E56" s="20" t="n">
-        <v>46316</v>
+        <v>46315</v>
       </c>
       <c r="F56" s="20" t="n">
-        <v>46316</v>
+        <v>46315</v>
       </c>
       <c r="G56" s="19" t="inlineStr">
         <is>
@@ -3072,7 +3068,7 @@
       </c>
       <c r="H56" s="21" t="inlineStr">
         <is>
-          <t>#42</t>
+          <t>#35</t>
         </is>
       </c>
       <c r="I56" s="22" t="n"/>
@@ -3094,70 +3090,85 @@
       <c r="Y56" s="22" t="n"/>
       <c r="Z56" s="22" t="n"/>
       <c r="AA56" s="22" t="n"/>
-      <c r="AC56" s="23" t="inlineStr">
-        <is>
-          <t>Hecho el 2026-10-21: plantillas, fuentes Mermaid y PNG (CU00-CU06 y arquitectura). docs/cambios-cu.md</t>
-        </is>
-      </c>
+      <c r="AC56" s="23" t="n"/>
     </row>
     <row r="57" ht="20.1" customHeight="1" s="1">
-      <c r="B57" s="16" t="n"/>
-      <c r="C57" s="17" t="inlineStr">
-        <is>
-          <t>HITOS DEL CURSO</t>
-        </is>
-      </c>
-      <c r="D57" s="16" t="n"/>
-      <c r="E57" s="16" t="n"/>
-      <c r="F57" s="16" t="n"/>
-      <c r="G57" s="16" t="n"/>
-      <c r="H57" s="16" t="n"/>
-      <c r="I57" s="16" t="n"/>
-      <c r="J57" s="16" t="n"/>
-      <c r="K57" s="16" t="n"/>
-      <c r="L57" s="16" t="n"/>
-      <c r="M57" s="16" t="n"/>
-      <c r="N57" s="16" t="n"/>
-      <c r="O57" s="16" t="n"/>
-      <c r="P57" s="16" t="n"/>
-      <c r="Q57" s="16" t="n"/>
-      <c r="R57" s="16" t="n"/>
-      <c r="S57" s="16" t="n"/>
-      <c r="T57" s="16" t="n"/>
-      <c r="U57" s="16" t="n"/>
-      <c r="V57" s="16" t="n"/>
-      <c r="W57" s="16" t="n"/>
-      <c r="X57" s="16" t="n"/>
-      <c r="Y57" s="16" t="n"/>
-      <c r="Z57" s="16" t="n"/>
-      <c r="AA57" s="16" t="n"/>
-      <c r="AB57" s="16" t="n"/>
-      <c r="AC57" s="16" t="n"/>
+      <c r="B57" s="18" t="n"/>
+      <c r="C57" s="19" t="inlineStr">
+        <is>
+          <t>Video de demostración (5 a 10 min)</t>
+        </is>
+      </c>
+      <c r="D57" s="19" t="inlineStr">
+        <is>
+          <t>Nicko</t>
+        </is>
+      </c>
+      <c r="E57" s="20" t="n">
+        <v>46316</v>
+      </c>
+      <c r="F57" s="20" t="n">
+        <v>46316</v>
+      </c>
+      <c r="G57" s="19" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="H57" s="21" t="inlineStr">
+        <is>
+          <t>#36</t>
+        </is>
+      </c>
+      <c r="I57" s="22" t="n"/>
+      <c r="J57" s="22" t="n"/>
+      <c r="K57" s="22" t="n"/>
+      <c r="L57" s="22" t="n"/>
+      <c r="M57" s="22" t="n"/>
+      <c r="N57" s="22" t="n"/>
+      <c r="O57" s="22" t="n"/>
+      <c r="P57" s="22" t="n"/>
+      <c r="Q57" s="22" t="n"/>
+      <c r="R57" s="22" t="n"/>
+      <c r="S57" s="22" t="n"/>
+      <c r="T57" s="22" t="n"/>
+      <c r="U57" s="22" t="n"/>
+      <c r="V57" s="22" t="n"/>
+      <c r="W57" s="22" t="n"/>
+      <c r="X57" s="22" t="n"/>
+      <c r="Y57" s="22" t="n"/>
+      <c r="Z57" s="22" t="n"/>
+      <c r="AA57" s="22" t="n"/>
+      <c r="AC57" s="23" t="n"/>
     </row>
     <row r="58" ht="20.1" customHeight="1" s="1">
       <c r="B58" s="18" t="n"/>
       <c r="C58" s="19" t="inlineStr">
         <is>
-          <t>Informe intermedio y video</t>
+          <t>Evidencias de avance: diario 2.1 y guía 2.4</t>
         </is>
       </c>
       <c r="D58" s="19" t="inlineStr">
         <is>
-          <t>Equipo</t>
+          <t>Mariana</t>
         </is>
       </c>
       <c r="E58" s="20" t="n">
-        <v>46316</v>
+        <v>46315</v>
       </c>
       <c r="F58" s="20" t="n">
-        <v>46316</v>
+        <v>46321</v>
       </c>
       <c r="G58" s="19" t="inlineStr">
         <is>
           <t>En curso</t>
         </is>
       </c>
-      <c r="H58" s="21" t="n"/>
+      <c r="H58" s="21" t="inlineStr">
+        <is>
+          <t>#37</t>
+        </is>
+      </c>
       <c r="I58" s="22" t="n"/>
       <c r="J58" s="22" t="n"/>
       <c r="K58" s="22" t="n"/>
@@ -3179,7 +3190,7 @@
       <c r="AA58" s="22" t="n"/>
       <c r="AC58" s="23" t="inlineStr">
         <is>
-          <t>Entrega 2026-10-21</t>
+          <t>Plazo 2026-10-26. Guía 2.4 llenada el 2026-10-20 (Fase 2/); falta el diario 2.1 y las partes de opinión del equipo</t>
         </is>
       </c>
     </row>
@@ -3187,28 +3198,28 @@
       <c r="B59" s="18" t="n"/>
       <c r="C59" s="19" t="inlineStr">
         <is>
-          <t>Feria de informática</t>
+          <t>Rehacer plantillas de C.U y diagramas según la app Django</t>
         </is>
       </c>
       <c r="D59" s="19" t="inlineStr">
         <is>
-          <t>Nicko</t>
+          <t>Mariana</t>
         </is>
       </c>
       <c r="E59" s="20" t="n">
-        <v>46321</v>
+        <v>46316</v>
       </c>
       <c r="F59" s="20" t="n">
-        <v>46325</v>
+        <v>46316</v>
       </c>
       <c r="G59" s="19" t="inlineStr">
         <is>
-          <t>Pendiente</t>
+          <t>Cumplido</t>
         </is>
       </c>
       <c r="H59" s="21" t="inlineStr">
         <is>
-          <t>#38</t>
+          <t>#42</t>
         </is>
       </c>
       <c r="I59" s="22" t="n"/>
@@ -3232,64 +3243,49 @@
       <c r="AA59" s="22" t="n"/>
       <c r="AC59" s="23" t="inlineStr">
         <is>
-          <t>Día y hora por informar</t>
+          <t>Hecho el 2026-10-21: plantillas, fuentes Mermaid y PNG (CU00-CU06 y arquitectura). docs/cambios-cu.md</t>
         </is>
       </c>
     </row>
     <row r="60" ht="20.1" customHeight="1" s="1">
-      <c r="B60" s="18" t="n"/>
-      <c r="C60" s="19" t="inlineStr">
-        <is>
-          <t>Evaluación 2 (Avance): 50% de los C.U y demo del Sprint 1</t>
-        </is>
-      </c>
-      <c r="D60" s="19" t="inlineStr">
-        <is>
-          <t>Equipo</t>
-        </is>
-      </c>
-      <c r="E60" s="20" t="n">
-        <v>46323</v>
-      </c>
-      <c r="F60" s="20" t="n">
-        <v>46325</v>
-      </c>
-      <c r="G60" s="19" t="inlineStr">
-        <is>
-          <t>Pendiente</t>
-        </is>
-      </c>
-      <c r="H60" s="21" t="n"/>
-      <c r="I60" s="22" t="n"/>
-      <c r="J60" s="22" t="n"/>
-      <c r="K60" s="22" t="n"/>
-      <c r="L60" s="22" t="n"/>
-      <c r="M60" s="22" t="n"/>
-      <c r="N60" s="22" t="n"/>
-      <c r="O60" s="22" t="n"/>
-      <c r="P60" s="22" t="n"/>
-      <c r="Q60" s="22" t="n"/>
-      <c r="R60" s="22" t="n"/>
-      <c r="S60" s="22" t="n"/>
-      <c r="T60" s="22" t="n"/>
-      <c r="U60" s="22" t="n"/>
-      <c r="V60" s="22" t="n"/>
-      <c r="W60" s="22" t="n"/>
-      <c r="X60" s="22" t="n"/>
-      <c r="Y60" s="22" t="n"/>
-      <c r="Z60" s="22" t="n"/>
-      <c r="AA60" s="22" t="n"/>
-      <c r="AC60" s="23" t="inlineStr">
-        <is>
-          <t>Día exacto por confirmar</t>
-        </is>
-      </c>
+      <c r="B60" s="16" t="n"/>
+      <c r="C60" s="17" t="inlineStr">
+        <is>
+          <t>HITOS DEL CURSO</t>
+        </is>
+      </c>
+      <c r="D60" s="16" t="n"/>
+      <c r="E60" s="16" t="n"/>
+      <c r="F60" s="16" t="n"/>
+      <c r="G60" s="16" t="n"/>
+      <c r="H60" s="16" t="n"/>
+      <c r="I60" s="16" t="n"/>
+      <c r="J60" s="16" t="n"/>
+      <c r="K60" s="16" t="n"/>
+      <c r="L60" s="16" t="n"/>
+      <c r="M60" s="16" t="n"/>
+      <c r="N60" s="16" t="n"/>
+      <c r="O60" s="16" t="n"/>
+      <c r="P60" s="16" t="n"/>
+      <c r="Q60" s="16" t="n"/>
+      <c r="R60" s="16" t="n"/>
+      <c r="S60" s="16" t="n"/>
+      <c r="T60" s="16" t="n"/>
+      <c r="U60" s="16" t="n"/>
+      <c r="V60" s="16" t="n"/>
+      <c r="W60" s="16" t="n"/>
+      <c r="X60" s="16" t="n"/>
+      <c r="Y60" s="16" t="n"/>
+      <c r="Z60" s="16" t="n"/>
+      <c r="AA60" s="16" t="n"/>
+      <c r="AB60" s="16" t="n"/>
+      <c r="AC60" s="16" t="n"/>
     </row>
     <row r="61" ht="20.1" customHeight="1" s="1">
       <c r="B61" s="18" t="n"/>
       <c r="C61" s="19" t="inlineStr">
         <is>
-          <t>Entrega final de la Fase 2</t>
+          <t>Informe intermedio y video</t>
         </is>
       </c>
       <c r="D61" s="19" t="inlineStr">
@@ -3298,14 +3294,14 @@
         </is>
       </c>
       <c r="E61" s="20" t="n">
-        <v>46349</v>
+        <v>46316</v>
       </c>
       <c r="F61" s="20" t="n">
-        <v>46353</v>
+        <v>46316</v>
       </c>
       <c r="G61" s="19" t="inlineStr">
         <is>
-          <t>Pendiente</t>
+          <t>En curso</t>
         </is>
       </c>
       <c r="H61" s="21" t="n"/>
@@ -3330,49 +3326,68 @@
       <c r="AA61" s="22" t="n"/>
       <c r="AC61" s="23" t="inlineStr">
         <is>
-          <t>Semana 15, por confirmar</t>
+          <t>Entrega 2026-10-21</t>
         </is>
       </c>
     </row>
     <row r="62" ht="20.1" customHeight="1" s="1">
-      <c r="B62" s="16" t="n"/>
-      <c r="C62" s="17" t="inlineStr">
-        <is>
-          <t>FASE 3</t>
-        </is>
-      </c>
-      <c r="D62" s="16" t="n"/>
-      <c r="E62" s="16" t="n"/>
-      <c r="F62" s="16" t="n"/>
-      <c r="G62" s="16" t="n"/>
-      <c r="H62" s="16" t="n"/>
-      <c r="I62" s="16" t="n"/>
-      <c r="J62" s="16" t="n"/>
-      <c r="K62" s="16" t="n"/>
-      <c r="L62" s="16" t="n"/>
-      <c r="M62" s="16" t="n"/>
-      <c r="N62" s="16" t="n"/>
-      <c r="O62" s="16" t="n"/>
-      <c r="P62" s="16" t="n"/>
-      <c r="Q62" s="16" t="n"/>
-      <c r="R62" s="16" t="n"/>
-      <c r="S62" s="16" t="n"/>
-      <c r="T62" s="16" t="n"/>
-      <c r="U62" s="16" t="n"/>
-      <c r="V62" s="16" t="n"/>
-      <c r="W62" s="16" t="n"/>
-      <c r="X62" s="16" t="n"/>
-      <c r="Y62" s="16" t="n"/>
-      <c r="Z62" s="16" t="n"/>
-      <c r="AA62" s="16" t="n"/>
-      <c r="AB62" s="16" t="n"/>
-      <c r="AC62" s="16" t="n"/>
+      <c r="B62" s="18" t="n"/>
+      <c r="C62" s="19" t="inlineStr">
+        <is>
+          <t>Feria de informática</t>
+        </is>
+      </c>
+      <c r="D62" s="19" t="inlineStr">
+        <is>
+          <t>Nicko</t>
+        </is>
+      </c>
+      <c r="E62" s="20" t="n">
+        <v>46321</v>
+      </c>
+      <c r="F62" s="20" t="n">
+        <v>46325</v>
+      </c>
+      <c r="G62" s="19" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="H62" s="21" t="inlineStr">
+        <is>
+          <t>#38</t>
+        </is>
+      </c>
+      <c r="I62" s="22" t="n"/>
+      <c r="J62" s="22" t="n"/>
+      <c r="K62" s="22" t="n"/>
+      <c r="L62" s="22" t="n"/>
+      <c r="M62" s="22" t="n"/>
+      <c r="N62" s="22" t="n"/>
+      <c r="O62" s="22" t="n"/>
+      <c r="P62" s="22" t="n"/>
+      <c r="Q62" s="22" t="n"/>
+      <c r="R62" s="22" t="n"/>
+      <c r="S62" s="22" t="n"/>
+      <c r="T62" s="22" t="n"/>
+      <c r="U62" s="22" t="n"/>
+      <c r="V62" s="22" t="n"/>
+      <c r="W62" s="22" t="n"/>
+      <c r="X62" s="22" t="n"/>
+      <c r="Y62" s="22" t="n"/>
+      <c r="Z62" s="22" t="n"/>
+      <c r="AA62" s="22" t="n"/>
+      <c r="AC62" s="23" t="inlineStr">
+        <is>
+          <t>Día y hora por informar</t>
+        </is>
+      </c>
     </row>
     <row r="63" ht="20.1" customHeight="1" s="1">
       <c r="B63" s="18" t="n"/>
       <c r="C63" s="19" t="inlineStr">
         <is>
-          <t>Ajustes finales, manuales y exposición ante la Comisión</t>
+          <t>Evaluación 2 (Avance): 50% de los C.U y demo del Sprint 1</t>
         </is>
       </c>
       <c r="D63" s="19" t="inlineStr">
@@ -3381,10 +3396,10 @@
         </is>
       </c>
       <c r="E63" s="20" t="n">
-        <v>46356</v>
+        <v>46323</v>
       </c>
       <c r="F63" s="20" t="n">
-        <v>46374</v>
+        <v>46325</v>
       </c>
       <c r="G63" s="19" t="inlineStr">
         <is>
@@ -3413,13 +3428,142 @@
       <c r="AA63" s="22" t="n"/>
       <c r="AC63" s="23" t="inlineStr">
         <is>
+          <t>Día exacto por confirmar</t>
+        </is>
+      </c>
+    </row>
+    <row r="64" ht="20.1" customHeight="1" s="1">
+      <c r="B64" s="18" t="n"/>
+      <c r="C64" s="19" t="inlineStr">
+        <is>
+          <t>Entrega final de la Fase 2</t>
+        </is>
+      </c>
+      <c r="D64" s="19" t="inlineStr">
+        <is>
+          <t>Equipo</t>
+        </is>
+      </c>
+      <c r="E64" s="20" t="n">
+        <v>46349</v>
+      </c>
+      <c r="F64" s="20" t="n">
+        <v>46353</v>
+      </c>
+      <c r="G64" s="19" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="H64" s="21" t="n"/>
+      <c r="I64" s="22" t="n"/>
+      <c r="J64" s="22" t="n"/>
+      <c r="K64" s="22" t="n"/>
+      <c r="L64" s="22" t="n"/>
+      <c r="M64" s="22" t="n"/>
+      <c r="N64" s="22" t="n"/>
+      <c r="O64" s="22" t="n"/>
+      <c r="P64" s="22" t="n"/>
+      <c r="Q64" s="22" t="n"/>
+      <c r="R64" s="22" t="n"/>
+      <c r="S64" s="22" t="n"/>
+      <c r="T64" s="22" t="n"/>
+      <c r="U64" s="22" t="n"/>
+      <c r="V64" s="22" t="n"/>
+      <c r="W64" s="22" t="n"/>
+      <c r="X64" s="22" t="n"/>
+      <c r="Y64" s="22" t="n"/>
+      <c r="Z64" s="22" t="n"/>
+      <c r="AA64" s="22" t="n"/>
+      <c r="AC64" s="23" t="inlineStr">
+        <is>
+          <t>Semana 15, por confirmar</t>
+        </is>
+      </c>
+    </row>
+    <row r="65" ht="20.1" customHeight="1" s="1">
+      <c r="B65" s="16" t="n"/>
+      <c r="C65" s="17" t="inlineStr">
+        <is>
+          <t>FASE 3</t>
+        </is>
+      </c>
+      <c r="D65" s="16" t="n"/>
+      <c r="E65" s="16" t="n"/>
+      <c r="F65" s="16" t="n"/>
+      <c r="G65" s="16" t="n"/>
+      <c r="H65" s="16" t="n"/>
+      <c r="I65" s="16" t="n"/>
+      <c r="J65" s="16" t="n"/>
+      <c r="K65" s="16" t="n"/>
+      <c r="L65" s="16" t="n"/>
+      <c r="M65" s="16" t="n"/>
+      <c r="N65" s="16" t="n"/>
+      <c r="O65" s="16" t="n"/>
+      <c r="P65" s="16" t="n"/>
+      <c r="Q65" s="16" t="n"/>
+      <c r="R65" s="16" t="n"/>
+      <c r="S65" s="16" t="n"/>
+      <c r="T65" s="16" t="n"/>
+      <c r="U65" s="16" t="n"/>
+      <c r="V65" s="16" t="n"/>
+      <c r="W65" s="16" t="n"/>
+      <c r="X65" s="16" t="n"/>
+      <c r="Y65" s="16" t="n"/>
+      <c r="Z65" s="16" t="n"/>
+      <c r="AA65" s="16" t="n"/>
+      <c r="AB65" s="16" t="n"/>
+      <c r="AC65" s="16" t="n"/>
+    </row>
+    <row r="66" ht="20.1" customHeight="1" s="1">
+      <c r="B66" s="18" t="n"/>
+      <c r="C66" s="19" t="inlineStr">
+        <is>
+          <t>Ajustes finales, manuales y exposición ante la Comisión</t>
+        </is>
+      </c>
+      <c r="D66" s="19" t="inlineStr">
+        <is>
+          <t>Equipo</t>
+        </is>
+      </c>
+      <c r="E66" s="20" t="n">
+        <v>46356</v>
+      </c>
+      <c r="F66" s="20" t="n">
+        <v>46374</v>
+      </c>
+      <c r="G66" s="19" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="H66" s="21" t="n"/>
+      <c r="I66" s="22" t="n"/>
+      <c r="J66" s="22" t="n"/>
+      <c r="K66" s="22" t="n"/>
+      <c r="L66" s="22" t="n"/>
+      <c r="M66" s="22" t="n"/>
+      <c r="N66" s="22" t="n"/>
+      <c r="O66" s="22" t="n"/>
+      <c r="P66" s="22" t="n"/>
+      <c r="Q66" s="22" t="n"/>
+      <c r="R66" s="22" t="n"/>
+      <c r="S66" s="22" t="n"/>
+      <c r="T66" s="22" t="n"/>
+      <c r="U66" s="22" t="n"/>
+      <c r="V66" s="22" t="n"/>
+      <c r="W66" s="22" t="n"/>
+      <c r="X66" s="22" t="n"/>
+      <c r="Y66" s="22" t="n"/>
+      <c r="Z66" s="22" t="n"/>
+      <c r="AA66" s="22" t="n"/>
+      <c r="AC66" s="23" t="inlineStr">
+        <is>
           <t>Fechas por definir</t>
         </is>
       </c>
     </row>
-    <row r="64" ht="15.75" customHeight="1" s="1"/>
-    <row r="65" ht="15.75" customHeight="1" s="1"/>
-    <row r="66" ht="15.75" customHeight="1" s="1"/>
     <row r="67" ht="15.75" customHeight="1" s="1"/>
     <row r="68" ht="15.75" customHeight="1" s="1"/>
     <row r="69" ht="15.75" customHeight="1" s="1"/>
@@ -4363,7 +4507,7 @@
     <mergeCell ref="Q8:T8"/>
     <mergeCell ref="I8:L8"/>
   </mergeCells>
-  <conditionalFormatting sqref="B10:B63">
+  <conditionalFormatting sqref="B10:B66">
     <cfRule type="expression" priority="2" dxfId="5" stopIfTrue="1">
       <formula>$G10="Cumplido"</formula>
     </cfRule>
@@ -4380,7 +4524,7 @@
       <formula>$G10="Bloqueado"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="I10:AA63">
+  <conditionalFormatting sqref="I10:AA66">
     <cfRule type="expression" priority="1" dxfId="5" stopIfTrue="1">
       <formula>AND($E10&lt;&gt;"",I$9&lt;=$F10,I$9+6&gt;=$E10,$G10="Cumplido")</formula>
     </cfRule>
@@ -4397,7 +4541,7 @@
       <formula>AND($E10&lt;&gt;"",I$9&lt;=$F10,I$9+6&gt;=$E10,$G10="Bloqueado")</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="S10:S63">
+  <conditionalFormatting sqref="S10:S66">
     <cfRule type="expression" priority="11" dxfId="0">
       <formula>$G10&lt;&gt;""</formula>
     </cfRule>

</xml_diff>

<commit_message>
docs: assign items #43, #44, #52 and #53 to Mariana
</commit_message>
<xml_diff>
--- a/Anexos/Gestion/Carta Gantt Fase 2.xlsx
+++ b/Anexos/Gestion/Carta Gantt Fase 2.xlsx
@@ -10,7 +10,7 @@
   </sheets>
   <definedNames>
     <definedName name="_xlnm.Print_Titles" localSheetId="0">'Carta Gantt'!$8:$9</definedName>
-    <definedName name="_xlnm.Print_Area" localSheetId="0">'Carta Gantt'!$B$1:$AC$66</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="0">'Carta Gantt'!$B$1:$AC$67</definedName>
   </definedNames>
   <calcPr calcId="191029" fullCalcOnLoad="1"/>
 </workbook>
@@ -655,7 +655,7 @@
     <outlinePr summaryBelow="0" summaryRight="0"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:AC66"/>
+  <dimension ref="A1:AC67"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="12.5703125" defaultRowHeight="15" customHeight="1"/>
   <cols>
     <col width="2" customWidth="1" style="1" min="1" max="1"/>
@@ -695,23 +695,23 @@
     <row r="4" ht="15.75" customHeight="1" s="1"/>
     <row r="5" ht="26.1" customHeight="1" s="1">
       <c r="D5" s="5">
-        <f>COUNTIF($G$10:$G$66,"Cumplido")</f>
+        <f>COUNTIF($G$10:$G$67,"Cumplido")</f>
         <v/>
       </c>
       <c r="E5" s="6">
-        <f>COUNTIF($G$10:$G$66,"En curso")</f>
+        <f>COUNTIF($G$10:$G$67,"En curso")</f>
         <v/>
       </c>
       <c r="F5" s="7">
-        <f>COUNTIF($G$10:$G$66,"Pendiente")</f>
+        <f>COUNTIF($G$10:$G$67,"Pendiente")</f>
         <v/>
       </c>
       <c r="G5" s="8">
-        <f>COUNTIF($G$10:$G$66,"Atrasado")</f>
+        <f>COUNTIF($G$10:$G$67,"Atrasado")</f>
         <v/>
       </c>
       <c r="H5" s="9">
-        <f>COUNTIF($G$10:$G$66,"Bloqueado")</f>
+        <f>COUNTIF($G$10:$G$67,"Bloqueado")</f>
         <v/>
       </c>
     </row>
@@ -2603,24 +2603,28 @@
       <c r="Y46" s="22" t="n"/>
       <c r="Z46" s="22" t="n"/>
       <c r="AA46" s="22" t="n"/>
-      <c r="AC46" s="23" t="n"/>
+      <c r="AC46" s="23" t="inlineStr">
+        <is>
+          <t>Francisco: #49 a #51; Mariana: #52 y #53</t>
+        </is>
+      </c>
     </row>
     <row r="47" ht="20.1" customHeight="1" s="1">
       <c r="B47" s="18" t="n"/>
       <c r="C47" s="19" t="inlineStr">
         <is>
-          <t>Limpieza de código y CI (#54)</t>
+          <t>Dashboard (CU03) y configuración de umbral y cámaras (CU05)</t>
         </is>
       </c>
       <c r="D47" s="19" t="inlineStr">
         <is>
-          <t>Nicko</t>
-        </is>
-      </c>
-      <c r="E47" s="20" t="n">
+          <t>Mariana</t>
+        </is>
+      </c>
+      <c r="E47" s="20">
         <v>46323</v>
       </c>
-      <c r="F47" s="20" t="n">
+      <c r="F47" s="20">
         <v>46325</v>
       </c>
       <c r="G47" s="19" t="inlineStr">
@@ -2630,7 +2634,7 @@
       </c>
       <c r="H47" s="21" t="inlineStr">
         <is>
-          <t>#54</t>
+          <t>#43, #44</t>
         </is>
       </c>
       <c r="I47" s="22" t="n"/>
@@ -2652,13 +2656,17 @@
       <c r="Y47" s="22" t="n"/>
       <c r="Z47" s="22" t="n"/>
       <c r="AA47" s="22" t="n"/>
-      <c r="AC47" s="23" t="n"/>
+      <c r="AC47" s="23" t="inlineStr">
+        <is>
+          <t>Fechas propuestas, a confirmar</t>
+        </is>
+      </c>
     </row>
     <row r="48" ht="20.1" customHeight="1" s="1">
       <c r="B48" s="18" t="n"/>
       <c r="C48" s="19" t="inlineStr">
         <is>
-          <t>Primer demo operativo ante Walmart</t>
+          <t>Limpieza de código y CI (#54)</t>
         </is>
       </c>
       <c r="D48" s="19" t="inlineStr">
@@ -2667,10 +2675,10 @@
         </is>
       </c>
       <c r="E48" s="20" t="n">
-        <v>46322</v>
+        <v>46323</v>
       </c>
       <c r="F48" s="20" t="n">
-        <v>46326</v>
+        <v>46325</v>
       </c>
       <c r="G48" s="19" t="inlineStr">
         <is>
@@ -2679,7 +2687,7 @@
       </c>
       <c r="H48" s="21" t="inlineStr">
         <is>
-          <t>#29</t>
+          <t>#54</t>
         </is>
       </c>
       <c r="I48" s="22" t="n"/>
@@ -2701,34 +2709,34 @@
       <c r="Y48" s="22" t="n"/>
       <c r="Z48" s="22" t="n"/>
       <c r="AA48" s="22" t="n"/>
-      <c r="AC48" s="23" t="inlineStr">
-        <is>
-          <t>Depende de #28</t>
-        </is>
-      </c>
+      <c r="AC48" s="23" t="n"/>
     </row>
     <row r="49" ht="20.1" customHeight="1" s="1">
       <c r="B49" s="18" t="n"/>
       <c r="C49" s="19" t="inlineStr">
         <is>
-          <t>Instalación en el servidor del CITT</t>
+          <t>Primer demo operativo ante Walmart</t>
         </is>
       </c>
       <c r="D49" s="19" t="inlineStr">
         <is>
-          <t>Por definir</t>
-        </is>
-      </c>
-      <c r="E49" s="20" t="n"/>
-      <c r="F49" s="20" t="n"/>
+          <t>Nicko</t>
+        </is>
+      </c>
+      <c r="E49" s="20" t="n">
+        <v>46322</v>
+      </c>
+      <c r="F49" s="20" t="n">
+        <v>46326</v>
+      </c>
       <c r="G49" s="19" t="inlineStr">
         <is>
-          <t>Bloqueado</t>
+          <t>Pendiente</t>
         </is>
       </c>
       <c r="H49" s="21" t="inlineStr">
         <is>
-          <t>#39</t>
+          <t>#29</t>
         </is>
       </c>
       <c r="I49" s="22" t="n"/>
@@ -2752,98 +2760,98 @@
       <c r="AA49" s="22" t="n"/>
       <c r="AC49" s="23" t="inlineStr">
         <is>
+          <t>Depende de #28</t>
+        </is>
+      </c>
+    </row>
+    <row r="50" ht="20.1" customHeight="1" s="1">
+      <c r="B50" s="18" t="n"/>
+      <c r="C50" s="19" t="inlineStr">
+        <is>
+          <t>Instalación en el servidor del CITT</t>
+        </is>
+      </c>
+      <c r="D50" s="19" t="inlineStr">
+        <is>
+          <t>Por definir</t>
+        </is>
+      </c>
+      <c r="E50" s="20" t="n"/>
+      <c r="F50" s="20" t="n"/>
+      <c r="G50" s="19" t="inlineStr">
+        <is>
+          <t>Bloqueado</t>
+        </is>
+      </c>
+      <c r="H50" s="21" t="inlineStr">
+        <is>
+          <t>#39</t>
+        </is>
+      </c>
+      <c r="I50" s="22" t="n"/>
+      <c r="J50" s="22" t="n"/>
+      <c r="K50" s="22" t="n"/>
+      <c r="L50" s="22" t="n"/>
+      <c r="M50" s="22" t="n"/>
+      <c r="N50" s="22" t="n"/>
+      <c r="O50" s="22" t="n"/>
+      <c r="P50" s="22" t="n"/>
+      <c r="Q50" s="22" t="n"/>
+      <c r="R50" s="22" t="n"/>
+      <c r="S50" s="22" t="n"/>
+      <c r="T50" s="22" t="n"/>
+      <c r="U50" s="22" t="n"/>
+      <c r="V50" s="22" t="n"/>
+      <c r="W50" s="22" t="n"/>
+      <c r="X50" s="22" t="n"/>
+      <c r="Y50" s="22" t="n"/>
+      <c r="Z50" s="22" t="n"/>
+      <c r="AA50" s="22" t="n"/>
+      <c r="AC50" s="23" t="inlineStr">
+        <is>
           <t>Faltan las instrucciones del CITT</t>
         </is>
       </c>
     </row>
-    <row r="50" ht="20.1" customHeight="1" s="1">
-      <c r="B50" s="16" t="n"/>
-      <c r="C50" s="17" t="inlineStr">
+    <row r="51" ht="20.1" customHeight="1" s="1">
+      <c r="B51" s="16" t="n"/>
+      <c r="C51" s="17" t="inlineStr">
         <is>
           <t>FASE 2 · DOCUMENTACIÓN</t>
         </is>
       </c>
-      <c r="D50" s="16" t="n"/>
-      <c r="E50" s="16" t="n"/>
-      <c r="F50" s="16" t="n"/>
-      <c r="G50" s="16" t="n"/>
-      <c r="H50" s="16" t="n"/>
-      <c r="I50" s="16" t="n"/>
-      <c r="J50" s="16" t="n"/>
-      <c r="K50" s="16" t="n"/>
-      <c r="L50" s="16" t="n"/>
-      <c r="M50" s="16" t="n"/>
-      <c r="N50" s="16" t="n"/>
-      <c r="O50" s="16" t="n"/>
-      <c r="P50" s="16" t="n"/>
-      <c r="Q50" s="16" t="n"/>
-      <c r="R50" s="16" t="n"/>
-      <c r="S50" s="16" t="n"/>
-      <c r="T50" s="16" t="n"/>
-      <c r="U50" s="16" t="n"/>
-      <c r="V50" s="16" t="n"/>
-      <c r="W50" s="16" t="n"/>
-      <c r="X50" s="16" t="n"/>
-      <c r="Y50" s="16" t="n"/>
-      <c r="Z50" s="16" t="n"/>
-      <c r="AA50" s="16" t="n"/>
-      <c r="AB50" s="16" t="n"/>
-      <c r="AC50" s="16" t="n"/>
-    </row>
-    <row r="51" ht="20.1" customHeight="1" s="1">
-      <c r="B51" s="18" t="n"/>
-      <c r="C51" s="19" t="inlineStr">
-        <is>
-          <t>Registro de requisitos y plazos del curso</t>
-        </is>
-      </c>
-      <c r="D51" s="19" t="inlineStr">
-        <is>
-          <t>Francisco</t>
-        </is>
-      </c>
-      <c r="E51" s="20" t="n">
-        <v>46304</v>
-      </c>
-      <c r="F51" s="20" t="n">
-        <v>46305</v>
-      </c>
-      <c r="G51" s="19" t="inlineStr">
-        <is>
-          <t>Cumplido</t>
-        </is>
-      </c>
-      <c r="H51" s="21" t="inlineStr">
-        <is>
-          <t>#23, #25</t>
-        </is>
-      </c>
-      <c r="I51" s="22" t="n"/>
-      <c r="J51" s="22" t="n"/>
-      <c r="K51" s="22" t="n"/>
-      <c r="L51" s="22" t="n"/>
-      <c r="M51" s="22" t="n"/>
-      <c r="N51" s="22" t="n"/>
-      <c r="O51" s="22" t="n"/>
-      <c r="P51" s="22" t="n"/>
-      <c r="Q51" s="22" t="n"/>
-      <c r="R51" s="22" t="n"/>
-      <c r="S51" s="22" t="n"/>
-      <c r="T51" s="22" t="n"/>
-      <c r="U51" s="22" t="n"/>
-      <c r="V51" s="22" t="n"/>
-      <c r="W51" s="22" t="n"/>
-      <c r="X51" s="22" t="n"/>
-      <c r="Y51" s="22" t="n"/>
-      <c r="Z51" s="22" t="n"/>
-      <c r="AA51" s="22" t="n"/>
-      <c r="AC51" s="23" t="n"/>
+      <c r="D51" s="16" t="n"/>
+      <c r="E51" s="16" t="n"/>
+      <c r="F51" s="16" t="n"/>
+      <c r="G51" s="16" t="n"/>
+      <c r="H51" s="16" t="n"/>
+      <c r="I51" s="16" t="n"/>
+      <c r="J51" s="16" t="n"/>
+      <c r="K51" s="16" t="n"/>
+      <c r="L51" s="16" t="n"/>
+      <c r="M51" s="16" t="n"/>
+      <c r="N51" s="16" t="n"/>
+      <c r="O51" s="16" t="n"/>
+      <c r="P51" s="16" t="n"/>
+      <c r="Q51" s="16" t="n"/>
+      <c r="R51" s="16" t="n"/>
+      <c r="S51" s="16" t="n"/>
+      <c r="T51" s="16" t="n"/>
+      <c r="U51" s="16" t="n"/>
+      <c r="V51" s="16" t="n"/>
+      <c r="W51" s="16" t="n"/>
+      <c r="X51" s="16" t="n"/>
+      <c r="Y51" s="16" t="n"/>
+      <c r="Z51" s="16" t="n"/>
+      <c r="AA51" s="16" t="n"/>
+      <c r="AB51" s="16" t="n"/>
+      <c r="AC51" s="16" t="n"/>
     </row>
     <row r="52" ht="20.1" customHeight="1" s="1">
       <c r="B52" s="18" t="n"/>
       <c r="C52" s="19" t="inlineStr">
         <is>
-          <t>Casos de uso y diagramas alineados con Walmart</t>
+          <t>Registro de requisitos y plazos del curso</t>
         </is>
       </c>
       <c r="D52" s="19" t="inlineStr">
@@ -2864,7 +2872,7 @@
       </c>
       <c r="H52" s="21" t="inlineStr">
         <is>
-          <t>#30</t>
+          <t>#23, #25</t>
         </is>
       </c>
       <c r="I52" s="22" t="n"/>
@@ -2892,19 +2900,19 @@
       <c r="B53" s="18" t="n"/>
       <c r="C53" s="19" t="inlineStr">
         <is>
-          <t>Plan de mejoras de la Fase 1</t>
+          <t>Casos de uso y diagramas alineados con Walmart</t>
         </is>
       </c>
       <c r="D53" s="19" t="inlineStr">
         <is>
-          <t>Mariana</t>
+          <t>Francisco</t>
         </is>
       </c>
       <c r="E53" s="20" t="n">
-        <v>46315</v>
+        <v>46304</v>
       </c>
       <c r="F53" s="20" t="n">
-        <v>46315</v>
+        <v>46305</v>
       </c>
       <c r="G53" s="19" t="inlineStr">
         <is>
@@ -2913,7 +2921,7 @@
       </c>
       <c r="H53" s="21" t="inlineStr">
         <is>
-          <t>#26</t>
+          <t>#30</t>
         </is>
       </c>
       <c r="I53" s="22" t="n"/>
@@ -2935,38 +2943,34 @@
       <c r="Y53" s="22" t="n"/>
       <c r="Z53" s="22" t="n"/>
       <c r="AA53" s="22" t="n"/>
-      <c r="AC53" s="23" t="inlineStr">
-        <is>
-          <t>Hecho el 2026-10-20, con atraso (plazo 2026-10-09). docs/plan-de-mejoras.md</t>
-        </is>
-      </c>
+      <c r="AC53" s="23" t="n"/>
     </row>
     <row r="54" ht="20.1" customHeight="1" s="1">
       <c r="B54" s="18" t="n"/>
       <c r="C54" s="19" t="inlineStr">
         <is>
-          <t>Informe intermedio: estado de avance y conclusiones</t>
+          <t>Plan de mejoras de la Fase 1</t>
         </is>
       </c>
       <c r="D54" s="19" t="inlineStr">
         <is>
-          <t>Francisco</t>
+          <t>Mariana</t>
         </is>
       </c>
       <c r="E54" s="20" t="n">
-        <v>46314</v>
+        <v>46315</v>
       </c>
       <c r="F54" s="20" t="n">
-        <v>46316</v>
+        <v>46315</v>
       </c>
       <c r="G54" s="19" t="inlineStr">
         <is>
-          <t>En curso</t>
+          <t>Cumplido</t>
         </is>
       </c>
       <c r="H54" s="21" t="inlineStr">
         <is>
-          <t>#27</t>
+          <t>#26</t>
         </is>
       </c>
       <c r="I54" s="22" t="n"/>
@@ -2990,7 +2994,7 @@
       <c r="AA54" s="22" t="n"/>
       <c r="AC54" s="23" t="inlineStr">
         <is>
-          <t>Antes de Nicko; Francisco lo arma en Word</t>
+          <t>Hecho el 2026-10-20, con atraso (plazo 2026-10-09). docs/plan-de-mejoras.md</t>
         </is>
       </c>
     </row>
@@ -2998,7 +3002,7 @@
       <c r="B55" s="18" t="n"/>
       <c r="C55" s="19" t="inlineStr">
         <is>
-          <t>Análisis de resultados: 10 mejores y 10 peores casos</t>
+          <t>Informe intermedio: estado de avance y conclusiones</t>
         </is>
       </c>
       <c r="D55" s="19" t="inlineStr">
@@ -3007,19 +3011,19 @@
         </is>
       </c>
       <c r="E55" s="20" t="n">
-        <v>46315</v>
+        <v>46314</v>
       </c>
       <c r="F55" s="20" t="n">
-        <v>46315</v>
+        <v>46316</v>
       </c>
       <c r="G55" s="19" t="inlineStr">
         <is>
-          <t>Cumplido</t>
+          <t>En curso</t>
         </is>
       </c>
       <c r="H55" s="21" t="inlineStr">
         <is>
-          <t>#34</t>
+          <t>#27</t>
         </is>
       </c>
       <c r="I55" s="22" t="n"/>
@@ -3041,13 +3045,17 @@
       <c r="Y55" s="22" t="n"/>
       <c r="Z55" s="22" t="n"/>
       <c r="AA55" s="22" t="n"/>
-      <c r="AC55" s="23" t="n"/>
+      <c r="AC55" s="23" t="inlineStr">
+        <is>
+          <t>Antes de Nicko; Francisco lo arma en Word</t>
+        </is>
+      </c>
     </row>
     <row r="56" ht="20.1" customHeight="1" s="1">
       <c r="B56" s="18" t="n"/>
       <c r="C56" s="19" t="inlineStr">
         <is>
-          <t>README completo</t>
+          <t>Análisis de resultados: 10 mejores y 10 peores casos</t>
         </is>
       </c>
       <c r="D56" s="19" t="inlineStr">
@@ -3068,7 +3076,7 @@
       </c>
       <c r="H56" s="21" t="inlineStr">
         <is>
-          <t>#35</t>
+          <t>#34</t>
         </is>
       </c>
       <c r="I56" s="22" t="n"/>
@@ -3096,28 +3104,28 @@
       <c r="B57" s="18" t="n"/>
       <c r="C57" s="19" t="inlineStr">
         <is>
-          <t>Video de demostración (5 a 10 min)</t>
+          <t>README completo</t>
         </is>
       </c>
       <c r="D57" s="19" t="inlineStr">
         <is>
-          <t>Nicko</t>
+          <t>Francisco</t>
         </is>
       </c>
       <c r="E57" s="20" t="n">
-        <v>46316</v>
+        <v>46315</v>
       </c>
       <c r="F57" s="20" t="n">
-        <v>46316</v>
+        <v>46315</v>
       </c>
       <c r="G57" s="19" t="inlineStr">
         <is>
-          <t>Pendiente</t>
+          <t>Cumplido</t>
         </is>
       </c>
       <c r="H57" s="21" t="inlineStr">
         <is>
-          <t>#36</t>
+          <t>#35</t>
         </is>
       </c>
       <c r="I57" s="22" t="n"/>
@@ -3145,28 +3153,28 @@
       <c r="B58" s="18" t="n"/>
       <c r="C58" s="19" t="inlineStr">
         <is>
-          <t>Evidencias de avance: diario 2.1 y guía 2.4</t>
+          <t>Video de demostración (5 a 10 min)</t>
         </is>
       </c>
       <c r="D58" s="19" t="inlineStr">
         <is>
-          <t>Mariana</t>
+          <t>Nicko</t>
         </is>
       </c>
       <c r="E58" s="20" t="n">
-        <v>46315</v>
+        <v>46316</v>
       </c>
       <c r="F58" s="20" t="n">
-        <v>46321</v>
+        <v>46316</v>
       </c>
       <c r="G58" s="19" t="inlineStr">
         <is>
-          <t>En curso</t>
+          <t>Pendiente</t>
         </is>
       </c>
       <c r="H58" s="21" t="inlineStr">
         <is>
-          <t>#37</t>
+          <t>#36</t>
         </is>
       </c>
       <c r="I58" s="22" t="n"/>
@@ -3188,17 +3196,13 @@
       <c r="Y58" s="22" t="n"/>
       <c r="Z58" s="22" t="n"/>
       <c r="AA58" s="22" t="n"/>
-      <c r="AC58" s="23" t="inlineStr">
-        <is>
-          <t>Plazo 2026-10-26. Guía 2.4 al 21-10; diario 2.1 y autoevaluación 2.2 de Mariana el 22-10 (Fase 2/). Faltan los diarios de Francisco y Nicko</t>
-        </is>
-      </c>
+      <c r="AC58" s="23" t="n"/>
     </row>
     <row r="59" ht="20.1" customHeight="1" s="1">
       <c r="B59" s="18" t="n"/>
       <c r="C59" s="19" t="inlineStr">
         <is>
-          <t>Rehacer plantillas de C.U y diagramas según la app Django</t>
+          <t>Evidencias de avance: diario 2.1 y guía 2.4</t>
         </is>
       </c>
       <c r="D59" s="19" t="inlineStr">
@@ -3207,19 +3211,19 @@
         </is>
       </c>
       <c r="E59" s="20" t="n">
-        <v>46316</v>
+        <v>46315</v>
       </c>
       <c r="F59" s="20" t="n">
-        <v>46316</v>
+        <v>46321</v>
       </c>
       <c r="G59" s="19" t="inlineStr">
         <is>
-          <t>Cumplido</t>
+          <t>En curso</t>
         </is>
       </c>
       <c r="H59" s="21" t="inlineStr">
         <is>
-          <t>#42</t>
+          <t>#37</t>
         </is>
       </c>
       <c r="I59" s="22" t="n"/>
@@ -3243,121 +3247,121 @@
       <c r="AA59" s="22" t="n"/>
       <c r="AC59" s="23" t="inlineStr">
         <is>
+          <t>Plazo 2026-10-26. Guía 2.4 al 21-10; diario 2.1 y autoevaluación 2.2 de Mariana el 22-10 (Fase 2/). Faltan los diarios de Francisco y Nicko</t>
+        </is>
+      </c>
+    </row>
+    <row r="60" ht="20.1" customHeight="1" s="1">
+      <c r="B60" s="18" t="n"/>
+      <c r="C60" s="19" t="inlineStr">
+        <is>
+          <t>Rehacer plantillas de C.U y diagramas según la app Django</t>
+        </is>
+      </c>
+      <c r="D60" s="19" t="inlineStr">
+        <is>
+          <t>Mariana</t>
+        </is>
+      </c>
+      <c r="E60" s="20" t="n">
+        <v>46316</v>
+      </c>
+      <c r="F60" s="20" t="n">
+        <v>46316</v>
+      </c>
+      <c r="G60" s="19" t="inlineStr">
+        <is>
+          <t>Cumplido</t>
+        </is>
+      </c>
+      <c r="H60" s="21" t="inlineStr">
+        <is>
+          <t>#42</t>
+        </is>
+      </c>
+      <c r="I60" s="22" t="n"/>
+      <c r="J60" s="22" t="n"/>
+      <c r="K60" s="22" t="n"/>
+      <c r="L60" s="22" t="n"/>
+      <c r="M60" s="22" t="n"/>
+      <c r="N60" s="22" t="n"/>
+      <c r="O60" s="22" t="n"/>
+      <c r="P60" s="22" t="n"/>
+      <c r="Q60" s="22" t="n"/>
+      <c r="R60" s="22" t="n"/>
+      <c r="S60" s="22" t="n"/>
+      <c r="T60" s="22" t="n"/>
+      <c r="U60" s="22" t="n"/>
+      <c r="V60" s="22" t="n"/>
+      <c r="W60" s="22" t="n"/>
+      <c r="X60" s="22" t="n"/>
+      <c r="Y60" s="22" t="n"/>
+      <c r="Z60" s="22" t="n"/>
+      <c r="AA60" s="22" t="n"/>
+      <c r="AC60" s="23" t="inlineStr">
+        <is>
           <t>Hecho el 2026-10-21: plantillas, fuentes Mermaid y PNG (CU00-CU06 y arquitectura). docs/cambios-cu.md</t>
         </is>
       </c>
     </row>
-    <row r="60" ht="20.1" customHeight="1" s="1">
-      <c r="B60" s="16" t="n"/>
-      <c r="C60" s="17" t="inlineStr">
+    <row r="61" ht="20.1" customHeight="1" s="1">
+      <c r="B61" s="16" t="n"/>
+      <c r="C61" s="17" t="inlineStr">
         <is>
           <t>HITOS DEL CURSO</t>
         </is>
       </c>
-      <c r="D60" s="16" t="n"/>
-      <c r="E60" s="16" t="n"/>
-      <c r="F60" s="16" t="n"/>
-      <c r="G60" s="16" t="n"/>
-      <c r="H60" s="16" t="n"/>
-      <c r="I60" s="16" t="n"/>
-      <c r="J60" s="16" t="n"/>
-      <c r="K60" s="16" t="n"/>
-      <c r="L60" s="16" t="n"/>
-      <c r="M60" s="16" t="n"/>
-      <c r="N60" s="16" t="n"/>
-      <c r="O60" s="16" t="n"/>
-      <c r="P60" s="16" t="n"/>
-      <c r="Q60" s="16" t="n"/>
-      <c r="R60" s="16" t="n"/>
-      <c r="S60" s="16" t="n"/>
-      <c r="T60" s="16" t="n"/>
-      <c r="U60" s="16" t="n"/>
-      <c r="V60" s="16" t="n"/>
-      <c r="W60" s="16" t="n"/>
-      <c r="X60" s="16" t="n"/>
-      <c r="Y60" s="16" t="n"/>
-      <c r="Z60" s="16" t="n"/>
-      <c r="AA60" s="16" t="n"/>
-      <c r="AB60" s="16" t="n"/>
-      <c r="AC60" s="16" t="n"/>
-    </row>
-    <row r="61" ht="20.1" customHeight="1" s="1">
-      <c r="B61" s="18" t="n"/>
-      <c r="C61" s="19" t="inlineStr">
-        <is>
-          <t>Informe intermedio y video</t>
-        </is>
-      </c>
-      <c r="D61" s="19" t="inlineStr">
-        <is>
-          <t>Equipo</t>
-        </is>
-      </c>
-      <c r="E61" s="20" t="n">
-        <v>46316</v>
-      </c>
-      <c r="F61" s="20" t="n">
-        <v>46316</v>
-      </c>
-      <c r="G61" s="19" t="inlineStr">
-        <is>
-          <t>En curso</t>
-        </is>
-      </c>
-      <c r="H61" s="21" t="n"/>
-      <c r="I61" s="22" t="n"/>
-      <c r="J61" s="22" t="n"/>
-      <c r="K61" s="22" t="n"/>
-      <c r="L61" s="22" t="n"/>
-      <c r="M61" s="22" t="n"/>
-      <c r="N61" s="22" t="n"/>
-      <c r="O61" s="22" t="n"/>
-      <c r="P61" s="22" t="n"/>
-      <c r="Q61" s="22" t="n"/>
-      <c r="R61" s="22" t="n"/>
-      <c r="S61" s="22" t="n"/>
-      <c r="T61" s="22" t="n"/>
-      <c r="U61" s="22" t="n"/>
-      <c r="V61" s="22" t="n"/>
-      <c r="W61" s="22" t="n"/>
-      <c r="X61" s="22" t="n"/>
-      <c r="Y61" s="22" t="n"/>
-      <c r="Z61" s="22" t="n"/>
-      <c r="AA61" s="22" t="n"/>
-      <c r="AC61" s="23" t="inlineStr">
-        <is>
-          <t>Entrega 2026-10-21</t>
-        </is>
-      </c>
+      <c r="D61" s="16" t="n"/>
+      <c r="E61" s="16" t="n"/>
+      <c r="F61" s="16" t="n"/>
+      <c r="G61" s="16" t="n"/>
+      <c r="H61" s="16" t="n"/>
+      <c r="I61" s="16" t="n"/>
+      <c r="J61" s="16" t="n"/>
+      <c r="K61" s="16" t="n"/>
+      <c r="L61" s="16" t="n"/>
+      <c r="M61" s="16" t="n"/>
+      <c r="N61" s="16" t="n"/>
+      <c r="O61" s="16" t="n"/>
+      <c r="P61" s="16" t="n"/>
+      <c r="Q61" s="16" t="n"/>
+      <c r="R61" s="16" t="n"/>
+      <c r="S61" s="16" t="n"/>
+      <c r="T61" s="16" t="n"/>
+      <c r="U61" s="16" t="n"/>
+      <c r="V61" s="16" t="n"/>
+      <c r="W61" s="16" t="n"/>
+      <c r="X61" s="16" t="n"/>
+      <c r="Y61" s="16" t="n"/>
+      <c r="Z61" s="16" t="n"/>
+      <c r="AA61" s="16" t="n"/>
+      <c r="AB61" s="16" t="n"/>
+      <c r="AC61" s="16" t="n"/>
     </row>
     <row r="62" ht="20.1" customHeight="1" s="1">
       <c r="B62" s="18" t="n"/>
       <c r="C62" s="19" t="inlineStr">
         <is>
-          <t>Feria de informática</t>
+          <t>Informe intermedio y video</t>
         </is>
       </c>
       <c r="D62" s="19" t="inlineStr">
         <is>
-          <t>Nicko</t>
+          <t>Equipo</t>
         </is>
       </c>
       <c r="E62" s="20" t="n">
-        <v>46321</v>
+        <v>46316</v>
       </c>
       <c r="F62" s="20" t="n">
-        <v>46325</v>
+        <v>46316</v>
       </c>
       <c r="G62" s="19" t="inlineStr">
         <is>
-          <t>Pendiente</t>
-        </is>
-      </c>
-      <c r="H62" s="21" t="inlineStr">
-        <is>
-          <t>#38</t>
-        </is>
-      </c>
+          <t>En curso</t>
+        </is>
+      </c>
+      <c r="H62" s="21" t="n"/>
       <c r="I62" s="22" t="n"/>
       <c r="J62" s="22" t="n"/>
       <c r="K62" s="22" t="n"/>
@@ -3379,7 +3383,7 @@
       <c r="AA62" s="22" t="n"/>
       <c r="AC62" s="23" t="inlineStr">
         <is>
-          <t>Día y hora por informar</t>
+          <t>Entrega 2026-10-21</t>
         </is>
       </c>
     </row>
@@ -3387,16 +3391,16 @@
       <c r="B63" s="18" t="n"/>
       <c r="C63" s="19" t="inlineStr">
         <is>
-          <t>Evaluación 2 (Avance): 50% de los C.U y demo del Sprint 1</t>
+          <t>Feria de informática</t>
         </is>
       </c>
       <c r="D63" s="19" t="inlineStr">
         <is>
-          <t>Equipo</t>
+          <t>Nicko</t>
         </is>
       </c>
       <c r="E63" s="20" t="n">
-        <v>46323</v>
+        <v>46321</v>
       </c>
       <c r="F63" s="20" t="n">
         <v>46325</v>
@@ -3406,7 +3410,11 @@
           <t>Pendiente</t>
         </is>
       </c>
-      <c r="H63" s="21" t="n"/>
+      <c r="H63" s="21" t="inlineStr">
+        <is>
+          <t>#38</t>
+        </is>
+      </c>
       <c r="I63" s="22" t="n"/>
       <c r="J63" s="22" t="n"/>
       <c r="K63" s="22" t="n"/>
@@ -3428,7 +3436,7 @@
       <c r="AA63" s="22" t="n"/>
       <c r="AC63" s="23" t="inlineStr">
         <is>
-          <t>Día exacto por confirmar</t>
+          <t>Día y hora por informar</t>
         </is>
       </c>
     </row>
@@ -3436,7 +3444,7 @@
       <c r="B64" s="18" t="n"/>
       <c r="C64" s="19" t="inlineStr">
         <is>
-          <t>Entrega final de la Fase 2</t>
+          <t>Evaluación 2 (Avance): 50% de los C.U y demo del Sprint 1</t>
         </is>
       </c>
       <c r="D64" s="19" t="inlineStr">
@@ -3445,10 +3453,10 @@
         </is>
       </c>
       <c r="E64" s="20" t="n">
-        <v>46349</v>
+        <v>46323</v>
       </c>
       <c r="F64" s="20" t="n">
-        <v>46353</v>
+        <v>46325</v>
       </c>
       <c r="G64" s="19" t="inlineStr">
         <is>
@@ -3477,94 +3485,142 @@
       <c r="AA64" s="22" t="n"/>
       <c r="AC64" s="23" t="inlineStr">
         <is>
+          <t>Día exacto por confirmar</t>
+        </is>
+      </c>
+    </row>
+    <row r="65" ht="20.1" customHeight="1" s="1">
+      <c r="B65" s="18" t="n"/>
+      <c r="C65" s="19" t="inlineStr">
+        <is>
+          <t>Entrega final de la Fase 2</t>
+        </is>
+      </c>
+      <c r="D65" s="19" t="inlineStr">
+        <is>
+          <t>Equipo</t>
+        </is>
+      </c>
+      <c r="E65" s="20" t="n">
+        <v>46349</v>
+      </c>
+      <c r="F65" s="20" t="n">
+        <v>46353</v>
+      </c>
+      <c r="G65" s="19" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="H65" s="21" t="n"/>
+      <c r="I65" s="22" t="n"/>
+      <c r="J65" s="22" t="n"/>
+      <c r="K65" s="22" t="n"/>
+      <c r="L65" s="22" t="n"/>
+      <c r="M65" s="22" t="n"/>
+      <c r="N65" s="22" t="n"/>
+      <c r="O65" s="22" t="n"/>
+      <c r="P65" s="22" t="n"/>
+      <c r="Q65" s="22" t="n"/>
+      <c r="R65" s="22" t="n"/>
+      <c r="S65" s="22" t="n"/>
+      <c r="T65" s="22" t="n"/>
+      <c r="U65" s="22" t="n"/>
+      <c r="V65" s="22" t="n"/>
+      <c r="W65" s="22" t="n"/>
+      <c r="X65" s="22" t="n"/>
+      <c r="Y65" s="22" t="n"/>
+      <c r="Z65" s="22" t="n"/>
+      <c r="AA65" s="22" t="n"/>
+      <c r="AC65" s="23" t="inlineStr">
+        <is>
           <t>Semana 15, por confirmar</t>
         </is>
       </c>
     </row>
-    <row r="65" ht="20.1" customHeight="1" s="1">
-      <c r="B65" s="16" t="n"/>
-      <c r="C65" s="17" t="inlineStr">
+    <row r="66" ht="20.1" customHeight="1" s="1">
+      <c r="B66" s="16" t="n"/>
+      <c r="C66" s="17" t="inlineStr">
         <is>
           <t>FASE 3</t>
         </is>
       </c>
-      <c r="D65" s="16" t="n"/>
-      <c r="E65" s="16" t="n"/>
-      <c r="F65" s="16" t="n"/>
-      <c r="G65" s="16" t="n"/>
-      <c r="H65" s="16" t="n"/>
-      <c r="I65" s="16" t="n"/>
-      <c r="J65" s="16" t="n"/>
-      <c r="K65" s="16" t="n"/>
-      <c r="L65" s="16" t="n"/>
-      <c r="M65" s="16" t="n"/>
-      <c r="N65" s="16" t="n"/>
-      <c r="O65" s="16" t="n"/>
-      <c r="P65" s="16" t="n"/>
-      <c r="Q65" s="16" t="n"/>
-      <c r="R65" s="16" t="n"/>
-      <c r="S65" s="16" t="n"/>
-      <c r="T65" s="16" t="n"/>
-      <c r="U65" s="16" t="n"/>
-      <c r="V65" s="16" t="n"/>
-      <c r="W65" s="16" t="n"/>
-      <c r="X65" s="16" t="n"/>
-      <c r="Y65" s="16" t="n"/>
-      <c r="Z65" s="16" t="n"/>
-      <c r="AA65" s="16" t="n"/>
-      <c r="AB65" s="16" t="n"/>
-      <c r="AC65" s="16" t="n"/>
-    </row>
-    <row r="66" ht="20.1" customHeight="1" s="1">
-      <c r="B66" s="18" t="n"/>
-      <c r="C66" s="19" t="inlineStr">
+      <c r="D66" s="16" t="n"/>
+      <c r="E66" s="16" t="n"/>
+      <c r="F66" s="16" t="n"/>
+      <c r="G66" s="16" t="n"/>
+      <c r="H66" s="16" t="n"/>
+      <c r="I66" s="16" t="n"/>
+      <c r="J66" s="16" t="n"/>
+      <c r="K66" s="16" t="n"/>
+      <c r="L66" s="16" t="n"/>
+      <c r="M66" s="16" t="n"/>
+      <c r="N66" s="16" t="n"/>
+      <c r="O66" s="16" t="n"/>
+      <c r="P66" s="16" t="n"/>
+      <c r="Q66" s="16" t="n"/>
+      <c r="R66" s="16" t="n"/>
+      <c r="S66" s="16" t="n"/>
+      <c r="T66" s="16" t="n"/>
+      <c r="U66" s="16" t="n"/>
+      <c r="V66" s="16" t="n"/>
+      <c r="W66" s="16" t="n"/>
+      <c r="X66" s="16" t="n"/>
+      <c r="Y66" s="16" t="n"/>
+      <c r="Z66" s="16" t="n"/>
+      <c r="AA66" s="16" t="n"/>
+      <c r="AB66" s="16" t="n"/>
+      <c r="AC66" s="16" t="n"/>
+    </row>
+    <row r="67" ht="20.1" customHeight="1" s="1">
+      <c r="B67" s="18" t="n"/>
+      <c r="C67" s="19" t="inlineStr">
         <is>
           <t>Ajustes finales, manuales y exposición ante la Comisión</t>
         </is>
       </c>
-      <c r="D66" s="19" t="inlineStr">
+      <c r="D67" s="19" t="inlineStr">
         <is>
           <t>Equipo</t>
         </is>
       </c>
-      <c r="E66" s="20" t="n">
+      <c r="E67" s="20" t="n">
         <v>46356</v>
       </c>
-      <c r="F66" s="20" t="n">
+      <c r="F67" s="20" t="n">
         <v>46374</v>
       </c>
-      <c r="G66" s="19" t="inlineStr">
+      <c r="G67" s="19" t="inlineStr">
         <is>
           <t>Pendiente</t>
         </is>
       </c>
-      <c r="H66" s="21" t="n"/>
-      <c r="I66" s="22" t="n"/>
-      <c r="J66" s="22" t="n"/>
-      <c r="K66" s="22" t="n"/>
-      <c r="L66" s="22" t="n"/>
-      <c r="M66" s="22" t="n"/>
-      <c r="N66" s="22" t="n"/>
-      <c r="O66" s="22" t="n"/>
-      <c r="P66" s="22" t="n"/>
-      <c r="Q66" s="22" t="n"/>
-      <c r="R66" s="22" t="n"/>
-      <c r="S66" s="22" t="n"/>
-      <c r="T66" s="22" t="n"/>
-      <c r="U66" s="22" t="n"/>
-      <c r="V66" s="22" t="n"/>
-      <c r="W66" s="22" t="n"/>
-      <c r="X66" s="22" t="n"/>
-      <c r="Y66" s="22" t="n"/>
-      <c r="Z66" s="22" t="n"/>
-      <c r="AA66" s="22" t="n"/>
-      <c r="AC66" s="23" t="inlineStr">
+      <c r="H67" s="21" t="n"/>
+      <c r="I67" s="22" t="n"/>
+      <c r="J67" s="22" t="n"/>
+      <c r="K67" s="22" t="n"/>
+      <c r="L67" s="22" t="n"/>
+      <c r="M67" s="22" t="n"/>
+      <c r="N67" s="22" t="n"/>
+      <c r="O67" s="22" t="n"/>
+      <c r="P67" s="22" t="n"/>
+      <c r="Q67" s="22" t="n"/>
+      <c r="R67" s="22" t="n"/>
+      <c r="S67" s="22" t="n"/>
+      <c r="T67" s="22" t="n"/>
+      <c r="U67" s="22" t="n"/>
+      <c r="V67" s="22" t="n"/>
+      <c r="W67" s="22" t="n"/>
+      <c r="X67" s="22" t="n"/>
+      <c r="Y67" s="22" t="n"/>
+      <c r="Z67" s="22" t="n"/>
+      <c r="AA67" s="22" t="n"/>
+      <c r="AC67" s="23" t="inlineStr">
         <is>
           <t>Fechas por definir</t>
         </is>
       </c>
     </row>
-    <row r="67" ht="15.75" customHeight="1" s="1"/>
     <row r="68" ht="15.75" customHeight="1" s="1"/>
     <row r="69" ht="15.75" customHeight="1" s="1"/>
     <row r="70" ht="15.75" customHeight="1" s="1"/>
@@ -4499,6 +4555,7 @@
     <row r="999" ht="15.75" customHeight="1" s="1"/>
     <row r="1000" ht="15.75" customHeight="1" s="1"/>
     <row r="1001" ht="15.75" customHeight="1" s="1"/>
+    <row r="1002" ht="15.75" customHeight="1" s="1"/>
   </sheetData>
   <mergeCells count="5">
     <mergeCell ref="U8:Y8"/>
@@ -4507,7 +4564,7 @@
     <mergeCell ref="Q8:T8"/>
     <mergeCell ref="I8:L8"/>
   </mergeCells>
-  <conditionalFormatting sqref="B10:B66">
+  <conditionalFormatting sqref="B10:B67">
     <cfRule type="expression" priority="2" dxfId="5" stopIfTrue="1">
       <formula>$G10="Cumplido"</formula>
     </cfRule>
@@ -4524,7 +4581,7 @@
       <formula>$G10="Bloqueado"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="I10:AA66">
+  <conditionalFormatting sqref="I10:AA67">
     <cfRule type="expression" priority="1" dxfId="5" stopIfTrue="1">
       <formula>AND($E10&lt;&gt;"",I$9&lt;=$F10,I$9+6&gt;=$E10,$G10="Cumplido")</formula>
     </cfRule>
@@ -4541,7 +4598,7 @@
       <formula>AND($E10&lt;&gt;"",I$9&lt;=$F10,I$9+6&gt;=$E10,$G10="Bloqueado")</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="S10:S66">
+  <conditionalFormatting sqref="S10:S67">
     <cfRule type="expression" priority="11" dxfId="0">
       <formula>$G10&lt;&gt;""</formula>
     </cfRule>

</xml_diff>

<commit_message>
docs: document photos without products and mark #52 done
</commit_message>
<xml_diff>
--- a/Anexos/Gestion/Carta Gantt Fase 2.xlsx
+++ b/Anexos/Gestion/Carta Gantt Fase 2.xlsx
@@ -2576,7 +2576,7 @@
       </c>
       <c r="G46" s="19" t="inlineStr">
         <is>
-          <t>Pendiente</t>
+          <t>En curso</t>
         </is>
       </c>
       <c r="H46" s="21" t="inlineStr">
@@ -2605,7 +2605,7 @@
       <c r="AA46" s="22" t="n"/>
       <c r="AC46" s="23" t="inlineStr">
         <is>
-          <t>Francisco: #49 a #51; Mariana: #52 y #53</t>
+          <t>Francisco: #49 a #51; Mariana: #52 (hecho el 22-10) y #53</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
docs: document CU05 and mark #44 done
</commit_message>
<xml_diff>
--- a/Anexos/Gestion/Carta Gantt Fase 2.xlsx
+++ b/Anexos/Gestion/Carta Gantt Fase 2.xlsx
@@ -2622,14 +2622,14 @@
         </is>
       </c>
       <c r="E47" s="20">
-        <v>46323</v>
+        <v>46317</v>
       </c>
       <c r="F47" s="20">
         <v>46325</v>
       </c>
       <c r="G47" s="19" t="inlineStr">
         <is>
-          <t>Pendiente</t>
+          <t>En curso</t>
         </is>
       </c>
       <c r="H47" s="21" t="inlineStr">
@@ -2658,7 +2658,7 @@
       <c r="AA47" s="22" t="n"/>
       <c r="AC47" s="23" t="inlineStr">
         <is>
-          <t>Fechas propuestas, a confirmar</t>
+          <t>#44 (CU05) hecho el 22-10; falta #43 (CU03). Fin propuesto, a confirmar</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
docs: document CU03 and mark #43 done
</commit_message>
<xml_diff>
--- a/Anexos/Gestion/Carta Gantt Fase 2.xlsx
+++ b/Anexos/Gestion/Carta Gantt Fase 2.xlsx
@@ -2625,11 +2625,11 @@
         <v>46317</v>
       </c>
       <c r="F47" s="20">
-        <v>46325</v>
+        <v>46317</v>
       </c>
       <c r="G47" s="19" t="inlineStr">
         <is>
-          <t>En curso</t>
+          <t>Cumplido</t>
         </is>
       </c>
       <c r="H47" s="21" t="inlineStr">
@@ -2658,7 +2658,7 @@
       <c r="AA47" s="22" t="n"/>
       <c r="AC47" s="23" t="inlineStr">
         <is>
-          <t>#44 (CU05) hecho el 22-10; falta #43 (CU03). Fin propuesto, a confirmar</t>
+          <t>#44 (CU05) y #43 (CU03) hechos el 22-10</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
chore: stop Claude Code from adding itself as co-author (#56)
</commit_message>
<xml_diff>
--- a/Anexos/Gestion/Carta Gantt Fase 2.xlsx
+++ b/Anexos/Gestion/Carta Gantt Fase 2.xlsx
@@ -10,7 +10,7 @@
   </sheets>
   <definedNames>
     <definedName name="_xlnm.Print_Titles" localSheetId="0">'Carta Gantt'!$8:$9</definedName>
-    <definedName name="_xlnm.Print_Area" localSheetId="0">'Carta Gantt'!$B$1:$AC$67</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="0">'Carta Gantt'!$B$1:$AC$68</definedName>
   </definedNames>
   <calcPr calcId="191029" fullCalcOnLoad="1"/>
 </workbook>
@@ -655,7 +655,7 @@
     <outlinePr summaryBelow="0" summaryRight="0"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:AC67"/>
+  <dimension ref="A1:AC68"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="12.5703125" defaultRowHeight="15" customHeight="1"/>
   <cols>
     <col width="2" customWidth="1" style="1" min="1" max="1"/>
@@ -695,23 +695,23 @@
     <row r="4" ht="15.75" customHeight="1" s="1"/>
     <row r="5" ht="26.1" customHeight="1" s="1">
       <c r="D5" s="5">
-        <f>COUNTIF($G$10:$G$67,"Cumplido")</f>
+        <f>COUNTIF($G$10:$G$68,"Cumplido")</f>
         <v/>
       </c>
       <c r="E5" s="6">
-        <f>COUNTIF($G$10:$G$67,"En curso")</f>
+        <f>COUNTIF($G$10:$G$68,"En curso")</f>
         <v/>
       </c>
       <c r="F5" s="7">
-        <f>COUNTIF($G$10:$G$67,"Pendiente")</f>
+        <f>COUNTIF($G$10:$G$68,"Pendiente")</f>
         <v/>
       </c>
       <c r="G5" s="8">
-        <f>COUNTIF($G$10:$G$67,"Atrasado")</f>
+        <f>COUNTIF($G$10:$G$68,"Atrasado")</f>
         <v/>
       </c>
       <c r="H5" s="9">
-        <f>COUNTIF($G$10:$G$67,"Bloqueado")</f>
+        <f>COUNTIF($G$10:$G$68,"Bloqueado")</f>
         <v/>
       </c>
     </row>
@@ -3305,116 +3305,116 @@
       </c>
     </row>
     <row r="61" ht="20.1" customHeight="1" s="1">
-      <c r="B61" s="16" t="n"/>
-      <c r="C61" s="17" t="inlineStr">
+      <c r="B61" s="18" t="n"/>
+      <c r="C61" s="19" t="inlineStr">
+        <is>
+          <t>Sin coautoría de Claude Code en commits y PR</t>
+        </is>
+      </c>
+      <c r="D61" s="19" t="inlineStr">
+        <is>
+          <t>Mariana</t>
+        </is>
+      </c>
+      <c r="E61" s="20">
+        <v>46317</v>
+      </c>
+      <c r="F61" s="20">
+        <v>46317</v>
+      </c>
+      <c r="G61" s="19" t="inlineStr">
+        <is>
+          <t>Cumplido</t>
+        </is>
+      </c>
+      <c r="H61" s="21" t="inlineStr">
+        <is>
+          <t>#56</t>
+        </is>
+      </c>
+      <c r="I61" s="22" t="n"/>
+      <c r="J61" s="22" t="n"/>
+      <c r="K61" s="22" t="n"/>
+      <c r="L61" s="22" t="n"/>
+      <c r="M61" s="22" t="n"/>
+      <c r="N61" s="22" t="n"/>
+      <c r="O61" s="22" t="n"/>
+      <c r="P61" s="22" t="n"/>
+      <c r="Q61" s="22" t="n"/>
+      <c r="R61" s="22" t="n"/>
+      <c r="S61" s="22" t="n"/>
+      <c r="T61" s="22" t="n"/>
+      <c r="U61" s="22" t="n"/>
+      <c r="V61" s="22" t="n"/>
+      <c r="W61" s="22" t="n"/>
+      <c r="X61" s="22" t="n"/>
+      <c r="Y61" s="22" t="n"/>
+      <c r="Z61" s="22" t="n"/>
+      <c r="AA61" s="22" t="n"/>
+      <c r="AC61" s="23" t="inlineStr">
+        <is>
+          <t>attribution vacío en .claude/settings.json; los commits ya publicados no cambian</t>
+        </is>
+      </c>
+    </row>
+    <row r="62" ht="20.1" customHeight="1" s="1">
+      <c r="B62" s="16" t="n"/>
+      <c r="C62" s="17" t="inlineStr">
         <is>
           <t>HITOS DEL CURSO</t>
         </is>
       </c>
-      <c r="D61" s="16" t="n"/>
-      <c r="E61" s="16" t="n"/>
-      <c r="F61" s="16" t="n"/>
-      <c r="G61" s="16" t="n"/>
-      <c r="H61" s="16" t="n"/>
-      <c r="I61" s="16" t="n"/>
-      <c r="J61" s="16" t="n"/>
-      <c r="K61" s="16" t="n"/>
-      <c r="L61" s="16" t="n"/>
-      <c r="M61" s="16" t="n"/>
-      <c r="N61" s="16" t="n"/>
-      <c r="O61" s="16" t="n"/>
-      <c r="P61" s="16" t="n"/>
-      <c r="Q61" s="16" t="n"/>
-      <c r="R61" s="16" t="n"/>
-      <c r="S61" s="16" t="n"/>
-      <c r="T61" s="16" t="n"/>
-      <c r="U61" s="16" t="n"/>
-      <c r="V61" s="16" t="n"/>
-      <c r="W61" s="16" t="n"/>
-      <c r="X61" s="16" t="n"/>
-      <c r="Y61" s="16" t="n"/>
-      <c r="Z61" s="16" t="n"/>
-      <c r="AA61" s="16" t="n"/>
-      <c r="AB61" s="16" t="n"/>
-      <c r="AC61" s="16" t="n"/>
-    </row>
-    <row r="62" ht="20.1" customHeight="1" s="1">
-      <c r="B62" s="18" t="n"/>
-      <c r="C62" s="19" t="inlineStr">
-        <is>
-          <t>Informe intermedio y video</t>
-        </is>
-      </c>
-      <c r="D62" s="19" t="inlineStr">
-        <is>
-          <t>Equipo</t>
-        </is>
-      </c>
-      <c r="E62" s="20" t="n">
-        <v>46316</v>
-      </c>
-      <c r="F62" s="20" t="n">
-        <v>46316</v>
-      </c>
-      <c r="G62" s="19" t="inlineStr">
-        <is>
-          <t>En curso</t>
-        </is>
-      </c>
-      <c r="H62" s="21" t="n"/>
-      <c r="I62" s="22" t="n"/>
-      <c r="J62" s="22" t="n"/>
-      <c r="K62" s="22" t="n"/>
-      <c r="L62" s="22" t="n"/>
-      <c r="M62" s="22" t="n"/>
-      <c r="N62" s="22" t="n"/>
-      <c r="O62" s="22" t="n"/>
-      <c r="P62" s="22" t="n"/>
-      <c r="Q62" s="22" t="n"/>
-      <c r="R62" s="22" t="n"/>
-      <c r="S62" s="22" t="n"/>
-      <c r="T62" s="22" t="n"/>
-      <c r="U62" s="22" t="n"/>
-      <c r="V62" s="22" t="n"/>
-      <c r="W62" s="22" t="n"/>
-      <c r="X62" s="22" t="n"/>
-      <c r="Y62" s="22" t="n"/>
-      <c r="Z62" s="22" t="n"/>
-      <c r="AA62" s="22" t="n"/>
-      <c r="AC62" s="23" t="inlineStr">
-        <is>
-          <t>Entrega 2026-10-21</t>
-        </is>
-      </c>
+      <c r="D62" s="16" t="n"/>
+      <c r="E62" s="16" t="n"/>
+      <c r="F62" s="16" t="n"/>
+      <c r="G62" s="16" t="n"/>
+      <c r="H62" s="16" t="n"/>
+      <c r="I62" s="16" t="n"/>
+      <c r="J62" s="16" t="n"/>
+      <c r="K62" s="16" t="n"/>
+      <c r="L62" s="16" t="n"/>
+      <c r="M62" s="16" t="n"/>
+      <c r="N62" s="16" t="n"/>
+      <c r="O62" s="16" t="n"/>
+      <c r="P62" s="16" t="n"/>
+      <c r="Q62" s="16" t="n"/>
+      <c r="R62" s="16" t="n"/>
+      <c r="S62" s="16" t="n"/>
+      <c r="T62" s="16" t="n"/>
+      <c r="U62" s="16" t="n"/>
+      <c r="V62" s="16" t="n"/>
+      <c r="W62" s="16" t="n"/>
+      <c r="X62" s="16" t="n"/>
+      <c r="Y62" s="16" t="n"/>
+      <c r="Z62" s="16" t="n"/>
+      <c r="AA62" s="16" t="n"/>
+      <c r="AB62" s="16" t="n"/>
+      <c r="AC62" s="16" t="n"/>
     </row>
     <row r="63" ht="20.1" customHeight="1" s="1">
       <c r="B63" s="18" t="n"/>
       <c r="C63" s="19" t="inlineStr">
         <is>
-          <t>Feria de informática</t>
+          <t>Informe intermedio y video</t>
         </is>
       </c>
       <c r="D63" s="19" t="inlineStr">
         <is>
-          <t>Nicko</t>
+          <t>Equipo</t>
         </is>
       </c>
       <c r="E63" s="20" t="n">
-        <v>46321</v>
+        <v>46316</v>
       </c>
       <c r="F63" s="20" t="n">
-        <v>46325</v>
+        <v>46316</v>
       </c>
       <c r="G63" s="19" t="inlineStr">
         <is>
-          <t>Pendiente</t>
-        </is>
-      </c>
-      <c r="H63" s="21" t="inlineStr">
-        <is>
-          <t>#38</t>
-        </is>
-      </c>
+          <t>En curso</t>
+        </is>
+      </c>
+      <c r="H63" s="21" t="n"/>
       <c r="I63" s="22" t="n"/>
       <c r="J63" s="22" t="n"/>
       <c r="K63" s="22" t="n"/>
@@ -3436,7 +3436,7 @@
       <c r="AA63" s="22" t="n"/>
       <c r="AC63" s="23" t="inlineStr">
         <is>
-          <t>Día y hora por informar</t>
+          <t>Entrega 2026-10-21</t>
         </is>
       </c>
     </row>
@@ -3444,16 +3444,16 @@
       <c r="B64" s="18" t="n"/>
       <c r="C64" s="19" t="inlineStr">
         <is>
-          <t>Evaluación 2 (Avance): 50% de los C.U y demo del Sprint 1</t>
+          <t>Feria de informática</t>
         </is>
       </c>
       <c r="D64" s="19" t="inlineStr">
         <is>
-          <t>Equipo</t>
+          <t>Nicko</t>
         </is>
       </c>
       <c r="E64" s="20" t="n">
-        <v>46323</v>
+        <v>46321</v>
       </c>
       <c r="F64" s="20" t="n">
         <v>46325</v>
@@ -3463,7 +3463,11 @@
           <t>Pendiente</t>
         </is>
       </c>
-      <c r="H64" s="21" t="n"/>
+      <c r="H64" s="21" t="inlineStr">
+        <is>
+          <t>#38</t>
+        </is>
+      </c>
       <c r="I64" s="22" t="n"/>
       <c r="J64" s="22" t="n"/>
       <c r="K64" s="22" t="n"/>
@@ -3485,7 +3489,7 @@
       <c r="AA64" s="22" t="n"/>
       <c r="AC64" s="23" t="inlineStr">
         <is>
-          <t>Día exacto por confirmar</t>
+          <t>Día y hora por informar</t>
         </is>
       </c>
     </row>
@@ -3493,7 +3497,7 @@
       <c r="B65" s="18" t="n"/>
       <c r="C65" s="19" t="inlineStr">
         <is>
-          <t>Entrega final de la Fase 2</t>
+          <t>Evaluación 2 (Avance): 50% de los C.U y demo del Sprint 1</t>
         </is>
       </c>
       <c r="D65" s="19" t="inlineStr">
@@ -3502,10 +3506,10 @@
         </is>
       </c>
       <c r="E65" s="20" t="n">
-        <v>46349</v>
+        <v>46323</v>
       </c>
       <c r="F65" s="20" t="n">
-        <v>46353</v>
+        <v>46325</v>
       </c>
       <c r="G65" s="19" t="inlineStr">
         <is>
@@ -3534,94 +3538,142 @@
       <c r="AA65" s="22" t="n"/>
       <c r="AC65" s="23" t="inlineStr">
         <is>
+          <t>Día exacto por confirmar</t>
+        </is>
+      </c>
+    </row>
+    <row r="66" ht="20.1" customHeight="1" s="1">
+      <c r="B66" s="18" t="n"/>
+      <c r="C66" s="19" t="inlineStr">
+        <is>
+          <t>Entrega final de la Fase 2</t>
+        </is>
+      </c>
+      <c r="D66" s="19" t="inlineStr">
+        <is>
+          <t>Equipo</t>
+        </is>
+      </c>
+      <c r="E66" s="20" t="n">
+        <v>46349</v>
+      </c>
+      <c r="F66" s="20" t="n">
+        <v>46353</v>
+      </c>
+      <c r="G66" s="19" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="H66" s="21" t="n"/>
+      <c r="I66" s="22" t="n"/>
+      <c r="J66" s="22" t="n"/>
+      <c r="K66" s="22" t="n"/>
+      <c r="L66" s="22" t="n"/>
+      <c r="M66" s="22" t="n"/>
+      <c r="N66" s="22" t="n"/>
+      <c r="O66" s="22" t="n"/>
+      <c r="P66" s="22" t="n"/>
+      <c r="Q66" s="22" t="n"/>
+      <c r="R66" s="22" t="n"/>
+      <c r="S66" s="22" t="n"/>
+      <c r="T66" s="22" t="n"/>
+      <c r="U66" s="22" t="n"/>
+      <c r="V66" s="22" t="n"/>
+      <c r="W66" s="22" t="n"/>
+      <c r="X66" s="22" t="n"/>
+      <c r="Y66" s="22" t="n"/>
+      <c r="Z66" s="22" t="n"/>
+      <c r="AA66" s="22" t="n"/>
+      <c r="AC66" s="23" t="inlineStr">
+        <is>
           <t>Semana 15, por confirmar</t>
         </is>
       </c>
     </row>
-    <row r="66" ht="20.1" customHeight="1" s="1">
-      <c r="B66" s="16" t="n"/>
-      <c r="C66" s="17" t="inlineStr">
+    <row r="67" ht="20.1" customHeight="1" s="1">
+      <c r="B67" s="16" t="n"/>
+      <c r="C67" s="17" t="inlineStr">
         <is>
           <t>FASE 3</t>
         </is>
       </c>
-      <c r="D66" s="16" t="n"/>
-      <c r="E66" s="16" t="n"/>
-      <c r="F66" s="16" t="n"/>
-      <c r="G66" s="16" t="n"/>
-      <c r="H66" s="16" t="n"/>
-      <c r="I66" s="16" t="n"/>
-      <c r="J66" s="16" t="n"/>
-      <c r="K66" s="16" t="n"/>
-      <c r="L66" s="16" t="n"/>
-      <c r="M66" s="16" t="n"/>
-      <c r="N66" s="16" t="n"/>
-      <c r="O66" s="16" t="n"/>
-      <c r="P66" s="16" t="n"/>
-      <c r="Q66" s="16" t="n"/>
-      <c r="R66" s="16" t="n"/>
-      <c r="S66" s="16" t="n"/>
-      <c r="T66" s="16" t="n"/>
-      <c r="U66" s="16" t="n"/>
-      <c r="V66" s="16" t="n"/>
-      <c r="W66" s="16" t="n"/>
-      <c r="X66" s="16" t="n"/>
-      <c r="Y66" s="16" t="n"/>
-      <c r="Z66" s="16" t="n"/>
-      <c r="AA66" s="16" t="n"/>
-      <c r="AB66" s="16" t="n"/>
-      <c r="AC66" s="16" t="n"/>
-    </row>
-    <row r="67" ht="20.1" customHeight="1" s="1">
-      <c r="B67" s="18" t="n"/>
-      <c r="C67" s="19" t="inlineStr">
+      <c r="D67" s="16" t="n"/>
+      <c r="E67" s="16" t="n"/>
+      <c r="F67" s="16" t="n"/>
+      <c r="G67" s="16" t="n"/>
+      <c r="H67" s="16" t="n"/>
+      <c r="I67" s="16" t="n"/>
+      <c r="J67" s="16" t="n"/>
+      <c r="K67" s="16" t="n"/>
+      <c r="L67" s="16" t="n"/>
+      <c r="M67" s="16" t="n"/>
+      <c r="N67" s="16" t="n"/>
+      <c r="O67" s="16" t="n"/>
+      <c r="P67" s="16" t="n"/>
+      <c r="Q67" s="16" t="n"/>
+      <c r="R67" s="16" t="n"/>
+      <c r="S67" s="16" t="n"/>
+      <c r="T67" s="16" t="n"/>
+      <c r="U67" s="16" t="n"/>
+      <c r="V67" s="16" t="n"/>
+      <c r="W67" s="16" t="n"/>
+      <c r="X67" s="16" t="n"/>
+      <c r="Y67" s="16" t="n"/>
+      <c r="Z67" s="16" t="n"/>
+      <c r="AA67" s="16" t="n"/>
+      <c r="AB67" s="16" t="n"/>
+      <c r="AC67" s="16" t="n"/>
+    </row>
+    <row r="68" ht="20.1" customHeight="1" s="1">
+      <c r="B68" s="18" t="n"/>
+      <c r="C68" s="19" t="inlineStr">
         <is>
           <t>Ajustes finales, manuales y exposición ante la Comisión</t>
         </is>
       </c>
-      <c r="D67" s="19" t="inlineStr">
+      <c r="D68" s="19" t="inlineStr">
         <is>
           <t>Equipo</t>
         </is>
       </c>
-      <c r="E67" s="20" t="n">
+      <c r="E68" s="20" t="n">
         <v>46356</v>
       </c>
-      <c r="F67" s="20" t="n">
+      <c r="F68" s="20" t="n">
         <v>46374</v>
       </c>
-      <c r="G67" s="19" t="inlineStr">
+      <c r="G68" s="19" t="inlineStr">
         <is>
           <t>Pendiente</t>
         </is>
       </c>
-      <c r="H67" s="21" t="n"/>
-      <c r="I67" s="22" t="n"/>
-      <c r="J67" s="22" t="n"/>
-      <c r="K67" s="22" t="n"/>
-      <c r="L67" s="22" t="n"/>
-      <c r="M67" s="22" t="n"/>
-      <c r="N67" s="22" t="n"/>
-      <c r="O67" s="22" t="n"/>
-      <c r="P67" s="22" t="n"/>
-      <c r="Q67" s="22" t="n"/>
-      <c r="R67" s="22" t="n"/>
-      <c r="S67" s="22" t="n"/>
-      <c r="T67" s="22" t="n"/>
-      <c r="U67" s="22" t="n"/>
-      <c r="V67" s="22" t="n"/>
-      <c r="W67" s="22" t="n"/>
-      <c r="X67" s="22" t="n"/>
-      <c r="Y67" s="22" t="n"/>
-      <c r="Z67" s="22" t="n"/>
-      <c r="AA67" s="22" t="n"/>
-      <c r="AC67" s="23" t="inlineStr">
+      <c r="H68" s="21" t="n"/>
+      <c r="I68" s="22" t="n"/>
+      <c r="J68" s="22" t="n"/>
+      <c r="K68" s="22" t="n"/>
+      <c r="L68" s="22" t="n"/>
+      <c r="M68" s="22" t="n"/>
+      <c r="N68" s="22" t="n"/>
+      <c r="O68" s="22" t="n"/>
+      <c r="P68" s="22" t="n"/>
+      <c r="Q68" s="22" t="n"/>
+      <c r="R68" s="22" t="n"/>
+      <c r="S68" s="22" t="n"/>
+      <c r="T68" s="22" t="n"/>
+      <c r="U68" s="22" t="n"/>
+      <c r="V68" s="22" t="n"/>
+      <c r="W68" s="22" t="n"/>
+      <c r="X68" s="22" t="n"/>
+      <c r="Y68" s="22" t="n"/>
+      <c r="Z68" s="22" t="n"/>
+      <c r="AA68" s="22" t="n"/>
+      <c r="AC68" s="23" t="inlineStr">
         <is>
           <t>Fechas por definir</t>
         </is>
       </c>
     </row>
-    <row r="68" ht="15.75" customHeight="1" s="1"/>
     <row r="69" ht="15.75" customHeight="1" s="1"/>
     <row r="70" ht="15.75" customHeight="1" s="1"/>
     <row r="71" ht="15.75" customHeight="1" s="1"/>
@@ -4556,6 +4608,7 @@
     <row r="1000" ht="15.75" customHeight="1" s="1"/>
     <row r="1001" ht="15.75" customHeight="1" s="1"/>
     <row r="1002" ht="15.75" customHeight="1" s="1"/>
+    <row r="1003" ht="15.75" customHeight="1" s="1"/>
   </sheetData>
   <mergeCells count="5">
     <mergeCell ref="U8:Y8"/>
@@ -4564,7 +4617,7 @@
     <mergeCell ref="Q8:T8"/>
     <mergeCell ref="I8:L8"/>
   </mergeCells>
-  <conditionalFormatting sqref="B10:B67">
+  <conditionalFormatting sqref="B10:B68">
     <cfRule type="expression" priority="2" dxfId="5" stopIfTrue="1">
       <formula>$G10="Cumplido"</formula>
     </cfRule>
@@ -4581,7 +4634,7 @@
       <formula>$G10="Bloqueado"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="I10:AA67">
+  <conditionalFormatting sqref="I10:AA68">
     <cfRule type="expression" priority="1" dxfId="5" stopIfTrue="1">
       <formula>AND($E10&lt;&gt;"",I$9&lt;=$F10,I$9+6&gt;=$E10,$G10="Cumplido")</formula>
     </cfRule>
@@ -4598,7 +4651,7 @@
       <formula>AND($E10&lt;&gt;"",I$9&lt;=$F10,I$9+6&gt;=$E10,$G10="Bloqueado")</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="S10:S67">
+  <conditionalFormatting sqref="S10:S68">
     <cfRule type="expression" priority="11" dxfId="0">
       <formula>$G10&lt;&gt;""</formula>
     </cfRule>

</xml_diff>

<commit_message>
chore: keep #56 out of the Gantt chart
</commit_message>
<xml_diff>
--- a/Anexos/Gestion/Carta Gantt Fase 2.xlsx
+++ b/Anexos/Gestion/Carta Gantt Fase 2.xlsx
@@ -10,7 +10,7 @@
   </sheets>
   <definedNames>
     <definedName name="_xlnm.Print_Titles" localSheetId="0">'Carta Gantt'!$8:$9</definedName>
-    <definedName name="_xlnm.Print_Area" localSheetId="0">'Carta Gantt'!$B$1:$AC$68</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="0">'Carta Gantt'!$B$1:$AC$67</definedName>
   </definedNames>
   <calcPr calcId="191029" fullCalcOnLoad="1"/>
 </workbook>
@@ -655,7 +655,7 @@
     <outlinePr summaryBelow="0" summaryRight="0"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:AC68"/>
+  <dimension ref="A1:AC67"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="12.5703125" defaultRowHeight="15" customHeight="1"/>
   <cols>
     <col width="2" customWidth="1" style="1" min="1" max="1"/>
@@ -695,23 +695,23 @@
     <row r="4" ht="15.75" customHeight="1" s="1"/>
     <row r="5" ht="26.1" customHeight="1" s="1">
       <c r="D5" s="5">
-        <f>COUNTIF($G$10:$G$68,"Cumplido")</f>
+        <f>COUNTIF($G$10:$G$67,"Cumplido")</f>
         <v/>
       </c>
       <c r="E5" s="6">
-        <f>COUNTIF($G$10:$G$68,"En curso")</f>
+        <f>COUNTIF($G$10:$G$67,"En curso")</f>
         <v/>
       </c>
       <c r="F5" s="7">
-        <f>COUNTIF($G$10:$G$68,"Pendiente")</f>
+        <f>COUNTIF($G$10:$G$67,"Pendiente")</f>
         <v/>
       </c>
       <c r="G5" s="8">
-        <f>COUNTIF($G$10:$G$68,"Atrasado")</f>
+        <f>COUNTIF($G$10:$G$67,"Atrasado")</f>
         <v/>
       </c>
       <c r="H5" s="9">
-        <f>COUNTIF($G$10:$G$68,"Bloqueado")</f>
+        <f>COUNTIF($G$10:$G$67,"Bloqueado")</f>
         <v/>
       </c>
     </row>
@@ -3305,116 +3305,116 @@
       </c>
     </row>
     <row r="61" ht="20.1" customHeight="1" s="1">
-      <c r="B61" s="18" t="n"/>
-      <c r="C61" s="19" t="inlineStr">
-        <is>
-          <t>Sin coautoría de Claude Code en commits y PR</t>
-        </is>
-      </c>
-      <c r="D61" s="19" t="inlineStr">
-        <is>
-          <t>Mariana</t>
-        </is>
-      </c>
-      <c r="E61" s="20">
-        <v>46317</v>
-      </c>
-      <c r="F61" s="20">
-        <v>46317</v>
-      </c>
-      <c r="G61" s="19" t="inlineStr">
-        <is>
-          <t>Cumplido</t>
-        </is>
-      </c>
-      <c r="H61" s="21" t="inlineStr">
-        <is>
-          <t>#56</t>
-        </is>
-      </c>
-      <c r="I61" s="22" t="n"/>
-      <c r="J61" s="22" t="n"/>
-      <c r="K61" s="22" t="n"/>
-      <c r="L61" s="22" t="n"/>
-      <c r="M61" s="22" t="n"/>
-      <c r="N61" s="22" t="n"/>
-      <c r="O61" s="22" t="n"/>
-      <c r="P61" s="22" t="n"/>
-      <c r="Q61" s="22" t="n"/>
-      <c r="R61" s="22" t="n"/>
-      <c r="S61" s="22" t="n"/>
-      <c r="T61" s="22" t="n"/>
-      <c r="U61" s="22" t="n"/>
-      <c r="V61" s="22" t="n"/>
-      <c r="W61" s="22" t="n"/>
-      <c r="X61" s="22" t="n"/>
-      <c r="Y61" s="22" t="n"/>
-      <c r="Z61" s="22" t="n"/>
-      <c r="AA61" s="22" t="n"/>
-      <c r="AC61" s="23" t="inlineStr">
-        <is>
-          <t>attribution vacío en .claude/settings.json; los commits ya publicados no cambian</t>
-        </is>
-      </c>
+      <c r="B61" s="16" t="n"/>
+      <c r="C61" s="17" t="inlineStr">
+        <is>
+          <t>HITOS DEL CURSO</t>
+        </is>
+      </c>
+      <c r="D61" s="16" t="n"/>
+      <c r="E61" s="16" t="n"/>
+      <c r="F61" s="16" t="n"/>
+      <c r="G61" s="16" t="n"/>
+      <c r="H61" s="16" t="n"/>
+      <c r="I61" s="16" t="n"/>
+      <c r="J61" s="16" t="n"/>
+      <c r="K61" s="16" t="n"/>
+      <c r="L61" s="16" t="n"/>
+      <c r="M61" s="16" t="n"/>
+      <c r="N61" s="16" t="n"/>
+      <c r="O61" s="16" t="n"/>
+      <c r="P61" s="16" t="n"/>
+      <c r="Q61" s="16" t="n"/>
+      <c r="R61" s="16" t="n"/>
+      <c r="S61" s="16" t="n"/>
+      <c r="T61" s="16" t="n"/>
+      <c r="U61" s="16" t="n"/>
+      <c r="V61" s="16" t="n"/>
+      <c r="W61" s="16" t="n"/>
+      <c r="X61" s="16" t="n"/>
+      <c r="Y61" s="16" t="n"/>
+      <c r="Z61" s="16" t="n"/>
+      <c r="AA61" s="16" t="n"/>
+      <c r="AB61" s="16" t="n"/>
+      <c r="AC61" s="16" t="n"/>
     </row>
     <row r="62" ht="20.1" customHeight="1" s="1">
-      <c r="B62" s="16" t="n"/>
-      <c r="C62" s="17" t="inlineStr">
-        <is>
-          <t>HITOS DEL CURSO</t>
-        </is>
-      </c>
-      <c r="D62" s="16" t="n"/>
-      <c r="E62" s="16" t="n"/>
-      <c r="F62" s="16" t="n"/>
-      <c r="G62" s="16" t="n"/>
-      <c r="H62" s="16" t="n"/>
-      <c r="I62" s="16" t="n"/>
-      <c r="J62" s="16" t="n"/>
-      <c r="K62" s="16" t="n"/>
-      <c r="L62" s="16" t="n"/>
-      <c r="M62" s="16" t="n"/>
-      <c r="N62" s="16" t="n"/>
-      <c r="O62" s="16" t="n"/>
-      <c r="P62" s="16" t="n"/>
-      <c r="Q62" s="16" t="n"/>
-      <c r="R62" s="16" t="n"/>
-      <c r="S62" s="16" t="n"/>
-      <c r="T62" s="16" t="n"/>
-      <c r="U62" s="16" t="n"/>
-      <c r="V62" s="16" t="n"/>
-      <c r="W62" s="16" t="n"/>
-      <c r="X62" s="16" t="n"/>
-      <c r="Y62" s="16" t="n"/>
-      <c r="Z62" s="16" t="n"/>
-      <c r="AA62" s="16" t="n"/>
-      <c r="AB62" s="16" t="n"/>
-      <c r="AC62" s="16" t="n"/>
+      <c r="B62" s="18" t="n"/>
+      <c r="C62" s="19" t="inlineStr">
+        <is>
+          <t>Informe intermedio y video</t>
+        </is>
+      </c>
+      <c r="D62" s="19" t="inlineStr">
+        <is>
+          <t>Equipo</t>
+        </is>
+      </c>
+      <c r="E62" s="20" t="n">
+        <v>46316</v>
+      </c>
+      <c r="F62" s="20" t="n">
+        <v>46316</v>
+      </c>
+      <c r="G62" s="19" t="inlineStr">
+        <is>
+          <t>En curso</t>
+        </is>
+      </c>
+      <c r="H62" s="21" t="n"/>
+      <c r="I62" s="22" t="n"/>
+      <c r="J62" s="22" t="n"/>
+      <c r="K62" s="22" t="n"/>
+      <c r="L62" s="22" t="n"/>
+      <c r="M62" s="22" t="n"/>
+      <c r="N62" s="22" t="n"/>
+      <c r="O62" s="22" t="n"/>
+      <c r="P62" s="22" t="n"/>
+      <c r="Q62" s="22" t="n"/>
+      <c r="R62" s="22" t="n"/>
+      <c r="S62" s="22" t="n"/>
+      <c r="T62" s="22" t="n"/>
+      <c r="U62" s="22" t="n"/>
+      <c r="V62" s="22" t="n"/>
+      <c r="W62" s="22" t="n"/>
+      <c r="X62" s="22" t="n"/>
+      <c r="Y62" s="22" t="n"/>
+      <c r="Z62" s="22" t="n"/>
+      <c r="AA62" s="22" t="n"/>
+      <c r="AC62" s="23" t="inlineStr">
+        <is>
+          <t>Entrega 2026-10-21</t>
+        </is>
+      </c>
     </row>
     <row r="63" ht="20.1" customHeight="1" s="1">
       <c r="B63" s="18" t="n"/>
       <c r="C63" s="19" t="inlineStr">
         <is>
-          <t>Informe intermedio y video</t>
+          <t>Feria de informática</t>
         </is>
       </c>
       <c r="D63" s="19" t="inlineStr">
         <is>
-          <t>Equipo</t>
+          <t>Nicko</t>
         </is>
       </c>
       <c r="E63" s="20" t="n">
-        <v>46316</v>
+        <v>46321</v>
       </c>
       <c r="F63" s="20" t="n">
-        <v>46316</v>
+        <v>46325</v>
       </c>
       <c r="G63" s="19" t="inlineStr">
         <is>
-          <t>En curso</t>
-        </is>
-      </c>
-      <c r="H63" s="21" t="n"/>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="H63" s="21" t="inlineStr">
+        <is>
+          <t>#38</t>
+        </is>
+      </c>
       <c r="I63" s="22" t="n"/>
       <c r="J63" s="22" t="n"/>
       <c r="K63" s="22" t="n"/>
@@ -3436,7 +3436,7 @@
       <c r="AA63" s="22" t="n"/>
       <c r="AC63" s="23" t="inlineStr">
         <is>
-          <t>Entrega 2026-10-21</t>
+          <t>Día y hora por informar</t>
         </is>
       </c>
     </row>
@@ -3444,16 +3444,16 @@
       <c r="B64" s="18" t="n"/>
       <c r="C64" s="19" t="inlineStr">
         <is>
-          <t>Feria de informática</t>
+          <t>Evaluación 2 (Avance): 50% de los C.U y demo del Sprint 1</t>
         </is>
       </c>
       <c r="D64" s="19" t="inlineStr">
         <is>
-          <t>Nicko</t>
+          <t>Equipo</t>
         </is>
       </c>
       <c r="E64" s="20" t="n">
-        <v>46321</v>
+        <v>46323</v>
       </c>
       <c r="F64" s="20" t="n">
         <v>46325</v>
@@ -3463,11 +3463,7 @@
           <t>Pendiente</t>
         </is>
       </c>
-      <c r="H64" s="21" t="inlineStr">
-        <is>
-          <t>#38</t>
-        </is>
-      </c>
+      <c r="H64" s="21" t="n"/>
       <c r="I64" s="22" t="n"/>
       <c r="J64" s="22" t="n"/>
       <c r="K64" s="22" t="n"/>
@@ -3489,7 +3485,7 @@
       <c r="AA64" s="22" t="n"/>
       <c r="AC64" s="23" t="inlineStr">
         <is>
-          <t>Día y hora por informar</t>
+          <t>Día exacto por confirmar</t>
         </is>
       </c>
     </row>
@@ -3497,7 +3493,7 @@
       <c r="B65" s="18" t="n"/>
       <c r="C65" s="19" t="inlineStr">
         <is>
-          <t>Evaluación 2 (Avance): 50% de los C.U y demo del Sprint 1</t>
+          <t>Entrega final de la Fase 2</t>
         </is>
       </c>
       <c r="D65" s="19" t="inlineStr">
@@ -3506,10 +3502,10 @@
         </is>
       </c>
       <c r="E65" s="20" t="n">
-        <v>46323</v>
+        <v>46349</v>
       </c>
       <c r="F65" s="20" t="n">
-        <v>46325</v>
+        <v>46353</v>
       </c>
       <c r="G65" s="19" t="inlineStr">
         <is>
@@ -3538,142 +3534,94 @@
       <c r="AA65" s="22" t="n"/>
       <c r="AC65" s="23" t="inlineStr">
         <is>
-          <t>Día exacto por confirmar</t>
+          <t>Semana 15, por confirmar</t>
         </is>
       </c>
     </row>
     <row r="66" ht="20.1" customHeight="1" s="1">
-      <c r="B66" s="18" t="n"/>
-      <c r="C66" s="19" t="inlineStr">
-        <is>
-          <t>Entrega final de la Fase 2</t>
-        </is>
-      </c>
-      <c r="D66" s="19" t="inlineStr">
+      <c r="B66" s="16" t="n"/>
+      <c r="C66" s="17" t="inlineStr">
+        <is>
+          <t>FASE 3</t>
+        </is>
+      </c>
+      <c r="D66" s="16" t="n"/>
+      <c r="E66" s="16" t="n"/>
+      <c r="F66" s="16" t="n"/>
+      <c r="G66" s="16" t="n"/>
+      <c r="H66" s="16" t="n"/>
+      <c r="I66" s="16" t="n"/>
+      <c r="J66" s="16" t="n"/>
+      <c r="K66" s="16" t="n"/>
+      <c r="L66" s="16" t="n"/>
+      <c r="M66" s="16" t="n"/>
+      <c r="N66" s="16" t="n"/>
+      <c r="O66" s="16" t="n"/>
+      <c r="P66" s="16" t="n"/>
+      <c r="Q66" s="16" t="n"/>
+      <c r="R66" s="16" t="n"/>
+      <c r="S66" s="16" t="n"/>
+      <c r="T66" s="16" t="n"/>
+      <c r="U66" s="16" t="n"/>
+      <c r="V66" s="16" t="n"/>
+      <c r="W66" s="16" t="n"/>
+      <c r="X66" s="16" t="n"/>
+      <c r="Y66" s="16" t="n"/>
+      <c r="Z66" s="16" t="n"/>
+      <c r="AA66" s="16" t="n"/>
+      <c r="AB66" s="16" t="n"/>
+      <c r="AC66" s="16" t="n"/>
+    </row>
+    <row r="67" ht="20.1" customHeight="1" s="1">
+      <c r="B67" s="18" t="n"/>
+      <c r="C67" s="19" t="inlineStr">
+        <is>
+          <t>Ajustes finales, manuales y exposición ante la Comisión</t>
+        </is>
+      </c>
+      <c r="D67" s="19" t="inlineStr">
         <is>
           <t>Equipo</t>
         </is>
       </c>
-      <c r="E66" s="20" t="n">
-        <v>46349</v>
-      </c>
-      <c r="F66" s="20" t="n">
-        <v>46353</v>
-      </c>
-      <c r="G66" s="19" t="inlineStr">
+      <c r="E67" s="20" t="n">
+        <v>46356</v>
+      </c>
+      <c r="F67" s="20" t="n">
+        <v>46374</v>
+      </c>
+      <c r="G67" s="19" t="inlineStr">
         <is>
           <t>Pendiente</t>
         </is>
       </c>
-      <c r="H66" s="21" t="n"/>
-      <c r="I66" s="22" t="n"/>
-      <c r="J66" s="22" t="n"/>
-      <c r="K66" s="22" t="n"/>
-      <c r="L66" s="22" t="n"/>
-      <c r="M66" s="22" t="n"/>
-      <c r="N66" s="22" t="n"/>
-      <c r="O66" s="22" t="n"/>
-      <c r="P66" s="22" t="n"/>
-      <c r="Q66" s="22" t="n"/>
-      <c r="R66" s="22" t="n"/>
-      <c r="S66" s="22" t="n"/>
-      <c r="T66" s="22" t="n"/>
-      <c r="U66" s="22" t="n"/>
-      <c r="V66" s="22" t="n"/>
-      <c r="W66" s="22" t="n"/>
-      <c r="X66" s="22" t="n"/>
-      <c r="Y66" s="22" t="n"/>
-      <c r="Z66" s="22" t="n"/>
-      <c r="AA66" s="22" t="n"/>
-      <c r="AC66" s="23" t="inlineStr">
-        <is>
-          <t>Semana 15, por confirmar</t>
-        </is>
-      </c>
-    </row>
-    <row r="67" ht="20.1" customHeight="1" s="1">
-      <c r="B67" s="16" t="n"/>
-      <c r="C67" s="17" t="inlineStr">
-        <is>
-          <t>FASE 3</t>
-        </is>
-      </c>
-      <c r="D67" s="16" t="n"/>
-      <c r="E67" s="16" t="n"/>
-      <c r="F67" s="16" t="n"/>
-      <c r="G67" s="16" t="n"/>
-      <c r="H67" s="16" t="n"/>
-      <c r="I67" s="16" t="n"/>
-      <c r="J67" s="16" t="n"/>
-      <c r="K67" s="16" t="n"/>
-      <c r="L67" s="16" t="n"/>
-      <c r="M67" s="16" t="n"/>
-      <c r="N67" s="16" t="n"/>
-      <c r="O67" s="16" t="n"/>
-      <c r="P67" s="16" t="n"/>
-      <c r="Q67" s="16" t="n"/>
-      <c r="R67" s="16" t="n"/>
-      <c r="S67" s="16" t="n"/>
-      <c r="T67" s="16" t="n"/>
-      <c r="U67" s="16" t="n"/>
-      <c r="V67" s="16" t="n"/>
-      <c r="W67" s="16" t="n"/>
-      <c r="X67" s="16" t="n"/>
-      <c r="Y67" s="16" t="n"/>
-      <c r="Z67" s="16" t="n"/>
-      <c r="AA67" s="16" t="n"/>
-      <c r="AB67" s="16" t="n"/>
-      <c r="AC67" s="16" t="n"/>
-    </row>
-    <row r="68" ht="20.1" customHeight="1" s="1">
-      <c r="B68" s="18" t="n"/>
-      <c r="C68" s="19" t="inlineStr">
-        <is>
-          <t>Ajustes finales, manuales y exposición ante la Comisión</t>
-        </is>
-      </c>
-      <c r="D68" s="19" t="inlineStr">
-        <is>
-          <t>Equipo</t>
-        </is>
-      </c>
-      <c r="E68" s="20" t="n">
-        <v>46356</v>
-      </c>
-      <c r="F68" s="20" t="n">
-        <v>46374</v>
-      </c>
-      <c r="G68" s="19" t="inlineStr">
-        <is>
-          <t>Pendiente</t>
-        </is>
-      </c>
-      <c r="H68" s="21" t="n"/>
-      <c r="I68" s="22" t="n"/>
-      <c r="J68" s="22" t="n"/>
-      <c r="K68" s="22" t="n"/>
-      <c r="L68" s="22" t="n"/>
-      <c r="M68" s="22" t="n"/>
-      <c r="N68" s="22" t="n"/>
-      <c r="O68" s="22" t="n"/>
-      <c r="P68" s="22" t="n"/>
-      <c r="Q68" s="22" t="n"/>
-      <c r="R68" s="22" t="n"/>
-      <c r="S68" s="22" t="n"/>
-      <c r="T68" s="22" t="n"/>
-      <c r="U68" s="22" t="n"/>
-      <c r="V68" s="22" t="n"/>
-      <c r="W68" s="22" t="n"/>
-      <c r="X68" s="22" t="n"/>
-      <c r="Y68" s="22" t="n"/>
-      <c r="Z68" s="22" t="n"/>
-      <c r="AA68" s="22" t="n"/>
-      <c r="AC68" s="23" t="inlineStr">
+      <c r="H67" s="21" t="n"/>
+      <c r="I67" s="22" t="n"/>
+      <c r="J67" s="22" t="n"/>
+      <c r="K67" s="22" t="n"/>
+      <c r="L67" s="22" t="n"/>
+      <c r="M67" s="22" t="n"/>
+      <c r="N67" s="22" t="n"/>
+      <c r="O67" s="22" t="n"/>
+      <c r="P67" s="22" t="n"/>
+      <c r="Q67" s="22" t="n"/>
+      <c r="R67" s="22" t="n"/>
+      <c r="S67" s="22" t="n"/>
+      <c r="T67" s="22" t="n"/>
+      <c r="U67" s="22" t="n"/>
+      <c r="V67" s="22" t="n"/>
+      <c r="W67" s="22" t="n"/>
+      <c r="X67" s="22" t="n"/>
+      <c r="Y67" s="22" t="n"/>
+      <c r="Z67" s="22" t="n"/>
+      <c r="AA67" s="22" t="n"/>
+      <c r="AC67" s="23" t="inlineStr">
         <is>
           <t>Fechas por definir</t>
         </is>
       </c>
     </row>
+    <row r="68" ht="15.75" customHeight="1" s="1"/>
     <row r="69" ht="15.75" customHeight="1" s="1"/>
     <row r="70" ht="15.75" customHeight="1" s="1"/>
     <row r="71" ht="15.75" customHeight="1" s="1"/>
@@ -4608,7 +4556,6 @@
     <row r="1000" ht="15.75" customHeight="1" s="1"/>
     <row r="1001" ht="15.75" customHeight="1" s="1"/>
     <row r="1002" ht="15.75" customHeight="1" s="1"/>
-    <row r="1003" ht="15.75" customHeight="1" s="1"/>
   </sheetData>
   <mergeCells count="5">
     <mergeCell ref="U8:Y8"/>
@@ -4617,7 +4564,7 @@
     <mergeCell ref="Q8:T8"/>
     <mergeCell ref="I8:L8"/>
   </mergeCells>
-  <conditionalFormatting sqref="B10:B68">
+  <conditionalFormatting sqref="B10:B67">
     <cfRule type="expression" priority="2" dxfId="5" stopIfTrue="1">
       <formula>$G10="Cumplido"</formula>
     </cfRule>
@@ -4634,7 +4581,7 @@
       <formula>$G10="Bloqueado"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="I10:AA68">
+  <conditionalFormatting sqref="I10:AA67">
     <cfRule type="expression" priority="1" dxfId="5" stopIfTrue="1">
       <formula>AND($E10&lt;&gt;"",I$9&lt;=$F10,I$9+6&gt;=$E10,$G10="Cumplido")</formula>
     </cfRule>
@@ -4651,7 +4598,7 @@
       <formula>AND($E10&lt;&gt;"",I$9&lt;=$F10,I$9+6&gt;=$E10,$G10="Bloqueado")</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="S10:S68">
+  <conditionalFormatting sqref="S10:S67">
     <cfRule type="expression" priority="11" dxfId="0">
       <formula>$G10&lt;&gt;""</formula>
     </cfRule>

</xml_diff>

<commit_message>
docs: document photo deletion and mark #45 done
</commit_message>
<xml_diff>
--- a/Anexos/Gestion/Carta Gantt Fase 2.xlsx
+++ b/Anexos/Gestion/Carta Gantt Fase 2.xlsx
@@ -10,7 +10,7 @@
   </sheets>
   <definedNames>
     <definedName name="_xlnm.Print_Titles" localSheetId="0">'Carta Gantt'!$8:$9</definedName>
-    <definedName name="_xlnm.Print_Area" localSheetId="0">'Carta Gantt'!$B$1:$AC$67</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="0">'Carta Gantt'!$B$1:$AC$68</definedName>
   </definedNames>
   <calcPr calcId="191029" fullCalcOnLoad="1"/>
 </workbook>
@@ -655,7 +655,7 @@
     <outlinePr summaryBelow="0" summaryRight="0"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:AC67"/>
+  <dimension ref="A1:AC68"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="12.5703125" defaultRowHeight="15" customHeight="1"/>
   <cols>
     <col width="2" customWidth="1" style="1" min="1" max="1"/>
@@ -695,23 +695,23 @@
     <row r="4" ht="15.75" customHeight="1" s="1"/>
     <row r="5" ht="26.1" customHeight="1" s="1">
       <c r="D5" s="5">
-        <f>COUNTIF($G$10:$G$67,"Cumplido")</f>
+        <f>COUNTIF($G$10:$G$68,"Cumplido")</f>
         <v/>
       </c>
       <c r="E5" s="6">
-        <f>COUNTIF($G$10:$G$67,"En curso")</f>
+        <f>COUNTIF($G$10:$G$68,"En curso")</f>
         <v/>
       </c>
       <c r="F5" s="7">
-        <f>COUNTIF($G$10:$G$67,"Pendiente")</f>
+        <f>COUNTIF($G$10:$G$68,"Pendiente")</f>
         <v/>
       </c>
       <c r="G5" s="8">
-        <f>COUNTIF($G$10:$G$67,"Atrasado")</f>
+        <f>COUNTIF($G$10:$G$68,"Atrasado")</f>
         <v/>
       </c>
       <c r="H5" s="9">
-        <f>COUNTIF($G$10:$G$67,"Bloqueado")</f>
+        <f>COUNTIF($G$10:$G$68,"Bloqueado")</f>
         <v/>
       </c>
     </row>
@@ -2666,28 +2666,28 @@
       <c r="B48" s="18" t="n"/>
       <c r="C48" s="19" t="inlineStr">
         <is>
-          <t>Limpieza de código y CI (#54)</t>
+          <t>Privacidad de las fotos: borrado tras N días (RNF05)</t>
         </is>
       </c>
       <c r="D48" s="19" t="inlineStr">
         <is>
-          <t>Nicko</t>
-        </is>
-      </c>
-      <c r="E48" s="20" t="n">
-        <v>46323</v>
-      </c>
-      <c r="F48" s="20" t="n">
-        <v>46325</v>
+          <t>Mariana</t>
+        </is>
+      </c>
+      <c r="E48" s="20">
+        <v>46317</v>
+      </c>
+      <c r="F48" s="20">
+        <v>46317</v>
       </c>
       <c r="G48" s="19" t="inlineStr">
         <is>
-          <t>Pendiente</t>
+          <t>Cumplido</t>
         </is>
       </c>
       <c r="H48" s="21" t="inlineStr">
         <is>
-          <t>#54</t>
+          <t>#45</t>
         </is>
       </c>
       <c r="I48" s="22" t="n"/>
@@ -2709,13 +2709,17 @@
       <c r="Y48" s="22" t="n"/>
       <c r="Z48" s="22" t="n"/>
       <c r="AA48" s="22" t="n"/>
-      <c r="AC48" s="23" t="n"/>
+      <c r="AC48" s="23" t="inlineStr">
+        <is>
+          <t>Comando borrar_fotos (30 días por defecto, a confirmar con Walmart, #24)</t>
+        </is>
+      </c>
     </row>
     <row r="49" ht="20.1" customHeight="1" s="1">
       <c r="B49" s="18" t="n"/>
       <c r="C49" s="19" t="inlineStr">
         <is>
-          <t>Primer demo operativo ante Walmart</t>
+          <t>Limpieza de código y CI (#54)</t>
         </is>
       </c>
       <c r="D49" s="19" t="inlineStr">
@@ -2724,10 +2728,10 @@
         </is>
       </c>
       <c r="E49" s="20" t="n">
-        <v>46322</v>
+        <v>46323</v>
       </c>
       <c r="F49" s="20" t="n">
-        <v>46326</v>
+        <v>46325</v>
       </c>
       <c r="G49" s="19" t="inlineStr">
         <is>
@@ -2736,7 +2740,7 @@
       </c>
       <c r="H49" s="21" t="inlineStr">
         <is>
-          <t>#29</t>
+          <t>#54</t>
         </is>
       </c>
       <c r="I49" s="22" t="n"/>
@@ -2758,34 +2762,34 @@
       <c r="Y49" s="22" t="n"/>
       <c r="Z49" s="22" t="n"/>
       <c r="AA49" s="22" t="n"/>
-      <c r="AC49" s="23" t="inlineStr">
-        <is>
-          <t>Depende de #28</t>
-        </is>
-      </c>
+      <c r="AC49" s="23" t="n"/>
     </row>
     <row r="50" ht="20.1" customHeight="1" s="1">
       <c r="B50" s="18" t="n"/>
       <c r="C50" s="19" t="inlineStr">
         <is>
-          <t>Instalación en el servidor del CITT</t>
+          <t>Primer demo operativo ante Walmart</t>
         </is>
       </c>
       <c r="D50" s="19" t="inlineStr">
         <is>
-          <t>Por definir</t>
-        </is>
-      </c>
-      <c r="E50" s="20" t="n"/>
-      <c r="F50" s="20" t="n"/>
+          <t>Nicko</t>
+        </is>
+      </c>
+      <c r="E50" s="20" t="n">
+        <v>46322</v>
+      </c>
+      <c r="F50" s="20" t="n">
+        <v>46326</v>
+      </c>
       <c r="G50" s="19" t="inlineStr">
         <is>
-          <t>Bloqueado</t>
+          <t>Pendiente</t>
         </is>
       </c>
       <c r="H50" s="21" t="inlineStr">
         <is>
-          <t>#39</t>
+          <t>#29</t>
         </is>
       </c>
       <c r="I50" s="22" t="n"/>
@@ -2809,98 +2813,98 @@
       <c r="AA50" s="22" t="n"/>
       <c r="AC50" s="23" t="inlineStr">
         <is>
+          <t>Depende de #28</t>
+        </is>
+      </c>
+    </row>
+    <row r="51" ht="20.1" customHeight="1" s="1">
+      <c r="B51" s="18" t="n"/>
+      <c r="C51" s="19" t="inlineStr">
+        <is>
+          <t>Instalación en el servidor del CITT</t>
+        </is>
+      </c>
+      <c r="D51" s="19" t="inlineStr">
+        <is>
+          <t>Por definir</t>
+        </is>
+      </c>
+      <c r="E51" s="20" t="n"/>
+      <c r="F51" s="20" t="n"/>
+      <c r="G51" s="19" t="inlineStr">
+        <is>
+          <t>Bloqueado</t>
+        </is>
+      </c>
+      <c r="H51" s="21" t="inlineStr">
+        <is>
+          <t>#39</t>
+        </is>
+      </c>
+      <c r="I51" s="22" t="n"/>
+      <c r="J51" s="22" t="n"/>
+      <c r="K51" s="22" t="n"/>
+      <c r="L51" s="22" t="n"/>
+      <c r="M51" s="22" t="n"/>
+      <c r="N51" s="22" t="n"/>
+      <c r="O51" s="22" t="n"/>
+      <c r="P51" s="22" t="n"/>
+      <c r="Q51" s="22" t="n"/>
+      <c r="R51" s="22" t="n"/>
+      <c r="S51" s="22" t="n"/>
+      <c r="T51" s="22" t="n"/>
+      <c r="U51" s="22" t="n"/>
+      <c r="V51" s="22" t="n"/>
+      <c r="W51" s="22" t="n"/>
+      <c r="X51" s="22" t="n"/>
+      <c r="Y51" s="22" t="n"/>
+      <c r="Z51" s="22" t="n"/>
+      <c r="AA51" s="22" t="n"/>
+      <c r="AC51" s="23" t="inlineStr">
+        <is>
           <t>Faltan las instrucciones del CITT</t>
         </is>
       </c>
     </row>
-    <row r="51" ht="20.1" customHeight="1" s="1">
-      <c r="B51" s="16" t="n"/>
-      <c r="C51" s="17" t="inlineStr">
+    <row r="52" ht="20.1" customHeight="1" s="1">
+      <c r="B52" s="16" t="n"/>
+      <c r="C52" s="17" t="inlineStr">
         <is>
           <t>FASE 2 · DOCUMENTACIÓN</t>
         </is>
       </c>
-      <c r="D51" s="16" t="n"/>
-      <c r="E51" s="16" t="n"/>
-      <c r="F51" s="16" t="n"/>
-      <c r="G51" s="16" t="n"/>
-      <c r="H51" s="16" t="n"/>
-      <c r="I51" s="16" t="n"/>
-      <c r="J51" s="16" t="n"/>
-      <c r="K51" s="16" t="n"/>
-      <c r="L51" s="16" t="n"/>
-      <c r="M51" s="16" t="n"/>
-      <c r="N51" s="16" t="n"/>
-      <c r="O51" s="16" t="n"/>
-      <c r="P51" s="16" t="n"/>
-      <c r="Q51" s="16" t="n"/>
-      <c r="R51" s="16" t="n"/>
-      <c r="S51" s="16" t="n"/>
-      <c r="T51" s="16" t="n"/>
-      <c r="U51" s="16" t="n"/>
-      <c r="V51" s="16" t="n"/>
-      <c r="W51" s="16" t="n"/>
-      <c r="X51" s="16" t="n"/>
-      <c r="Y51" s="16" t="n"/>
-      <c r="Z51" s="16" t="n"/>
-      <c r="AA51" s="16" t="n"/>
-      <c r="AB51" s="16" t="n"/>
-      <c r="AC51" s="16" t="n"/>
-    </row>
-    <row r="52" ht="20.1" customHeight="1" s="1">
-      <c r="B52" s="18" t="n"/>
-      <c r="C52" s="19" t="inlineStr">
-        <is>
-          <t>Registro de requisitos y plazos del curso</t>
-        </is>
-      </c>
-      <c r="D52" s="19" t="inlineStr">
-        <is>
-          <t>Francisco</t>
-        </is>
-      </c>
-      <c r="E52" s="20" t="n">
-        <v>46304</v>
-      </c>
-      <c r="F52" s="20" t="n">
-        <v>46305</v>
-      </c>
-      <c r="G52" s="19" t="inlineStr">
-        <is>
-          <t>Cumplido</t>
-        </is>
-      </c>
-      <c r="H52" s="21" t="inlineStr">
-        <is>
-          <t>#23, #25</t>
-        </is>
-      </c>
-      <c r="I52" s="22" t="n"/>
-      <c r="J52" s="22" t="n"/>
-      <c r="K52" s="22" t="n"/>
-      <c r="L52" s="22" t="n"/>
-      <c r="M52" s="22" t="n"/>
-      <c r="N52" s="22" t="n"/>
-      <c r="O52" s="22" t="n"/>
-      <c r="P52" s="22" t="n"/>
-      <c r="Q52" s="22" t="n"/>
-      <c r="R52" s="22" t="n"/>
-      <c r="S52" s="22" t="n"/>
-      <c r="T52" s="22" t="n"/>
-      <c r="U52" s="22" t="n"/>
-      <c r="V52" s="22" t="n"/>
-      <c r="W52" s="22" t="n"/>
-      <c r="X52" s="22" t="n"/>
-      <c r="Y52" s="22" t="n"/>
-      <c r="Z52" s="22" t="n"/>
-      <c r="AA52" s="22" t="n"/>
-      <c r="AC52" s="23" t="n"/>
+      <c r="D52" s="16" t="n"/>
+      <c r="E52" s="16" t="n"/>
+      <c r="F52" s="16" t="n"/>
+      <c r="G52" s="16" t="n"/>
+      <c r="H52" s="16" t="n"/>
+      <c r="I52" s="16" t="n"/>
+      <c r="J52" s="16" t="n"/>
+      <c r="K52" s="16" t="n"/>
+      <c r="L52" s="16" t="n"/>
+      <c r="M52" s="16" t="n"/>
+      <c r="N52" s="16" t="n"/>
+      <c r="O52" s="16" t="n"/>
+      <c r="P52" s="16" t="n"/>
+      <c r="Q52" s="16" t="n"/>
+      <c r="R52" s="16" t="n"/>
+      <c r="S52" s="16" t="n"/>
+      <c r="T52" s="16" t="n"/>
+      <c r="U52" s="16" t="n"/>
+      <c r="V52" s="16" t="n"/>
+      <c r="W52" s="16" t="n"/>
+      <c r="X52" s="16" t="n"/>
+      <c r="Y52" s="16" t="n"/>
+      <c r="Z52" s="16" t="n"/>
+      <c r="AA52" s="16" t="n"/>
+      <c r="AB52" s="16" t="n"/>
+      <c r="AC52" s="16" t="n"/>
     </row>
     <row r="53" ht="20.1" customHeight="1" s="1">
       <c r="B53" s="18" t="n"/>
       <c r="C53" s="19" t="inlineStr">
         <is>
-          <t>Casos de uso y diagramas alineados con Walmart</t>
+          <t>Registro de requisitos y plazos del curso</t>
         </is>
       </c>
       <c r="D53" s="19" t="inlineStr">
@@ -2921,7 +2925,7 @@
       </c>
       <c r="H53" s="21" t="inlineStr">
         <is>
-          <t>#30</t>
+          <t>#23, #25</t>
         </is>
       </c>
       <c r="I53" s="22" t="n"/>
@@ -2949,19 +2953,19 @@
       <c r="B54" s="18" t="n"/>
       <c r="C54" s="19" t="inlineStr">
         <is>
-          <t>Plan de mejoras de la Fase 1</t>
+          <t>Casos de uso y diagramas alineados con Walmart</t>
         </is>
       </c>
       <c r="D54" s="19" t="inlineStr">
         <is>
-          <t>Mariana</t>
+          <t>Francisco</t>
         </is>
       </c>
       <c r="E54" s="20" t="n">
-        <v>46315</v>
+        <v>46304</v>
       </c>
       <c r="F54" s="20" t="n">
-        <v>46315</v>
+        <v>46305</v>
       </c>
       <c r="G54" s="19" t="inlineStr">
         <is>
@@ -2970,7 +2974,7 @@
       </c>
       <c r="H54" s="21" t="inlineStr">
         <is>
-          <t>#26</t>
+          <t>#30</t>
         </is>
       </c>
       <c r="I54" s="22" t="n"/>
@@ -2992,38 +2996,34 @@
       <c r="Y54" s="22" t="n"/>
       <c r="Z54" s="22" t="n"/>
       <c r="AA54" s="22" t="n"/>
-      <c r="AC54" s="23" t="inlineStr">
-        <is>
-          <t>Hecho el 2026-10-20, con atraso (plazo 2026-10-09). docs/plan-de-mejoras.md</t>
-        </is>
-      </c>
+      <c r="AC54" s="23" t="n"/>
     </row>
     <row r="55" ht="20.1" customHeight="1" s="1">
       <c r="B55" s="18" t="n"/>
       <c r="C55" s="19" t="inlineStr">
         <is>
-          <t>Informe intermedio: estado de avance y conclusiones</t>
+          <t>Plan de mejoras de la Fase 1</t>
         </is>
       </c>
       <c r="D55" s="19" t="inlineStr">
         <is>
-          <t>Francisco</t>
+          <t>Mariana</t>
         </is>
       </c>
       <c r="E55" s="20" t="n">
-        <v>46314</v>
+        <v>46315</v>
       </c>
       <c r="F55" s="20" t="n">
-        <v>46316</v>
+        <v>46315</v>
       </c>
       <c r="G55" s="19" t="inlineStr">
         <is>
-          <t>En curso</t>
+          <t>Cumplido</t>
         </is>
       </c>
       <c r="H55" s="21" t="inlineStr">
         <is>
-          <t>#27</t>
+          <t>#26</t>
         </is>
       </c>
       <c r="I55" s="22" t="n"/>
@@ -3047,7 +3047,7 @@
       <c r="AA55" s="22" t="n"/>
       <c r="AC55" s="23" t="inlineStr">
         <is>
-          <t>Antes de Nicko; Francisco lo arma en Word</t>
+          <t>Hecho el 2026-10-20, con atraso (plazo 2026-10-09). docs/plan-de-mejoras.md</t>
         </is>
       </c>
     </row>
@@ -3055,7 +3055,7 @@
       <c r="B56" s="18" t="n"/>
       <c r="C56" s="19" t="inlineStr">
         <is>
-          <t>Análisis de resultados: 10 mejores y 10 peores casos</t>
+          <t>Informe intermedio: estado de avance y conclusiones</t>
         </is>
       </c>
       <c r="D56" s="19" t="inlineStr">
@@ -3064,19 +3064,19 @@
         </is>
       </c>
       <c r="E56" s="20" t="n">
-        <v>46315</v>
+        <v>46314</v>
       </c>
       <c r="F56" s="20" t="n">
-        <v>46315</v>
+        <v>46316</v>
       </c>
       <c r="G56" s="19" t="inlineStr">
         <is>
-          <t>Cumplido</t>
+          <t>En curso</t>
         </is>
       </c>
       <c r="H56" s="21" t="inlineStr">
         <is>
-          <t>#34</t>
+          <t>#27</t>
         </is>
       </c>
       <c r="I56" s="22" t="n"/>
@@ -3098,13 +3098,17 @@
       <c r="Y56" s="22" t="n"/>
       <c r="Z56" s="22" t="n"/>
       <c r="AA56" s="22" t="n"/>
-      <c r="AC56" s="23" t="n"/>
+      <c r="AC56" s="23" t="inlineStr">
+        <is>
+          <t>Antes de Nicko; Francisco lo arma en Word</t>
+        </is>
+      </c>
     </row>
     <row r="57" ht="20.1" customHeight="1" s="1">
       <c r="B57" s="18" t="n"/>
       <c r="C57" s="19" t="inlineStr">
         <is>
-          <t>README completo</t>
+          <t>Análisis de resultados: 10 mejores y 10 peores casos</t>
         </is>
       </c>
       <c r="D57" s="19" t="inlineStr">
@@ -3125,7 +3129,7 @@
       </c>
       <c r="H57" s="21" t="inlineStr">
         <is>
-          <t>#35</t>
+          <t>#34</t>
         </is>
       </c>
       <c r="I57" s="22" t="n"/>
@@ -3153,28 +3157,28 @@
       <c r="B58" s="18" t="n"/>
       <c r="C58" s="19" t="inlineStr">
         <is>
-          <t>Video de demostración (5 a 10 min)</t>
+          <t>README completo</t>
         </is>
       </c>
       <c r="D58" s="19" t="inlineStr">
         <is>
-          <t>Nicko</t>
+          <t>Francisco</t>
         </is>
       </c>
       <c r="E58" s="20" t="n">
-        <v>46316</v>
+        <v>46315</v>
       </c>
       <c r="F58" s="20" t="n">
-        <v>46316</v>
+        <v>46315</v>
       </c>
       <c r="G58" s="19" t="inlineStr">
         <is>
-          <t>Pendiente</t>
+          <t>Cumplido</t>
         </is>
       </c>
       <c r="H58" s="21" t="inlineStr">
         <is>
-          <t>#36</t>
+          <t>#35</t>
         </is>
       </c>
       <c r="I58" s="22" t="n"/>
@@ -3202,28 +3206,28 @@
       <c r="B59" s="18" t="n"/>
       <c r="C59" s="19" t="inlineStr">
         <is>
-          <t>Evidencias de avance: diario 2.1 y guía 2.4</t>
+          <t>Video de demostración (5 a 10 min)</t>
         </is>
       </c>
       <c r="D59" s="19" t="inlineStr">
         <is>
-          <t>Mariana</t>
+          <t>Nicko</t>
         </is>
       </c>
       <c r="E59" s="20" t="n">
-        <v>46315</v>
+        <v>46316</v>
       </c>
       <c r="F59" s="20" t="n">
-        <v>46321</v>
+        <v>46316</v>
       </c>
       <c r="G59" s="19" t="inlineStr">
         <is>
-          <t>En curso</t>
+          <t>Pendiente</t>
         </is>
       </c>
       <c r="H59" s="21" t="inlineStr">
         <is>
-          <t>#37</t>
+          <t>#36</t>
         </is>
       </c>
       <c r="I59" s="22" t="n"/>
@@ -3245,17 +3249,13 @@
       <c r="Y59" s="22" t="n"/>
       <c r="Z59" s="22" t="n"/>
       <c r="AA59" s="22" t="n"/>
-      <c r="AC59" s="23" t="inlineStr">
-        <is>
-          <t>Plazo 2026-10-26. Guía 2.4 al 21-10; diario 2.1 y autoevaluación 2.2 de Mariana el 22-10 (Fase 2/). Faltan los diarios de Francisco y Nicko</t>
-        </is>
-      </c>
+      <c r="AC59" s="23" t="n"/>
     </row>
     <row r="60" ht="20.1" customHeight="1" s="1">
       <c r="B60" s="18" t="n"/>
       <c r="C60" s="19" t="inlineStr">
         <is>
-          <t>Rehacer plantillas de C.U y diagramas según la app Django</t>
+          <t>Evidencias de avance: diario 2.1 y guía 2.4</t>
         </is>
       </c>
       <c r="D60" s="19" t="inlineStr">
@@ -3264,19 +3264,19 @@
         </is>
       </c>
       <c r="E60" s="20" t="n">
-        <v>46316</v>
+        <v>46315</v>
       </c>
       <c r="F60" s="20" t="n">
-        <v>46316</v>
+        <v>46321</v>
       </c>
       <c r="G60" s="19" t="inlineStr">
         <is>
-          <t>Cumplido</t>
+          <t>En curso</t>
         </is>
       </c>
       <c r="H60" s="21" t="inlineStr">
         <is>
-          <t>#42</t>
+          <t>#37</t>
         </is>
       </c>
       <c r="I60" s="22" t="n"/>
@@ -3300,121 +3300,121 @@
       <c r="AA60" s="22" t="n"/>
       <c r="AC60" s="23" t="inlineStr">
         <is>
+          <t>Plazo 2026-10-26. Guía 2.4 al 21-10; diario 2.1 y autoevaluación 2.2 de Mariana el 22-10 (Fase 2/). Faltan los diarios de Francisco y Nicko</t>
+        </is>
+      </c>
+    </row>
+    <row r="61" ht="20.1" customHeight="1" s="1">
+      <c r="B61" s="18" t="n"/>
+      <c r="C61" s="19" t="inlineStr">
+        <is>
+          <t>Rehacer plantillas de C.U y diagramas según la app Django</t>
+        </is>
+      </c>
+      <c r="D61" s="19" t="inlineStr">
+        <is>
+          <t>Mariana</t>
+        </is>
+      </c>
+      <c r="E61" s="20" t="n">
+        <v>46316</v>
+      </c>
+      <c r="F61" s="20" t="n">
+        <v>46316</v>
+      </c>
+      <c r="G61" s="19" t="inlineStr">
+        <is>
+          <t>Cumplido</t>
+        </is>
+      </c>
+      <c r="H61" s="21" t="inlineStr">
+        <is>
+          <t>#42</t>
+        </is>
+      </c>
+      <c r="I61" s="22" t="n"/>
+      <c r="J61" s="22" t="n"/>
+      <c r="K61" s="22" t="n"/>
+      <c r="L61" s="22" t="n"/>
+      <c r="M61" s="22" t="n"/>
+      <c r="N61" s="22" t="n"/>
+      <c r="O61" s="22" t="n"/>
+      <c r="P61" s="22" t="n"/>
+      <c r="Q61" s="22" t="n"/>
+      <c r="R61" s="22" t="n"/>
+      <c r="S61" s="22" t="n"/>
+      <c r="T61" s="22" t="n"/>
+      <c r="U61" s="22" t="n"/>
+      <c r="V61" s="22" t="n"/>
+      <c r="W61" s="22" t="n"/>
+      <c r="X61" s="22" t="n"/>
+      <c r="Y61" s="22" t="n"/>
+      <c r="Z61" s="22" t="n"/>
+      <c r="AA61" s="22" t="n"/>
+      <c r="AC61" s="23" t="inlineStr">
+        <is>
           <t>Hecho el 2026-10-21: plantillas, fuentes Mermaid y PNG (CU00-CU06 y arquitectura). docs/cambios-cu.md</t>
         </is>
       </c>
     </row>
-    <row r="61" ht="20.1" customHeight="1" s="1">
-      <c r="B61" s="16" t="n"/>
-      <c r="C61" s="17" t="inlineStr">
+    <row r="62" ht="20.1" customHeight="1" s="1">
+      <c r="B62" s="16" t="n"/>
+      <c r="C62" s="17" t="inlineStr">
         <is>
           <t>HITOS DEL CURSO</t>
         </is>
       </c>
-      <c r="D61" s="16" t="n"/>
-      <c r="E61" s="16" t="n"/>
-      <c r="F61" s="16" t="n"/>
-      <c r="G61" s="16" t="n"/>
-      <c r="H61" s="16" t="n"/>
-      <c r="I61" s="16" t="n"/>
-      <c r="J61" s="16" t="n"/>
-      <c r="K61" s="16" t="n"/>
-      <c r="L61" s="16" t="n"/>
-      <c r="M61" s="16" t="n"/>
-      <c r="N61" s="16" t="n"/>
-      <c r="O61" s="16" t="n"/>
-      <c r="P61" s="16" t="n"/>
-      <c r="Q61" s="16" t="n"/>
-      <c r="R61" s="16" t="n"/>
-      <c r="S61" s="16" t="n"/>
-      <c r="T61" s="16" t="n"/>
-      <c r="U61" s="16" t="n"/>
-      <c r="V61" s="16" t="n"/>
-      <c r="W61" s="16" t="n"/>
-      <c r="X61" s="16" t="n"/>
-      <c r="Y61" s="16" t="n"/>
-      <c r="Z61" s="16" t="n"/>
-      <c r="AA61" s="16" t="n"/>
-      <c r="AB61" s="16" t="n"/>
-      <c r="AC61" s="16" t="n"/>
-    </row>
-    <row r="62" ht="20.1" customHeight="1" s="1">
-      <c r="B62" s="18" t="n"/>
-      <c r="C62" s="19" t="inlineStr">
-        <is>
-          <t>Informe intermedio y video</t>
-        </is>
-      </c>
-      <c r="D62" s="19" t="inlineStr">
-        <is>
-          <t>Equipo</t>
-        </is>
-      </c>
-      <c r="E62" s="20" t="n">
-        <v>46316</v>
-      </c>
-      <c r="F62" s="20" t="n">
-        <v>46316</v>
-      </c>
-      <c r="G62" s="19" t="inlineStr">
-        <is>
-          <t>En curso</t>
-        </is>
-      </c>
-      <c r="H62" s="21" t="n"/>
-      <c r="I62" s="22" t="n"/>
-      <c r="J62" s="22" t="n"/>
-      <c r="K62" s="22" t="n"/>
-      <c r="L62" s="22" t="n"/>
-      <c r="M62" s="22" t="n"/>
-      <c r="N62" s="22" t="n"/>
-      <c r="O62" s="22" t="n"/>
-      <c r="P62" s="22" t="n"/>
-      <c r="Q62" s="22" t="n"/>
-      <c r="R62" s="22" t="n"/>
-      <c r="S62" s="22" t="n"/>
-      <c r="T62" s="22" t="n"/>
-      <c r="U62" s="22" t="n"/>
-      <c r="V62" s="22" t="n"/>
-      <c r="W62" s="22" t="n"/>
-      <c r="X62" s="22" t="n"/>
-      <c r="Y62" s="22" t="n"/>
-      <c r="Z62" s="22" t="n"/>
-      <c r="AA62" s="22" t="n"/>
-      <c r="AC62" s="23" t="inlineStr">
-        <is>
-          <t>Entrega 2026-10-21</t>
-        </is>
-      </c>
+      <c r="D62" s="16" t="n"/>
+      <c r="E62" s="16" t="n"/>
+      <c r="F62" s="16" t="n"/>
+      <c r="G62" s="16" t="n"/>
+      <c r="H62" s="16" t="n"/>
+      <c r="I62" s="16" t="n"/>
+      <c r="J62" s="16" t="n"/>
+      <c r="K62" s="16" t="n"/>
+      <c r="L62" s="16" t="n"/>
+      <c r="M62" s="16" t="n"/>
+      <c r="N62" s="16" t="n"/>
+      <c r="O62" s="16" t="n"/>
+      <c r="P62" s="16" t="n"/>
+      <c r="Q62" s="16" t="n"/>
+      <c r="R62" s="16" t="n"/>
+      <c r="S62" s="16" t="n"/>
+      <c r="T62" s="16" t="n"/>
+      <c r="U62" s="16" t="n"/>
+      <c r="V62" s="16" t="n"/>
+      <c r="W62" s="16" t="n"/>
+      <c r="X62" s="16" t="n"/>
+      <c r="Y62" s="16" t="n"/>
+      <c r="Z62" s="16" t="n"/>
+      <c r="AA62" s="16" t="n"/>
+      <c r="AB62" s="16" t="n"/>
+      <c r="AC62" s="16" t="n"/>
     </row>
     <row r="63" ht="20.1" customHeight="1" s="1">
       <c r="B63" s="18" t="n"/>
       <c r="C63" s="19" t="inlineStr">
         <is>
-          <t>Feria de informática</t>
+          <t>Informe intermedio y video</t>
         </is>
       </c>
       <c r="D63" s="19" t="inlineStr">
         <is>
-          <t>Nicko</t>
+          <t>Equipo</t>
         </is>
       </c>
       <c r="E63" s="20" t="n">
-        <v>46321</v>
+        <v>46316</v>
       </c>
       <c r="F63" s="20" t="n">
-        <v>46325</v>
+        <v>46316</v>
       </c>
       <c r="G63" s="19" t="inlineStr">
         <is>
-          <t>Pendiente</t>
-        </is>
-      </c>
-      <c r="H63" s="21" t="inlineStr">
-        <is>
-          <t>#38</t>
-        </is>
-      </c>
+          <t>En curso</t>
+        </is>
+      </c>
+      <c r="H63" s="21" t="n"/>
       <c r="I63" s="22" t="n"/>
       <c r="J63" s="22" t="n"/>
       <c r="K63" s="22" t="n"/>
@@ -3436,7 +3436,7 @@
       <c r="AA63" s="22" t="n"/>
       <c r="AC63" s="23" t="inlineStr">
         <is>
-          <t>Día y hora por informar</t>
+          <t>Entrega 2026-10-21</t>
         </is>
       </c>
     </row>
@@ -3444,16 +3444,16 @@
       <c r="B64" s="18" t="n"/>
       <c r="C64" s="19" t="inlineStr">
         <is>
-          <t>Evaluación 2 (Avance): 50% de los C.U y demo del Sprint 1</t>
+          <t>Feria de informática</t>
         </is>
       </c>
       <c r="D64" s="19" t="inlineStr">
         <is>
-          <t>Equipo</t>
+          <t>Nicko</t>
         </is>
       </c>
       <c r="E64" s="20" t="n">
-        <v>46323</v>
+        <v>46321</v>
       </c>
       <c r="F64" s="20" t="n">
         <v>46325</v>
@@ -3463,7 +3463,11 @@
           <t>Pendiente</t>
         </is>
       </c>
-      <c r="H64" s="21" t="n"/>
+      <c r="H64" s="21" t="inlineStr">
+        <is>
+          <t>#38</t>
+        </is>
+      </c>
       <c r="I64" s="22" t="n"/>
       <c r="J64" s="22" t="n"/>
       <c r="K64" s="22" t="n"/>
@@ -3485,7 +3489,7 @@
       <c r="AA64" s="22" t="n"/>
       <c r="AC64" s="23" t="inlineStr">
         <is>
-          <t>Día exacto por confirmar</t>
+          <t>Día y hora por informar</t>
         </is>
       </c>
     </row>
@@ -3493,7 +3497,7 @@
       <c r="B65" s="18" t="n"/>
       <c r="C65" s="19" t="inlineStr">
         <is>
-          <t>Entrega final de la Fase 2</t>
+          <t>Evaluación 2 (Avance): 50% de los C.U y demo del Sprint 1</t>
         </is>
       </c>
       <c r="D65" s="19" t="inlineStr">
@@ -3502,10 +3506,10 @@
         </is>
       </c>
       <c r="E65" s="20" t="n">
-        <v>46349</v>
+        <v>46323</v>
       </c>
       <c r="F65" s="20" t="n">
-        <v>46353</v>
+        <v>46325</v>
       </c>
       <c r="G65" s="19" t="inlineStr">
         <is>
@@ -3534,94 +3538,142 @@
       <c r="AA65" s="22" t="n"/>
       <c r="AC65" s="23" t="inlineStr">
         <is>
+          <t>Día exacto por confirmar</t>
+        </is>
+      </c>
+    </row>
+    <row r="66" ht="20.1" customHeight="1" s="1">
+      <c r="B66" s="18" t="n"/>
+      <c r="C66" s="19" t="inlineStr">
+        <is>
+          <t>Entrega final de la Fase 2</t>
+        </is>
+      </c>
+      <c r="D66" s="19" t="inlineStr">
+        <is>
+          <t>Equipo</t>
+        </is>
+      </c>
+      <c r="E66" s="20" t="n">
+        <v>46349</v>
+      </c>
+      <c r="F66" s="20" t="n">
+        <v>46353</v>
+      </c>
+      <c r="G66" s="19" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="H66" s="21" t="n"/>
+      <c r="I66" s="22" t="n"/>
+      <c r="J66" s="22" t="n"/>
+      <c r="K66" s="22" t="n"/>
+      <c r="L66" s="22" t="n"/>
+      <c r="M66" s="22" t="n"/>
+      <c r="N66" s="22" t="n"/>
+      <c r="O66" s="22" t="n"/>
+      <c r="P66" s="22" t="n"/>
+      <c r="Q66" s="22" t="n"/>
+      <c r="R66" s="22" t="n"/>
+      <c r="S66" s="22" t="n"/>
+      <c r="T66" s="22" t="n"/>
+      <c r="U66" s="22" t="n"/>
+      <c r="V66" s="22" t="n"/>
+      <c r="W66" s="22" t="n"/>
+      <c r="X66" s="22" t="n"/>
+      <c r="Y66" s="22" t="n"/>
+      <c r="Z66" s="22" t="n"/>
+      <c r="AA66" s="22" t="n"/>
+      <c r="AC66" s="23" t="inlineStr">
+        <is>
           <t>Semana 15, por confirmar</t>
         </is>
       </c>
     </row>
-    <row r="66" ht="20.1" customHeight="1" s="1">
-      <c r="B66" s="16" t="n"/>
-      <c r="C66" s="17" t="inlineStr">
+    <row r="67" ht="20.1" customHeight="1" s="1">
+      <c r="B67" s="16" t="n"/>
+      <c r="C67" s="17" t="inlineStr">
         <is>
           <t>FASE 3</t>
         </is>
       </c>
-      <c r="D66" s="16" t="n"/>
-      <c r="E66" s="16" t="n"/>
-      <c r="F66" s="16" t="n"/>
-      <c r="G66" s="16" t="n"/>
-      <c r="H66" s="16" t="n"/>
-      <c r="I66" s="16" t="n"/>
-      <c r="J66" s="16" t="n"/>
-      <c r="K66" s="16" t="n"/>
-      <c r="L66" s="16" t="n"/>
-      <c r="M66" s="16" t="n"/>
-      <c r="N66" s="16" t="n"/>
-      <c r="O66" s="16" t="n"/>
-      <c r="P66" s="16" t="n"/>
-      <c r="Q66" s="16" t="n"/>
-      <c r="R66" s="16" t="n"/>
-      <c r="S66" s="16" t="n"/>
-      <c r="T66" s="16" t="n"/>
-      <c r="U66" s="16" t="n"/>
-      <c r="V66" s="16" t="n"/>
-      <c r="W66" s="16" t="n"/>
-      <c r="X66" s="16" t="n"/>
-      <c r="Y66" s="16" t="n"/>
-      <c r="Z66" s="16" t="n"/>
-      <c r="AA66" s="16" t="n"/>
-      <c r="AB66" s="16" t="n"/>
-      <c r="AC66" s="16" t="n"/>
-    </row>
-    <row r="67" ht="20.1" customHeight="1" s="1">
-      <c r="B67" s="18" t="n"/>
-      <c r="C67" s="19" t="inlineStr">
+      <c r="D67" s="16" t="n"/>
+      <c r="E67" s="16" t="n"/>
+      <c r="F67" s="16" t="n"/>
+      <c r="G67" s="16" t="n"/>
+      <c r="H67" s="16" t="n"/>
+      <c r="I67" s="16" t="n"/>
+      <c r="J67" s="16" t="n"/>
+      <c r="K67" s="16" t="n"/>
+      <c r="L67" s="16" t="n"/>
+      <c r="M67" s="16" t="n"/>
+      <c r="N67" s="16" t="n"/>
+      <c r="O67" s="16" t="n"/>
+      <c r="P67" s="16" t="n"/>
+      <c r="Q67" s="16" t="n"/>
+      <c r="R67" s="16" t="n"/>
+      <c r="S67" s="16" t="n"/>
+      <c r="T67" s="16" t="n"/>
+      <c r="U67" s="16" t="n"/>
+      <c r="V67" s="16" t="n"/>
+      <c r="W67" s="16" t="n"/>
+      <c r="X67" s="16" t="n"/>
+      <c r="Y67" s="16" t="n"/>
+      <c r="Z67" s="16" t="n"/>
+      <c r="AA67" s="16" t="n"/>
+      <c r="AB67" s="16" t="n"/>
+      <c r="AC67" s="16" t="n"/>
+    </row>
+    <row r="68" ht="20.1" customHeight="1" s="1">
+      <c r="B68" s="18" t="n"/>
+      <c r="C68" s="19" t="inlineStr">
         <is>
           <t>Ajustes finales, manuales y exposición ante la Comisión</t>
         </is>
       </c>
-      <c r="D67" s="19" t="inlineStr">
+      <c r="D68" s="19" t="inlineStr">
         <is>
           <t>Equipo</t>
         </is>
       </c>
-      <c r="E67" s="20" t="n">
+      <c r="E68" s="20" t="n">
         <v>46356</v>
       </c>
-      <c r="F67" s="20" t="n">
+      <c r="F68" s="20" t="n">
         <v>46374</v>
       </c>
-      <c r="G67" s="19" t="inlineStr">
+      <c r="G68" s="19" t="inlineStr">
         <is>
           <t>Pendiente</t>
         </is>
       </c>
-      <c r="H67" s="21" t="n"/>
-      <c r="I67" s="22" t="n"/>
-      <c r="J67" s="22" t="n"/>
-      <c r="K67" s="22" t="n"/>
-      <c r="L67" s="22" t="n"/>
-      <c r="M67" s="22" t="n"/>
-      <c r="N67" s="22" t="n"/>
-      <c r="O67" s="22" t="n"/>
-      <c r="P67" s="22" t="n"/>
-      <c r="Q67" s="22" t="n"/>
-      <c r="R67" s="22" t="n"/>
-      <c r="S67" s="22" t="n"/>
-      <c r="T67" s="22" t="n"/>
-      <c r="U67" s="22" t="n"/>
-      <c r="V67" s="22" t="n"/>
-      <c r="W67" s="22" t="n"/>
-      <c r="X67" s="22" t="n"/>
-      <c r="Y67" s="22" t="n"/>
-      <c r="Z67" s="22" t="n"/>
-      <c r="AA67" s="22" t="n"/>
-      <c r="AC67" s="23" t="inlineStr">
+      <c r="H68" s="21" t="n"/>
+      <c r="I68" s="22" t="n"/>
+      <c r="J68" s="22" t="n"/>
+      <c r="K68" s="22" t="n"/>
+      <c r="L68" s="22" t="n"/>
+      <c r="M68" s="22" t="n"/>
+      <c r="N68" s="22" t="n"/>
+      <c r="O68" s="22" t="n"/>
+      <c r="P68" s="22" t="n"/>
+      <c r="Q68" s="22" t="n"/>
+      <c r="R68" s="22" t="n"/>
+      <c r="S68" s="22" t="n"/>
+      <c r="T68" s="22" t="n"/>
+      <c r="U68" s="22" t="n"/>
+      <c r="V68" s="22" t="n"/>
+      <c r="W68" s="22" t="n"/>
+      <c r="X68" s="22" t="n"/>
+      <c r="Y68" s="22" t="n"/>
+      <c r="Z68" s="22" t="n"/>
+      <c r="AA68" s="22" t="n"/>
+      <c r="AC68" s="23" t="inlineStr">
         <is>
           <t>Fechas por definir</t>
         </is>
       </c>
     </row>
-    <row r="68" ht="15.75" customHeight="1" s="1"/>
     <row r="69" ht="15.75" customHeight="1" s="1"/>
     <row r="70" ht="15.75" customHeight="1" s="1"/>
     <row r="71" ht="15.75" customHeight="1" s="1"/>
@@ -4556,6 +4608,7 @@
     <row r="1000" ht="15.75" customHeight="1" s="1"/>
     <row r="1001" ht="15.75" customHeight="1" s="1"/>
     <row r="1002" ht="15.75" customHeight="1" s="1"/>
+    <row r="1003" ht="15.75" customHeight="1" s="1"/>
   </sheetData>
   <mergeCells count="5">
     <mergeCell ref="U8:Y8"/>
@@ -4564,7 +4617,7 @@
     <mergeCell ref="Q8:T8"/>
     <mergeCell ref="I8:L8"/>
   </mergeCells>
-  <conditionalFormatting sqref="B10:B67">
+  <conditionalFormatting sqref="B10:B68">
     <cfRule type="expression" priority="2" dxfId="5" stopIfTrue="1">
       <formula>$G10="Cumplido"</formula>
     </cfRule>
@@ -4581,7 +4634,7 @@
       <formula>$G10="Bloqueado"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="I10:AA67">
+  <conditionalFormatting sqref="I10:AA68">
     <cfRule type="expression" priority="1" dxfId="5" stopIfTrue="1">
       <formula>AND($E10&lt;&gt;"",I$9&lt;=$F10,I$9+6&gt;=$E10,$G10="Cumplido")</formula>
     </cfRule>
@@ -4598,7 +4651,7 @@
       <formula>AND($E10&lt;&gt;"",I$9&lt;=$F10,I$9+6&gt;=$E10,$G10="Bloqueado")</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="S10:S67">
+  <conditionalFormatting sqref="S10:S68">
     <cfRule type="expression" priority="11" dxfId="0">
       <formula>$G10&lt;&gt;""</formula>
     </cfRule>

</xml_diff>

<commit_message>
docs: marca #27 como hecho, asigna los ítems de la auditoría (#49, #50, #51, #54) y agrega el #57
</commit_message>
<xml_diff>
--- a/Anexos/Gestion/Carta Gantt Fase 2.xlsx
+++ b/Anexos/Gestion/Carta Gantt Fase 2.xlsx
@@ -655,7 +655,7 @@
     <outlinePr summaryBelow="0" summaryRight="0"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:AC68"/>
+  <dimension ref="A1:AC69"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="12.5703125" defaultRowHeight="15" customHeight="1"/>
   <cols>
     <col width="2" customWidth="1" style="1" min="1" max="1"/>
@@ -695,23 +695,23 @@
     <row r="4" ht="15.75" customHeight="1" s="1"/>
     <row r="5" ht="26.1" customHeight="1" s="1">
       <c r="D5" s="5">
-        <f>COUNTIF($G$10:$G$68,"Cumplido")</f>
+        <f>COUNTIF($G$10:$G$69,"Cumplido")</f>
         <v/>
       </c>
       <c r="E5" s="6">
-        <f>COUNTIF($G$10:$G$68,"En curso")</f>
+        <f>COUNTIF($G$10:$G$69,"En curso")</f>
         <v/>
       </c>
       <c r="F5" s="7">
-        <f>COUNTIF($G$10:$G$68,"Pendiente")</f>
+        <f>COUNTIF($G$10:$G$69,"Pendiente")</f>
         <v/>
       </c>
       <c r="G5" s="8">
-        <f>COUNTIF($G$10:$G$68,"Atrasado")</f>
+        <f>COUNTIF($G$10:$G$69,"Atrasado")</f>
         <v/>
       </c>
       <c r="H5" s="9">
-        <f>COUNTIF($G$10:$G$68,"Bloqueado")</f>
+        <f>COUNTIF($G$10:$G$69,"Bloqueado")</f>
         <v/>
       </c>
     </row>
@@ -2621,10 +2621,10 @@
           <t>Mariana</t>
         </is>
       </c>
-      <c r="E47" s="20">
+      <c r="E47" s="20" t="n">
         <v>46317</v>
       </c>
-      <c r="F47" s="20">
+      <c r="F47" s="20" t="n">
         <v>46317</v>
       </c>
       <c r="G47" s="19" t="inlineStr">
@@ -2674,10 +2674,10 @@
           <t>Mariana</t>
         </is>
       </c>
-      <c r="E48" s="20">
+      <c r="E48" s="20" t="n">
         <v>46317</v>
       </c>
-      <c r="F48" s="20">
+      <c r="F48" s="20" t="n">
         <v>46317</v>
       </c>
       <c r="G48" s="19" t="inlineStr">
@@ -2724,7 +2724,7 @@
       </c>
       <c r="D49" s="19" t="inlineStr">
         <is>
-          <t>Nicko</t>
+          <t>Francisco</t>
         </is>
       </c>
       <c r="E49" s="20" t="n">
@@ -2768,28 +2768,28 @@
       <c r="B50" s="18" t="n"/>
       <c r="C50" s="19" t="inlineStr">
         <is>
-          <t>Primer demo operativo ante Walmart</t>
+          <t>Auditoría de seguridad por vulnerabilidades recientes (#57)</t>
         </is>
       </c>
       <c r="D50" s="19" t="inlineStr">
         <is>
-          <t>Nicko</t>
+          <t>Francisco</t>
         </is>
       </c>
       <c r="E50" s="20" t="n">
-        <v>46322</v>
+        <v>46317</v>
       </c>
       <c r="F50" s="20" t="n">
-        <v>46326</v>
+        <v>46323</v>
       </c>
       <c r="G50" s="19" t="inlineStr">
         <is>
-          <t>Pendiente</t>
+          <t>En curso</t>
         </is>
       </c>
       <c r="H50" s="21" t="inlineStr">
         <is>
-          <t>#29</t>
+          <t>#57</t>
         </is>
       </c>
       <c r="I50" s="22" t="n"/>
@@ -2821,24 +2821,28 @@
       <c r="B51" s="18" t="n"/>
       <c r="C51" s="19" t="inlineStr">
         <is>
-          <t>Instalación en el servidor del CITT</t>
+          <t>Primer demo operativo ante Walmart</t>
         </is>
       </c>
       <c r="D51" s="19" t="inlineStr">
         <is>
-          <t>Por definir</t>
-        </is>
-      </c>
-      <c r="E51" s="20" t="n"/>
-      <c r="F51" s="20" t="n"/>
+          <t>Nicko</t>
+        </is>
+      </c>
+      <c r="E51" s="20" t="n">
+        <v>46322</v>
+      </c>
+      <c r="F51" s="20" t="n">
+        <v>46326</v>
+      </c>
       <c r="G51" s="19" t="inlineStr">
         <is>
-          <t>Bloqueado</t>
+          <t>Pendiente</t>
         </is>
       </c>
       <c r="H51" s="21" t="inlineStr">
         <is>
-          <t>#39</t>
+          <t>#29</t>
         </is>
       </c>
       <c r="I51" s="22" t="n"/>
@@ -2867,93 +2871,89 @@
       </c>
     </row>
     <row r="52" ht="20.1" customHeight="1" s="1">
-      <c r="B52" s="16" t="n"/>
-      <c r="C52" s="17" t="inlineStr">
-        <is>
-          <t>FASE 2 · DOCUMENTACIÓN</t>
-        </is>
-      </c>
-      <c r="D52" s="16" t="n"/>
-      <c r="E52" s="16" t="n"/>
-      <c r="F52" s="16" t="n"/>
-      <c r="G52" s="16" t="n"/>
-      <c r="H52" s="16" t="n"/>
-      <c r="I52" s="16" t="n"/>
-      <c r="J52" s="16" t="n"/>
-      <c r="K52" s="16" t="n"/>
-      <c r="L52" s="16" t="n"/>
-      <c r="M52" s="16" t="n"/>
-      <c r="N52" s="16" t="n"/>
-      <c r="O52" s="16" t="n"/>
-      <c r="P52" s="16" t="n"/>
-      <c r="Q52" s="16" t="n"/>
-      <c r="R52" s="16" t="n"/>
-      <c r="S52" s="16" t="n"/>
-      <c r="T52" s="16" t="n"/>
-      <c r="U52" s="16" t="n"/>
-      <c r="V52" s="16" t="n"/>
-      <c r="W52" s="16" t="n"/>
-      <c r="X52" s="16" t="n"/>
-      <c r="Y52" s="16" t="n"/>
-      <c r="Z52" s="16" t="n"/>
-      <c r="AA52" s="16" t="n"/>
+      <c r="B52" s="18" t="n"/>
+      <c r="C52" s="19" t="inlineStr">
+        <is>
+          <t>Instalación en el servidor del CITT</t>
+        </is>
+      </c>
+      <c r="D52" s="19" t="inlineStr">
+        <is>
+          <t>Por definir</t>
+        </is>
+      </c>
+      <c r="E52" s="20" t="n"/>
+      <c r="F52" s="20" t="n"/>
+      <c r="G52" s="19" t="inlineStr">
+        <is>
+          <t>Bloqueado</t>
+        </is>
+      </c>
+      <c r="H52" s="21" t="inlineStr">
+        <is>
+          <t>#39</t>
+        </is>
+      </c>
+      <c r="I52" s="22" t="n"/>
+      <c r="J52" s="22" t="n"/>
+      <c r="K52" s="22" t="n"/>
+      <c r="L52" s="22" t="n"/>
+      <c r="M52" s="22" t="n"/>
+      <c r="N52" s="22" t="n"/>
+      <c r="O52" s="22" t="n"/>
+      <c r="P52" s="22" t="n"/>
+      <c r="Q52" s="22" t="n"/>
+      <c r="R52" s="22" t="n"/>
+      <c r="S52" s="22" t="n"/>
+      <c r="T52" s="22" t="n"/>
+      <c r="U52" s="22" t="n"/>
+      <c r="V52" s="22" t="n"/>
+      <c r="W52" s="22" t="n"/>
+      <c r="X52" s="22" t="n"/>
+      <c r="Y52" s="22" t="n"/>
+      <c r="Z52" s="22" t="n"/>
+      <c r="AA52" s="22" t="n"/>
       <c r="AB52" s="16" t="n"/>
       <c r="AC52" s="16" t="n"/>
     </row>
     <row r="53" ht="20.1" customHeight="1" s="1">
-      <c r="B53" s="18" t="n"/>
-      <c r="C53" s="19" t="inlineStr">
-        <is>
-          <t>Registro de requisitos y plazos del curso</t>
-        </is>
-      </c>
-      <c r="D53" s="19" t="inlineStr">
-        <is>
-          <t>Francisco</t>
-        </is>
-      </c>
-      <c r="E53" s="20" t="n">
-        <v>46304</v>
-      </c>
-      <c r="F53" s="20" t="n">
-        <v>46305</v>
-      </c>
-      <c r="G53" s="19" t="inlineStr">
-        <is>
-          <t>Cumplido</t>
-        </is>
-      </c>
-      <c r="H53" s="21" t="inlineStr">
-        <is>
-          <t>#23, #25</t>
-        </is>
-      </c>
-      <c r="I53" s="22" t="n"/>
-      <c r="J53" s="22" t="n"/>
-      <c r="K53" s="22" t="n"/>
-      <c r="L53" s="22" t="n"/>
-      <c r="M53" s="22" t="n"/>
-      <c r="N53" s="22" t="n"/>
-      <c r="O53" s="22" t="n"/>
-      <c r="P53" s="22" t="n"/>
-      <c r="Q53" s="22" t="n"/>
-      <c r="R53" s="22" t="n"/>
-      <c r="S53" s="22" t="n"/>
-      <c r="T53" s="22" t="n"/>
-      <c r="U53" s="22" t="n"/>
-      <c r="V53" s="22" t="n"/>
-      <c r="W53" s="22" t="n"/>
-      <c r="X53" s="22" t="n"/>
-      <c r="Y53" s="22" t="n"/>
-      <c r="Z53" s="22" t="n"/>
-      <c r="AA53" s="22" t="n"/>
+      <c r="B53" s="16" t="n"/>
+      <c r="C53" s="17" t="inlineStr">
+        <is>
+          <t>FASE 2 · DOCUMENTACIÓN</t>
+        </is>
+      </c>
+      <c r="D53" s="16" t="n"/>
+      <c r="E53" s="16" t="n"/>
+      <c r="F53" s="16" t="n"/>
+      <c r="G53" s="16" t="n"/>
+      <c r="H53" s="16" t="n"/>
+      <c r="I53" s="16" t="n"/>
+      <c r="J53" s="16" t="n"/>
+      <c r="K53" s="16" t="n"/>
+      <c r="L53" s="16" t="n"/>
+      <c r="M53" s="16" t="n"/>
+      <c r="N53" s="16" t="n"/>
+      <c r="O53" s="16" t="n"/>
+      <c r="P53" s="16" t="n"/>
+      <c r="Q53" s="16" t="n"/>
+      <c r="R53" s="16" t="n"/>
+      <c r="S53" s="16" t="n"/>
+      <c r="T53" s="16" t="n"/>
+      <c r="U53" s="16" t="n"/>
+      <c r="V53" s="16" t="n"/>
+      <c r="W53" s="16" t="n"/>
+      <c r="X53" s="16" t="n"/>
+      <c r="Y53" s="16" t="n"/>
+      <c r="Z53" s="16" t="n"/>
+      <c r="AA53" s="16" t="n"/>
       <c r="AC53" s="23" t="n"/>
     </row>
     <row r="54" ht="20.1" customHeight="1" s="1">
       <c r="B54" s="18" t="n"/>
       <c r="C54" s="19" t="inlineStr">
         <is>
-          <t>Casos de uso y diagramas alineados con Walmart</t>
+          <t>Registro de requisitos y plazos del curso</t>
         </is>
       </c>
       <c r="D54" s="19" t="inlineStr">
@@ -2974,7 +2974,7 @@
       </c>
       <c r="H54" s="21" t="inlineStr">
         <is>
-          <t>#30</t>
+          <t>#23, #25</t>
         </is>
       </c>
       <c r="I54" s="22" t="n"/>
@@ -3002,19 +3002,19 @@
       <c r="B55" s="18" t="n"/>
       <c r="C55" s="19" t="inlineStr">
         <is>
-          <t>Plan de mejoras de la Fase 1</t>
+          <t>Casos de uso y diagramas alineados con Walmart</t>
         </is>
       </c>
       <c r="D55" s="19" t="inlineStr">
         <is>
-          <t>Mariana</t>
+          <t>Francisco</t>
         </is>
       </c>
       <c r="E55" s="20" t="n">
-        <v>46315</v>
+        <v>46304</v>
       </c>
       <c r="F55" s="20" t="n">
-        <v>46315</v>
+        <v>46305</v>
       </c>
       <c r="G55" s="19" t="inlineStr">
         <is>
@@ -3023,7 +3023,7 @@
       </c>
       <c r="H55" s="21" t="inlineStr">
         <is>
-          <t>#26</t>
+          <t>#30</t>
         </is>
       </c>
       <c r="I55" s="22" t="n"/>
@@ -3055,28 +3055,28 @@
       <c r="B56" s="18" t="n"/>
       <c r="C56" s="19" t="inlineStr">
         <is>
-          <t>Informe intermedio: estado de avance y conclusiones</t>
+          <t>Plan de mejoras de la Fase 1</t>
         </is>
       </c>
       <c r="D56" s="19" t="inlineStr">
         <is>
-          <t>Francisco</t>
+          <t>Mariana</t>
         </is>
       </c>
       <c r="E56" s="20" t="n">
-        <v>46314</v>
+        <v>46315</v>
       </c>
       <c r="F56" s="20" t="n">
-        <v>46316</v>
+        <v>46315</v>
       </c>
       <c r="G56" s="19" t="inlineStr">
         <is>
-          <t>En curso</t>
+          <t>Cumplido</t>
         </is>
       </c>
       <c r="H56" s="21" t="inlineStr">
         <is>
-          <t>#27</t>
+          <t>#26</t>
         </is>
       </c>
       <c r="I56" s="22" t="n"/>
@@ -3108,7 +3108,7 @@
       <c r="B57" s="18" t="n"/>
       <c r="C57" s="19" t="inlineStr">
         <is>
-          <t>Análisis de resultados: 10 mejores y 10 peores casos</t>
+          <t>Informe intermedio: estado de avance y conclusiones</t>
         </is>
       </c>
       <c r="D57" s="19" t="inlineStr">
@@ -3117,10 +3117,10 @@
         </is>
       </c>
       <c r="E57" s="20" t="n">
-        <v>46315</v>
+        <v>46314</v>
       </c>
       <c r="F57" s="20" t="n">
-        <v>46315</v>
+        <v>46316</v>
       </c>
       <c r="G57" s="19" t="inlineStr">
         <is>
@@ -3129,7 +3129,7 @@
       </c>
       <c r="H57" s="21" t="inlineStr">
         <is>
-          <t>#34</t>
+          <t>#27</t>
         </is>
       </c>
       <c r="I57" s="22" t="n"/>
@@ -3157,7 +3157,7 @@
       <c r="B58" s="18" t="n"/>
       <c r="C58" s="19" t="inlineStr">
         <is>
-          <t>README completo</t>
+          <t>Análisis de resultados: 10 mejores y 10 peores casos</t>
         </is>
       </c>
       <c r="D58" s="19" t="inlineStr">
@@ -3178,7 +3178,7 @@
       </c>
       <c r="H58" s="21" t="inlineStr">
         <is>
-          <t>#35</t>
+          <t>#34</t>
         </is>
       </c>
       <c r="I58" s="22" t="n"/>
@@ -3206,28 +3206,28 @@
       <c r="B59" s="18" t="n"/>
       <c r="C59" s="19" t="inlineStr">
         <is>
-          <t>Video de demostración (5 a 10 min)</t>
+          <t>README completo</t>
         </is>
       </c>
       <c r="D59" s="19" t="inlineStr">
         <is>
-          <t>Nicko</t>
+          <t>Francisco</t>
         </is>
       </c>
       <c r="E59" s="20" t="n">
-        <v>46316</v>
+        <v>46315</v>
       </c>
       <c r="F59" s="20" t="n">
-        <v>46316</v>
+        <v>46315</v>
       </c>
       <c r="G59" s="19" t="inlineStr">
         <is>
-          <t>Pendiente</t>
+          <t>Cumplido</t>
         </is>
       </c>
       <c r="H59" s="21" t="inlineStr">
         <is>
-          <t>#36</t>
+          <t>#35</t>
         </is>
       </c>
       <c r="I59" s="22" t="n"/>
@@ -3255,28 +3255,28 @@
       <c r="B60" s="18" t="n"/>
       <c r="C60" s="19" t="inlineStr">
         <is>
-          <t>Evidencias de avance: diario 2.1 y guía 2.4</t>
+          <t>Video de demostración (5 a 10 min)</t>
         </is>
       </c>
       <c r="D60" s="19" t="inlineStr">
         <is>
-          <t>Mariana</t>
+          <t>Nicko</t>
         </is>
       </c>
       <c r="E60" s="20" t="n">
-        <v>46315</v>
+        <v>46316</v>
       </c>
       <c r="F60" s="20" t="n">
-        <v>46321</v>
+        <v>46316</v>
       </c>
       <c r="G60" s="19" t="inlineStr">
         <is>
-          <t>En curso</t>
+          <t>Pendiente</t>
         </is>
       </c>
       <c r="H60" s="21" t="inlineStr">
         <is>
-          <t>#37</t>
+          <t>#36</t>
         </is>
       </c>
       <c r="I60" s="22" t="n"/>
@@ -3308,7 +3308,7 @@
       <c r="B61" s="18" t="n"/>
       <c r="C61" s="19" t="inlineStr">
         <is>
-          <t>Rehacer plantillas de C.U y diagramas según la app Django</t>
+          <t>Evidencias de avance: diario 2.1 y guía 2.4</t>
         </is>
       </c>
       <c r="D61" s="19" t="inlineStr">
@@ -3317,19 +3317,19 @@
         </is>
       </c>
       <c r="E61" s="20" t="n">
-        <v>46316</v>
+        <v>46315</v>
       </c>
       <c r="F61" s="20" t="n">
-        <v>46316</v>
+        <v>46321</v>
       </c>
       <c r="G61" s="19" t="inlineStr">
         <is>
-          <t>Cumplido</t>
+          <t>En curso</t>
         </is>
       </c>
       <c r="H61" s="21" t="inlineStr">
         <is>
-          <t>#42</t>
+          <t>#37</t>
         </is>
       </c>
       <c r="I61" s="22" t="n"/>
@@ -3358,82 +3358,86 @@
       </c>
     </row>
     <row r="62" ht="20.1" customHeight="1" s="1">
-      <c r="B62" s="16" t="n"/>
-      <c r="C62" s="17" t="inlineStr">
-        <is>
-          <t>HITOS DEL CURSO</t>
-        </is>
-      </c>
-      <c r="D62" s="16" t="n"/>
-      <c r="E62" s="16" t="n"/>
-      <c r="F62" s="16" t="n"/>
-      <c r="G62" s="16" t="n"/>
-      <c r="H62" s="16" t="n"/>
-      <c r="I62" s="16" t="n"/>
-      <c r="J62" s="16" t="n"/>
-      <c r="K62" s="16" t="n"/>
-      <c r="L62" s="16" t="n"/>
-      <c r="M62" s="16" t="n"/>
-      <c r="N62" s="16" t="n"/>
-      <c r="O62" s="16" t="n"/>
-      <c r="P62" s="16" t="n"/>
-      <c r="Q62" s="16" t="n"/>
-      <c r="R62" s="16" t="n"/>
-      <c r="S62" s="16" t="n"/>
-      <c r="T62" s="16" t="n"/>
-      <c r="U62" s="16" t="n"/>
-      <c r="V62" s="16" t="n"/>
-      <c r="W62" s="16" t="n"/>
-      <c r="X62" s="16" t="n"/>
-      <c r="Y62" s="16" t="n"/>
-      <c r="Z62" s="16" t="n"/>
-      <c r="AA62" s="16" t="n"/>
+      <c r="B62" s="18" t="n"/>
+      <c r="C62" s="19" t="inlineStr">
+        <is>
+          <t>Rehacer plantillas de C.U y diagramas según la app Django</t>
+        </is>
+      </c>
+      <c r="D62" s="19" t="inlineStr">
+        <is>
+          <t>Mariana</t>
+        </is>
+      </c>
+      <c r="E62" s="20" t="n">
+        <v>46316</v>
+      </c>
+      <c r="F62" s="20" t="n">
+        <v>46316</v>
+      </c>
+      <c r="G62" s="19" t="inlineStr">
+        <is>
+          <t>Cumplido</t>
+        </is>
+      </c>
+      <c r="H62" s="21" t="inlineStr">
+        <is>
+          <t>#42</t>
+        </is>
+      </c>
+      <c r="I62" s="22" t="n"/>
+      <c r="J62" s="22" t="n"/>
+      <c r="K62" s="22" t="n"/>
+      <c r="L62" s="22" t="n"/>
+      <c r="M62" s="22" t="n"/>
+      <c r="N62" s="22" t="n"/>
+      <c r="O62" s="22" t="n"/>
+      <c r="P62" s="22" t="n"/>
+      <c r="Q62" s="22" t="n"/>
+      <c r="R62" s="22" t="n"/>
+      <c r="S62" s="22" t="n"/>
+      <c r="T62" s="22" t="n"/>
+      <c r="U62" s="22" t="n"/>
+      <c r="V62" s="22" t="n"/>
+      <c r="W62" s="22" t="n"/>
+      <c r="X62" s="22" t="n"/>
+      <c r="Y62" s="22" t="n"/>
+      <c r="Z62" s="22" t="n"/>
+      <c r="AA62" s="22" t="n"/>
       <c r="AB62" s="16" t="n"/>
       <c r="AC62" s="16" t="n"/>
     </row>
     <row r="63" ht="20.1" customHeight="1" s="1">
-      <c r="B63" s="18" t="n"/>
-      <c r="C63" s="19" t="inlineStr">
-        <is>
-          <t>Informe intermedio y video</t>
-        </is>
-      </c>
-      <c r="D63" s="19" t="inlineStr">
-        <is>
-          <t>Equipo</t>
-        </is>
-      </c>
-      <c r="E63" s="20" t="n">
-        <v>46316</v>
-      </c>
-      <c r="F63" s="20" t="n">
-        <v>46316</v>
-      </c>
-      <c r="G63" s="19" t="inlineStr">
-        <is>
-          <t>En curso</t>
-        </is>
-      </c>
-      <c r="H63" s="21" t="n"/>
-      <c r="I63" s="22" t="n"/>
-      <c r="J63" s="22" t="n"/>
-      <c r="K63" s="22" t="n"/>
-      <c r="L63" s="22" t="n"/>
-      <c r="M63" s="22" t="n"/>
-      <c r="N63" s="22" t="n"/>
-      <c r="O63" s="22" t="n"/>
-      <c r="P63" s="22" t="n"/>
-      <c r="Q63" s="22" t="n"/>
-      <c r="R63" s="22" t="n"/>
-      <c r="S63" s="22" t="n"/>
-      <c r="T63" s="22" t="n"/>
-      <c r="U63" s="22" t="n"/>
-      <c r="V63" s="22" t="n"/>
-      <c r="W63" s="22" t="n"/>
-      <c r="X63" s="22" t="n"/>
-      <c r="Y63" s="22" t="n"/>
-      <c r="Z63" s="22" t="n"/>
-      <c r="AA63" s="22" t="n"/>
+      <c r="B63" s="16" t="n"/>
+      <c r="C63" s="17" t="inlineStr">
+        <is>
+          <t>HITOS DEL CURSO</t>
+        </is>
+      </c>
+      <c r="D63" s="16" t="n"/>
+      <c r="E63" s="16" t="n"/>
+      <c r="F63" s="16" t="n"/>
+      <c r="G63" s="16" t="n"/>
+      <c r="H63" s="16" t="n"/>
+      <c r="I63" s="16" t="n"/>
+      <c r="J63" s="16" t="n"/>
+      <c r="K63" s="16" t="n"/>
+      <c r="L63" s="16" t="n"/>
+      <c r="M63" s="16" t="n"/>
+      <c r="N63" s="16" t="n"/>
+      <c r="O63" s="16" t="n"/>
+      <c r="P63" s="16" t="n"/>
+      <c r="Q63" s="16" t="n"/>
+      <c r="R63" s="16" t="n"/>
+      <c r="S63" s="16" t="n"/>
+      <c r="T63" s="16" t="n"/>
+      <c r="U63" s="16" t="n"/>
+      <c r="V63" s="16" t="n"/>
+      <c r="W63" s="16" t="n"/>
+      <c r="X63" s="16" t="n"/>
+      <c r="Y63" s="16" t="n"/>
+      <c r="Z63" s="16" t="n"/>
+      <c r="AA63" s="16" t="n"/>
       <c r="AC63" s="23" t="inlineStr">
         <is>
           <t>Entrega 2026-10-21</t>
@@ -3444,30 +3448,26 @@
       <c r="B64" s="18" t="n"/>
       <c r="C64" s="19" t="inlineStr">
         <is>
-          <t>Feria de informática</t>
+          <t>Informe intermedio y video</t>
         </is>
       </c>
       <c r="D64" s="19" t="inlineStr">
         <is>
-          <t>Nicko</t>
+          <t>Equipo</t>
         </is>
       </c>
       <c r="E64" s="20" t="n">
-        <v>46321</v>
+        <v>46316</v>
       </c>
       <c r="F64" s="20" t="n">
-        <v>46325</v>
+        <v>46316</v>
       </c>
       <c r="G64" s="19" t="inlineStr">
         <is>
-          <t>Pendiente</t>
-        </is>
-      </c>
-      <c r="H64" s="21" t="inlineStr">
-        <is>
-          <t>#38</t>
-        </is>
-      </c>
+          <t>En curso</t>
+        </is>
+      </c>
+      <c r="H64" s="21" t="n"/>
       <c r="I64" s="22" t="n"/>
       <c r="J64" s="22" t="n"/>
       <c r="K64" s="22" t="n"/>
@@ -3497,16 +3497,16 @@
       <c r="B65" s="18" t="n"/>
       <c r="C65" s="19" t="inlineStr">
         <is>
-          <t>Evaluación 2 (Avance): 50% de los C.U y demo del Sprint 1</t>
+          <t>Feria de informática</t>
         </is>
       </c>
       <c r="D65" s="19" t="inlineStr">
         <is>
-          <t>Equipo</t>
+          <t>Nicko</t>
         </is>
       </c>
       <c r="E65" s="20" t="n">
-        <v>46323</v>
+        <v>46321</v>
       </c>
       <c r="F65" s="20" t="n">
         <v>46325</v>
@@ -3516,7 +3516,11 @@
           <t>Pendiente</t>
         </is>
       </c>
-      <c r="H65" s="21" t="n"/>
+      <c r="H65" s="21" t="inlineStr">
+        <is>
+          <t>#38</t>
+        </is>
+      </c>
       <c r="I65" s="22" t="n"/>
       <c r="J65" s="22" t="n"/>
       <c r="K65" s="22" t="n"/>
@@ -3546,7 +3550,7 @@
       <c r="B66" s="18" t="n"/>
       <c r="C66" s="19" t="inlineStr">
         <is>
-          <t>Entrega final de la Fase 2</t>
+          <t>Evaluación 2 (Avance): 50% de los C.U y demo del Sprint 1</t>
         </is>
       </c>
       <c r="D66" s="19" t="inlineStr">
@@ -3555,10 +3559,10 @@
         </is>
       </c>
       <c r="E66" s="20" t="n">
-        <v>46349</v>
+        <v>46323</v>
       </c>
       <c r="F66" s="20" t="n">
-        <v>46353</v>
+        <v>46325</v>
       </c>
       <c r="G66" s="19" t="inlineStr">
         <is>
@@ -3592,89 +3596,132 @@
       </c>
     </row>
     <row r="67" ht="20.1" customHeight="1" s="1">
-      <c r="B67" s="16" t="n"/>
-      <c r="C67" s="17" t="inlineStr">
-        <is>
-          <t>FASE 3</t>
-        </is>
-      </c>
-      <c r="D67" s="16" t="n"/>
-      <c r="E67" s="16" t="n"/>
-      <c r="F67" s="16" t="n"/>
-      <c r="G67" s="16" t="n"/>
-      <c r="H67" s="16" t="n"/>
-      <c r="I67" s="16" t="n"/>
-      <c r="J67" s="16" t="n"/>
-      <c r="K67" s="16" t="n"/>
-      <c r="L67" s="16" t="n"/>
-      <c r="M67" s="16" t="n"/>
-      <c r="N67" s="16" t="n"/>
-      <c r="O67" s="16" t="n"/>
-      <c r="P67" s="16" t="n"/>
-      <c r="Q67" s="16" t="n"/>
-      <c r="R67" s="16" t="n"/>
-      <c r="S67" s="16" t="n"/>
-      <c r="T67" s="16" t="n"/>
-      <c r="U67" s="16" t="n"/>
-      <c r="V67" s="16" t="n"/>
-      <c r="W67" s="16" t="n"/>
-      <c r="X67" s="16" t="n"/>
-      <c r="Y67" s="16" t="n"/>
-      <c r="Z67" s="16" t="n"/>
-      <c r="AA67" s="16" t="n"/>
+      <c r="B67" s="18" t="n"/>
+      <c r="C67" s="19" t="inlineStr">
+        <is>
+          <t>Entrega final de la Fase 2</t>
+        </is>
+      </c>
+      <c r="D67" s="19" t="inlineStr">
+        <is>
+          <t>Equipo</t>
+        </is>
+      </c>
+      <c r="E67" s="20" t="n">
+        <v>46349</v>
+      </c>
+      <c r="F67" s="20" t="n">
+        <v>46353</v>
+      </c>
+      <c r="G67" s="19" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="H67" s="21" t="n"/>
+      <c r="I67" s="22" t="n"/>
+      <c r="J67" s="22" t="n"/>
+      <c r="K67" s="22" t="n"/>
+      <c r="L67" s="22" t="n"/>
+      <c r="M67" s="22" t="n"/>
+      <c r="N67" s="22" t="n"/>
+      <c r="O67" s="22" t="n"/>
+      <c r="P67" s="22" t="n"/>
+      <c r="Q67" s="22" t="n"/>
+      <c r="R67" s="22" t="n"/>
+      <c r="S67" s="22" t="n"/>
+      <c r="T67" s="22" t="n"/>
+      <c r="U67" s="22" t="n"/>
+      <c r="V67" s="22" t="n"/>
+      <c r="W67" s="22" t="n"/>
+      <c r="X67" s="22" t="n"/>
+      <c r="Y67" s="22" t="n"/>
+      <c r="Z67" s="22" t="n"/>
+      <c r="AA67" s="22" t="n"/>
       <c r="AB67" s="16" t="n"/>
       <c r="AC67" s="16" t="n"/>
     </row>
     <row r="68" ht="20.1" customHeight="1" s="1">
-      <c r="B68" s="18" t="n"/>
-      <c r="C68" s="19" t="inlineStr">
+      <c r="B68" s="16" t="n"/>
+      <c r="C68" s="17" t="inlineStr">
+        <is>
+          <t>FASE 3</t>
+        </is>
+      </c>
+      <c r="D68" s="16" t="n"/>
+      <c r="E68" s="16" t="n"/>
+      <c r="F68" s="16" t="n"/>
+      <c r="G68" s="16" t="n"/>
+      <c r="H68" s="16" t="n"/>
+      <c r="I68" s="16" t="n"/>
+      <c r="J68" s="16" t="n"/>
+      <c r="K68" s="16" t="n"/>
+      <c r="L68" s="16" t="n"/>
+      <c r="M68" s="16" t="n"/>
+      <c r="N68" s="16" t="n"/>
+      <c r="O68" s="16" t="n"/>
+      <c r="P68" s="16" t="n"/>
+      <c r="Q68" s="16" t="n"/>
+      <c r="R68" s="16" t="n"/>
+      <c r="S68" s="16" t="n"/>
+      <c r="T68" s="16" t="n"/>
+      <c r="U68" s="16" t="n"/>
+      <c r="V68" s="16" t="n"/>
+      <c r="W68" s="16" t="n"/>
+      <c r="X68" s="16" t="n"/>
+      <c r="Y68" s="16" t="n"/>
+      <c r="Z68" s="16" t="n"/>
+      <c r="AA68" s="16" t="n"/>
+      <c r="AC68" s="23" t="inlineStr">
+        <is>
+          <t>Fechas por definir</t>
+        </is>
+      </c>
+    </row>
+    <row r="69" ht="15.75" customHeight="1" s="1">
+      <c r="B69" s="18" t="n"/>
+      <c r="C69" s="19" t="inlineStr">
         <is>
           <t>Ajustes finales, manuales y exposición ante la Comisión</t>
         </is>
       </c>
-      <c r="D68" s="19" t="inlineStr">
+      <c r="D69" s="19" t="inlineStr">
         <is>
           <t>Equipo</t>
         </is>
       </c>
-      <c r="E68" s="20" t="n">
+      <c r="E69" s="20" t="n">
         <v>46356</v>
       </c>
-      <c r="F68" s="20" t="n">
+      <c r="F69" s="20" t="n">
         <v>46374</v>
       </c>
-      <c r="G68" s="19" t="inlineStr">
+      <c r="G69" s="19" t="inlineStr">
         <is>
           <t>Pendiente</t>
         </is>
       </c>
-      <c r="H68" s="21" t="n"/>
-      <c r="I68" s="22" t="n"/>
-      <c r="J68" s="22" t="n"/>
-      <c r="K68" s="22" t="n"/>
-      <c r="L68" s="22" t="n"/>
-      <c r="M68" s="22" t="n"/>
-      <c r="N68" s="22" t="n"/>
-      <c r="O68" s="22" t="n"/>
-      <c r="P68" s="22" t="n"/>
-      <c r="Q68" s="22" t="n"/>
-      <c r="R68" s="22" t="n"/>
-      <c r="S68" s="22" t="n"/>
-      <c r="T68" s="22" t="n"/>
-      <c r="U68" s="22" t="n"/>
-      <c r="V68" s="22" t="n"/>
-      <c r="W68" s="22" t="n"/>
-      <c r="X68" s="22" t="n"/>
-      <c r="Y68" s="22" t="n"/>
-      <c r="Z68" s="22" t="n"/>
-      <c r="AA68" s="22" t="n"/>
-      <c r="AC68" s="23" t="inlineStr">
-        <is>
-          <t>Fechas por definir</t>
-        </is>
-      </c>
-    </row>
-    <row r="69" ht="15.75" customHeight="1" s="1"/>
+      <c r="H69" s="21" t="n"/>
+      <c r="I69" s="22" t="n"/>
+      <c r="J69" s="22" t="n"/>
+      <c r="K69" s="22" t="n"/>
+      <c r="L69" s="22" t="n"/>
+      <c r="M69" s="22" t="n"/>
+      <c r="N69" s="22" t="n"/>
+      <c r="O69" s="22" t="n"/>
+      <c r="P69" s="22" t="n"/>
+      <c r="Q69" s="22" t="n"/>
+      <c r="R69" s="22" t="n"/>
+      <c r="S69" s="22" t="n"/>
+      <c r="T69" s="22" t="n"/>
+      <c r="U69" s="22" t="n"/>
+      <c r="V69" s="22" t="n"/>
+      <c r="W69" s="22" t="n"/>
+      <c r="X69" s="22" t="n"/>
+      <c r="Y69" s="22" t="n"/>
+      <c r="Z69" s="22" t="n"/>
+      <c r="AA69" s="22" t="n"/>
+    </row>
     <row r="70" ht="15.75" customHeight="1" s="1"/>
     <row r="71" ht="15.75" customHeight="1" s="1"/>
     <row r="72" ht="15.75" customHeight="1" s="1"/>
@@ -4617,7 +4664,7 @@
     <mergeCell ref="Q8:T8"/>
     <mergeCell ref="I8:L8"/>
   </mergeCells>
-  <conditionalFormatting sqref="B10:B68">
+  <conditionalFormatting sqref="B10:B69">
     <cfRule type="expression" priority="2" dxfId="5" stopIfTrue="1">
       <formula>$G10="Cumplido"</formula>
     </cfRule>
@@ -4634,7 +4681,7 @@
       <formula>$G10="Bloqueado"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="I10:AA68">
+  <conditionalFormatting sqref="I10:AA69">
     <cfRule type="expression" priority="1" dxfId="5" stopIfTrue="1">
       <formula>AND($E10&lt;&gt;"",I$9&lt;=$F10,I$9+6&gt;=$E10,$G10="Cumplido")</formula>
     </cfRule>
@@ -4651,7 +4698,7 @@
       <formula>AND($E10&lt;&gt;"",I$9&lt;=$F10,I$9+6&gt;=$E10,$G10="Bloqueado")</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="S10:S68">
+  <conditionalFormatting sqref="S10:S69">
     <cfRule type="expression" priority="11" dxfId="0">
       <formula>$G10&lt;&gt;""</formula>
     </cfRule>

</xml_diff>

<commit_message>
fix: la app web arranca segura por defecto (debug apagado, HTTPS y contenedor sin root) (#50)
Pasa #49, #51 y #54 a Mariana en el backlog y en la Carta Gantt.
</commit_message>
<xml_diff>
--- a/Anexos/Gestion/Carta Gantt Fase 2.xlsx
+++ b/Anexos/Gestion/Carta Gantt Fase 2.xlsx
@@ -655,7 +655,7 @@
     <outlinePr summaryBelow="0" summaryRight="0"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:AC69"/>
+  <dimension ref="B1:AC69"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="12.5703125" defaultRowHeight="15" customHeight="1"/>
   <cols>
     <col width="2" customWidth="1" style="1" min="1" max="1"/>
@@ -2724,7 +2724,7 @@
       </c>
       <c r="D49" s="19" t="inlineStr">
         <is>
-          <t>Francisco</t>
+          <t>Mariana</t>
         </is>
       </c>
       <c r="E49" s="20" t="n">

</xml_diff>

<commit_message>
docs: link the technical specification and mark #9 done
</commit_message>
<xml_diff>
--- a/Anexos/Gestion/Carta Gantt Fase 2.xlsx
+++ b/Anexos/Gestion/Carta Gantt Fase 2.xlsx
@@ -655,7 +655,7 @@
     <outlinePr summaryBelow="0" summaryRight="0"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:AC69"/>
+  <dimension ref="A1:AC70"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="12.5703125" defaultRowHeight="15" customHeight="1"/>
   <cols>
     <col width="2" customWidth="1" style="1" min="1" max="1"/>
@@ -695,23 +695,23 @@
     <row r="4" ht="15.75" customHeight="1" s="1"/>
     <row r="5" ht="26.1" customHeight="1" s="1">
       <c r="D5" s="5">
-        <f>COUNTIF($G$10:$G$69,"Cumplido")</f>
+        <f>COUNTIF($G$10:$G$70,"Cumplido")</f>
         <v/>
       </c>
       <c r="E5" s="6">
-        <f>COUNTIF($G$10:$G$69,"En curso")</f>
+        <f>COUNTIF($G$10:$G$70,"En curso")</f>
         <v/>
       </c>
       <c r="F5" s="7">
-        <f>COUNTIF($G$10:$G$69,"Pendiente")</f>
+        <f>COUNTIF($G$10:$G$70,"Pendiente")</f>
         <v/>
       </c>
       <c r="G5" s="8">
-        <f>COUNTIF($G$10:$G$69,"Atrasado")</f>
+        <f>COUNTIF($G$10:$G$70,"Atrasado")</f>
         <v/>
       </c>
       <c r="H5" s="9">
-        <f>COUNTIF($G$10:$G$69,"Bloqueado")</f>
+        <f>COUNTIF($G$10:$G$70,"Bloqueado")</f>
         <v/>
       </c>
     </row>
@@ -3408,88 +3408,93 @@
       <c r="AC62" s="16" t="n"/>
     </row>
     <row r="63" ht="20.1" customHeight="1" s="1">
-      <c r="B63" s="16" t="n"/>
-      <c r="C63" s="17" t="inlineStr">
+      <c r="B63" s="18" t="n"/>
+      <c r="C63" s="19" t="inlineStr">
+        <is>
+          <t>Especificación técnica del sistema</t>
+        </is>
+      </c>
+      <c r="D63" s="19" t="inlineStr">
+        <is>
+          <t>Mariana</t>
+        </is>
+      </c>
+      <c r="E63" s="20">
+        <v>46317</v>
+      </c>
+      <c r="F63" s="20">
+        <v>46317</v>
+      </c>
+      <c r="G63" s="19" t="inlineStr">
+        <is>
+          <t>Cumplido</t>
+        </is>
+      </c>
+      <c r="H63" s="21" t="inlineStr">
+        <is>
+          <t>#9</t>
+        </is>
+      </c>
+      <c r="I63" s="22" t="n"/>
+      <c r="J63" s="22" t="n"/>
+      <c r="K63" s="22" t="n"/>
+      <c r="L63" s="22" t="n"/>
+      <c r="M63" s="22" t="n"/>
+      <c r="N63" s="22" t="n"/>
+      <c r="O63" s="22" t="n"/>
+      <c r="P63" s="22" t="n"/>
+      <c r="Q63" s="22" t="n"/>
+      <c r="R63" s="22" t="n"/>
+      <c r="S63" s="22" t="n"/>
+      <c r="T63" s="22" t="n"/>
+      <c r="U63" s="22" t="n"/>
+      <c r="V63" s="22" t="n"/>
+      <c r="W63" s="22" t="n"/>
+      <c r="X63" s="22" t="n"/>
+      <c r="Y63" s="22" t="n"/>
+      <c r="Z63" s="22" t="n"/>
+      <c r="AA63" s="22" t="n"/>
+      <c r="AB63" s="16" t="n"/>
+      <c r="AC63" s="16" t="inlineStr">
+        <is>
+          <t>docs/especificacion-tecnica.md, sacada del código</t>
+        </is>
+      </c>
+    </row>
+    <row r="64" ht="20.1" customHeight="1" s="1">
+      <c r="B64" s="16" t="n"/>
+      <c r="C64" s="17" t="inlineStr">
         <is>
           <t>HITOS DEL CURSO</t>
         </is>
       </c>
-      <c r="D63" s="16" t="n"/>
-      <c r="E63" s="16" t="n"/>
-      <c r="F63" s="16" t="n"/>
-      <c r="G63" s="16" t="n"/>
-      <c r="H63" s="16" t="n"/>
-      <c r="I63" s="16" t="n"/>
-      <c r="J63" s="16" t="n"/>
-      <c r="K63" s="16" t="n"/>
-      <c r="L63" s="16" t="n"/>
-      <c r="M63" s="16" t="n"/>
-      <c r="N63" s="16" t="n"/>
-      <c r="O63" s="16" t="n"/>
-      <c r="P63" s="16" t="n"/>
-      <c r="Q63" s="16" t="n"/>
-      <c r="R63" s="16" t="n"/>
-      <c r="S63" s="16" t="n"/>
-      <c r="T63" s="16" t="n"/>
-      <c r="U63" s="16" t="n"/>
-      <c r="V63" s="16" t="n"/>
-      <c r="W63" s="16" t="n"/>
-      <c r="X63" s="16" t="n"/>
-      <c r="Y63" s="16" t="n"/>
-      <c r="Z63" s="16" t="n"/>
-      <c r="AA63" s="16" t="n"/>
-      <c r="AC63" s="23" t="inlineStr">
+      <c r="D64" s="16" t="n"/>
+      <c r="E64" s="16" t="n"/>
+      <c r="F64" s="16" t="n"/>
+      <c r="G64" s="16" t="n"/>
+      <c r="H64" s="16" t="n"/>
+      <c r="I64" s="16" t="n"/>
+      <c r="J64" s="16" t="n"/>
+      <c r="K64" s="16" t="n"/>
+      <c r="L64" s="16" t="n"/>
+      <c r="M64" s="16" t="n"/>
+      <c r="N64" s="16" t="n"/>
+      <c r="O64" s="16" t="n"/>
+      <c r="P64" s="16" t="n"/>
+      <c r="Q64" s="16" t="n"/>
+      <c r="R64" s="16" t="n"/>
+      <c r="S64" s="16" t="n"/>
+      <c r="T64" s="16" t="n"/>
+      <c r="U64" s="16" t="n"/>
+      <c r="V64" s="16" t="n"/>
+      <c r="W64" s="16" t="n"/>
+      <c r="X64" s="16" t="n"/>
+      <c r="Y64" s="16" t="n"/>
+      <c r="Z64" s="16" t="n"/>
+      <c r="AA64" s="16" t="n"/>
+      <c r="AC64" s="23" t="inlineStr">
         <is>
           <t>Entrega 2026-10-21</t>
-        </is>
-      </c>
-    </row>
-    <row r="64" ht="20.1" customHeight="1" s="1">
-      <c r="B64" s="18" t="n"/>
-      <c r="C64" s="19" t="inlineStr">
-        <is>
-          <t>Informe intermedio y video</t>
-        </is>
-      </c>
-      <c r="D64" s="19" t="inlineStr">
-        <is>
-          <t>Equipo</t>
-        </is>
-      </c>
-      <c r="E64" s="20" t="n">
-        <v>46316</v>
-      </c>
-      <c r="F64" s="20" t="n">
-        <v>46316</v>
-      </c>
-      <c r="G64" s="19" t="inlineStr">
-        <is>
-          <t>En curso</t>
-        </is>
-      </c>
-      <c r="H64" s="21" t="n"/>
-      <c r="I64" s="22" t="n"/>
-      <c r="J64" s="22" t="n"/>
-      <c r="K64" s="22" t="n"/>
-      <c r="L64" s="22" t="n"/>
-      <c r="M64" s="22" t="n"/>
-      <c r="N64" s="22" t="n"/>
-      <c r="O64" s="22" t="n"/>
-      <c r="P64" s="22" t="n"/>
-      <c r="Q64" s="22" t="n"/>
-      <c r="R64" s="22" t="n"/>
-      <c r="S64" s="22" t="n"/>
-      <c r="T64" s="22" t="n"/>
-      <c r="U64" s="22" t="n"/>
-      <c r="V64" s="22" t="n"/>
-      <c r="W64" s="22" t="n"/>
-      <c r="X64" s="22" t="n"/>
-      <c r="Y64" s="22" t="n"/>
-      <c r="Z64" s="22" t="n"/>
-      <c r="AA64" s="22" t="n"/>
-      <c r="AC64" s="23" t="inlineStr">
-        <is>
-          <t>Día y hora por informar</t>
         </is>
       </c>
     </row>
@@ -3497,30 +3502,26 @@
       <c r="B65" s="18" t="n"/>
       <c r="C65" s="19" t="inlineStr">
         <is>
-          <t>Feria de informática</t>
+          <t>Informe intermedio y video</t>
         </is>
       </c>
       <c r="D65" s="19" t="inlineStr">
         <is>
-          <t>Nicko</t>
+          <t>Equipo</t>
         </is>
       </c>
       <c r="E65" s="20" t="n">
-        <v>46321</v>
+        <v>46316</v>
       </c>
       <c r="F65" s="20" t="n">
-        <v>46325</v>
+        <v>46316</v>
       </c>
       <c r="G65" s="19" t="inlineStr">
         <is>
-          <t>Pendiente</t>
-        </is>
-      </c>
-      <c r="H65" s="21" t="inlineStr">
-        <is>
-          <t>#38</t>
-        </is>
-      </c>
+          <t>En curso</t>
+        </is>
+      </c>
+      <c r="H65" s="21" t="n"/>
       <c r="I65" s="22" t="n"/>
       <c r="J65" s="22" t="n"/>
       <c r="K65" s="22" t="n"/>
@@ -3542,7 +3543,7 @@
       <c r="AA65" s="22" t="n"/>
       <c r="AC65" s="23" t="inlineStr">
         <is>
-          <t>Día exacto por confirmar</t>
+          <t>Día y hora por informar</t>
         </is>
       </c>
     </row>
@@ -3550,16 +3551,16 @@
       <c r="B66" s="18" t="n"/>
       <c r="C66" s="19" t="inlineStr">
         <is>
-          <t>Evaluación 2 (Avance): 50% de los C.U y demo del Sprint 1</t>
+          <t>Feria de informática</t>
         </is>
       </c>
       <c r="D66" s="19" t="inlineStr">
         <is>
-          <t>Equipo</t>
+          <t>Nicko</t>
         </is>
       </c>
       <c r="E66" s="20" t="n">
-        <v>46323</v>
+        <v>46321</v>
       </c>
       <c r="F66" s="20" t="n">
         <v>46325</v>
@@ -3569,7 +3570,11 @@
           <t>Pendiente</t>
         </is>
       </c>
-      <c r="H66" s="21" t="n"/>
+      <c r="H66" s="21" t="inlineStr">
+        <is>
+          <t>#38</t>
+        </is>
+      </c>
       <c r="I66" s="22" t="n"/>
       <c r="J66" s="22" t="n"/>
       <c r="K66" s="22" t="n"/>
@@ -3591,7 +3596,7 @@
       <c r="AA66" s="22" t="n"/>
       <c r="AC66" s="23" t="inlineStr">
         <is>
-          <t>Semana 15, por confirmar</t>
+          <t>Día exacto por confirmar</t>
         </is>
       </c>
     </row>
@@ -3599,7 +3604,7 @@
       <c r="B67" s="18" t="n"/>
       <c r="C67" s="19" t="inlineStr">
         <is>
-          <t>Entrega final de la Fase 2</t>
+          <t>Evaluación 2 (Avance): 50% de los C.U y demo del Sprint 1</t>
         </is>
       </c>
       <c r="D67" s="19" t="inlineStr">
@@ -3608,10 +3613,10 @@
         </is>
       </c>
       <c r="E67" s="20" t="n">
-        <v>46349</v>
+        <v>46323</v>
       </c>
       <c r="F67" s="20" t="n">
-        <v>46353</v>
+        <v>46325</v>
       </c>
       <c r="G67" s="19" t="inlineStr">
         <is>
@@ -3638,91 +3643,139 @@
       <c r="Y67" s="22" t="n"/>
       <c r="Z67" s="22" t="n"/>
       <c r="AA67" s="22" t="n"/>
-      <c r="AB67" s="16" t="n"/>
-      <c r="AC67" s="16" t="n"/>
+      <c r="AC67" s="23" t="inlineStr">
+        <is>
+          <t>Semana 15, por confirmar</t>
+        </is>
+      </c>
     </row>
     <row r="68" ht="20.1" customHeight="1" s="1">
-      <c r="B68" s="16" t="n"/>
-      <c r="C68" s="17" t="inlineStr">
+      <c r="B68" s="18" t="n"/>
+      <c r="C68" s="19" t="inlineStr">
+        <is>
+          <t>Entrega final de la Fase 2</t>
+        </is>
+      </c>
+      <c r="D68" s="19" t="inlineStr">
+        <is>
+          <t>Equipo</t>
+        </is>
+      </c>
+      <c r="E68" s="20" t="n">
+        <v>46349</v>
+      </c>
+      <c r="F68" s="20" t="n">
+        <v>46353</v>
+      </c>
+      <c r="G68" s="19" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="H68" s="21" t="n"/>
+      <c r="I68" s="22" t="n"/>
+      <c r="J68" s="22" t="n"/>
+      <c r="K68" s="22" t="n"/>
+      <c r="L68" s="22" t="n"/>
+      <c r="M68" s="22" t="n"/>
+      <c r="N68" s="22" t="n"/>
+      <c r="O68" s="22" t="n"/>
+      <c r="P68" s="22" t="n"/>
+      <c r="Q68" s="22" t="n"/>
+      <c r="R68" s="22" t="n"/>
+      <c r="S68" s="22" t="n"/>
+      <c r="T68" s="22" t="n"/>
+      <c r="U68" s="22" t="n"/>
+      <c r="V68" s="22" t="n"/>
+      <c r="W68" s="22" t="n"/>
+      <c r="X68" s="22" t="n"/>
+      <c r="Y68" s="22" t="n"/>
+      <c r="Z68" s="22" t="n"/>
+      <c r="AA68" s="22" t="n"/>
+      <c r="AB68" s="16" t="n"/>
+      <c r="AC68" s="16" t="n"/>
+    </row>
+    <row r="69" ht="20.1" customHeight="1" s="1">
+      <c r="B69" s="16" t="n"/>
+      <c r="C69" s="17" t="inlineStr">
         <is>
           <t>FASE 3</t>
         </is>
       </c>
-      <c r="D68" s="16" t="n"/>
-      <c r="E68" s="16" t="n"/>
-      <c r="F68" s="16" t="n"/>
-      <c r="G68" s="16" t="n"/>
-      <c r="H68" s="16" t="n"/>
-      <c r="I68" s="16" t="n"/>
-      <c r="J68" s="16" t="n"/>
-      <c r="K68" s="16" t="n"/>
-      <c r="L68" s="16" t="n"/>
-      <c r="M68" s="16" t="n"/>
-      <c r="N68" s="16" t="n"/>
-      <c r="O68" s="16" t="n"/>
-      <c r="P68" s="16" t="n"/>
-      <c r="Q68" s="16" t="n"/>
-      <c r="R68" s="16" t="n"/>
-      <c r="S68" s="16" t="n"/>
-      <c r="T68" s="16" t="n"/>
-      <c r="U68" s="16" t="n"/>
-      <c r="V68" s="16" t="n"/>
-      <c r="W68" s="16" t="n"/>
-      <c r="X68" s="16" t="n"/>
-      <c r="Y68" s="16" t="n"/>
-      <c r="Z68" s="16" t="n"/>
-      <c r="AA68" s="16" t="n"/>
-      <c r="AC68" s="23" t="inlineStr">
+      <c r="D69" s="16" t="n"/>
+      <c r="E69" s="16" t="n"/>
+      <c r="F69" s="16" t="n"/>
+      <c r="G69" s="16" t="n"/>
+      <c r="H69" s="16" t="n"/>
+      <c r="I69" s="16" t="n"/>
+      <c r="J69" s="16" t="n"/>
+      <c r="K69" s="16" t="n"/>
+      <c r="L69" s="16" t="n"/>
+      <c r="M69" s="16" t="n"/>
+      <c r="N69" s="16" t="n"/>
+      <c r="O69" s="16" t="n"/>
+      <c r="P69" s="16" t="n"/>
+      <c r="Q69" s="16" t="n"/>
+      <c r="R69" s="16" t="n"/>
+      <c r="S69" s="16" t="n"/>
+      <c r="T69" s="16" t="n"/>
+      <c r="U69" s="16" t="n"/>
+      <c r="V69" s="16" t="n"/>
+      <c r="W69" s="16" t="n"/>
+      <c r="X69" s="16" t="n"/>
+      <c r="Y69" s="16" t="n"/>
+      <c r="Z69" s="16" t="n"/>
+      <c r="AA69" s="16" t="n"/>
+      <c r="AC69" s="23" t="inlineStr">
         <is>
           <t>Fechas por definir</t>
         </is>
       </c>
     </row>
-    <row r="69" ht="15.75" customHeight="1" s="1">
-      <c r="B69" s="18" t="n"/>
-      <c r="C69" s="19" t="inlineStr">
+    <row r="70" ht="15.75" customHeight="1" s="1">
+      <c r="B70" s="18" t="n"/>
+      <c r="C70" s="19" t="inlineStr">
         <is>
           <t>Ajustes finales, manuales y exposición ante la Comisión</t>
         </is>
       </c>
-      <c r="D69" s="19" t="inlineStr">
+      <c r="D70" s="19" t="inlineStr">
         <is>
           <t>Equipo</t>
         </is>
       </c>
-      <c r="E69" s="20" t="n">
+      <c r="E70" s="20" t="n">
         <v>46356</v>
       </c>
-      <c r="F69" s="20" t="n">
+      <c r="F70" s="20" t="n">
         <v>46374</v>
       </c>
-      <c r="G69" s="19" t="inlineStr">
+      <c r="G70" s="19" t="inlineStr">
         <is>
           <t>Pendiente</t>
         </is>
       </c>
-      <c r="H69" s="21" t="n"/>
-      <c r="I69" s="22" t="n"/>
-      <c r="J69" s="22" t="n"/>
-      <c r="K69" s="22" t="n"/>
-      <c r="L69" s="22" t="n"/>
-      <c r="M69" s="22" t="n"/>
-      <c r="N69" s="22" t="n"/>
-      <c r="O69" s="22" t="n"/>
-      <c r="P69" s="22" t="n"/>
-      <c r="Q69" s="22" t="n"/>
-      <c r="R69" s="22" t="n"/>
-      <c r="S69" s="22" t="n"/>
-      <c r="T69" s="22" t="n"/>
-      <c r="U69" s="22" t="n"/>
-      <c r="V69" s="22" t="n"/>
-      <c r="W69" s="22" t="n"/>
-      <c r="X69" s="22" t="n"/>
-      <c r="Y69" s="22" t="n"/>
-      <c r="Z69" s="22" t="n"/>
-      <c r="AA69" s="22" t="n"/>
-    </row>
-    <row r="70" ht="15.75" customHeight="1" s="1"/>
+      <c r="H70" s="21" t="n"/>
+      <c r="I70" s="22" t="n"/>
+      <c r="J70" s="22" t="n"/>
+      <c r="K70" s="22" t="n"/>
+      <c r="L70" s="22" t="n"/>
+      <c r="M70" s="22" t="n"/>
+      <c r="N70" s="22" t="n"/>
+      <c r="O70" s="22" t="n"/>
+      <c r="P70" s="22" t="n"/>
+      <c r="Q70" s="22" t="n"/>
+      <c r="R70" s="22" t="n"/>
+      <c r="S70" s="22" t="n"/>
+      <c r="T70" s="22" t="n"/>
+      <c r="U70" s="22" t="n"/>
+      <c r="V70" s="22" t="n"/>
+      <c r="W70" s="22" t="n"/>
+      <c r="X70" s="22" t="n"/>
+      <c r="Y70" s="22" t="n"/>
+      <c r="Z70" s="22" t="n"/>
+      <c r="AA70" s="22" t="n"/>
+    </row>
     <row r="71" ht="15.75" customHeight="1" s="1"/>
     <row r="72" ht="15.75" customHeight="1" s="1"/>
     <row r="73" ht="15.75" customHeight="1" s="1"/>
@@ -4656,6 +4709,7 @@
     <row r="1001" ht="15.75" customHeight="1" s="1"/>
     <row r="1002" ht="15.75" customHeight="1" s="1"/>
     <row r="1003" ht="15.75" customHeight="1" s="1"/>
+    <row r="1004" ht="15.75" customHeight="1" s="1"/>
   </sheetData>
   <mergeCells count="5">
     <mergeCell ref="U8:Y8"/>
@@ -4664,7 +4718,7 @@
     <mergeCell ref="Q8:T8"/>
     <mergeCell ref="I8:L8"/>
   </mergeCells>
-  <conditionalFormatting sqref="B10:B69">
+  <conditionalFormatting sqref="B10:B70">
     <cfRule type="expression" priority="2" dxfId="5" stopIfTrue="1">
       <formula>$G10="Cumplido"</formula>
     </cfRule>
@@ -4681,7 +4735,7 @@
       <formula>$G10="Bloqueado"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="I10:AA69">
+  <conditionalFormatting sqref="I10:AA70">
     <cfRule type="expression" priority="1" dxfId="5" stopIfTrue="1">
       <formula>AND($E10&lt;&gt;"",I$9&lt;=$F10,I$9+6&gt;=$E10,$G10="Cumplido")</formula>
     </cfRule>
@@ -4698,7 +4752,7 @@
       <formula>AND($E10&lt;&gt;"",I$9&lt;=$F10,I$9+6&gt;=$E10,$G10="Bloqueado")</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="S10:S69">
+  <conditionalFormatting sqref="S10:S70">
     <cfRule type="expression" priority="11" dxfId="0">
       <formula>$G10&lt;&gt;""</formula>
     </cfRule>

</xml_diff>

<commit_message>
docs: documenta el bloqueo por tiempo y marca #51 como hecho
</commit_message>
<xml_diff>
--- a/Anexos/Gestion/Carta Gantt Fase 2.xlsx
+++ b/Anexos/Gestion/Carta Gantt Fase 2.xlsx
@@ -2571,12 +2571,12 @@
       <c r="E46" s="20" t="n">
         <v>46317</v>
       </c>
-      <c r="F46" s="20" t="n">
-        <v>46323</v>
+      <c r="F46" s="20">
+        <v>46318</v>
       </c>
       <c r="G46" s="19" t="inlineStr">
         <is>
-          <t>En curso</t>
+          <t>Cumplido</t>
         </is>
       </c>
       <c r="H46" s="21" t="inlineStr">
@@ -2605,7 +2605,7 @@
       <c r="AA46" s="22" t="n"/>
       <c r="AC46" s="23" t="inlineStr">
         <is>
-          <t>Francisco: #50 (hecho el 22-10); Mariana: #49, #52 y #53 (hechos el 22-10) y #51</t>
+          <t>Francisco: #50 (22-10); Mariana: #49, #52 y #53 (22-10) y #51 (23-10)</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
docs: marca #54 como hecho
</commit_message>
<xml_diff>
--- a/Anexos/Gestion/Carta Gantt Fase 2.xlsx
+++ b/Anexos/Gestion/Carta Gantt Fase 2.xlsx
@@ -2727,15 +2727,15 @@
           <t>Mariana</t>
         </is>
       </c>
-      <c r="E49" s="20" t="n">
-        <v>46323</v>
-      </c>
-      <c r="F49" s="20" t="n">
-        <v>46325</v>
+      <c r="E49" s="20">
+        <v>46318</v>
+      </c>
+      <c r="F49" s="20">
+        <v>46318</v>
       </c>
       <c r="G49" s="19" t="inlineStr">
         <is>
-          <t>Pendiente</t>
+          <t>Cumplido</t>
         </is>
       </c>
       <c r="H49" s="21" t="inlineStr">
@@ -2762,7 +2762,11 @@
       <c r="Y49" s="22" t="n"/>
       <c r="Z49" s="22" t="n"/>
       <c r="AA49" s="22" t="n"/>
-      <c r="AC49" s="23" t="n"/>
+      <c r="AC49" s="23" t="inlineStr">
+        <is>
+          <t>Sin free_volume_cm3(); acciones del CI fijadas por commit</t>
+        </is>
+      </c>
     </row>
     <row r="50" ht="20.1" customHeight="1" s="1">
       <c r="B50" s="18" t="n"/>

</xml_diff>